<commit_message>
Change to scaled indicators
</commit_message>
<xml_diff>
--- a/IndicatorsForClusters.xlsx
+++ b/IndicatorsForClusters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1c3256d208fb6548/Personlig/Aske Banke Consultancy/YALE/Metodeartikel_WorldDevelopmentJournal/WorldDevelopmentArticleGit/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="378" documentId="8_{9856C943-DD01-465B-AD17-0E409E296684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D1A4087-8AD9-4244-BD0C-2C8BE0F7DC61}"/>
+  <xr:revisionPtr revIDLastSave="387" documentId="8_{9856C943-DD01-465B-AD17-0E409E296684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8AAB6F5-8537-4C3C-BE36-255FD9E56484}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{726B2859-724A-4801-8E74-5A4E1AFAB973}"/>
   </bookViews>
@@ -56,7 +56,7 @@
       </extLst>
     </bk>
   </futureMetadata>
-  <futureMetadata name="XLRICHVALUE" count="8">
+  <futureMetadata name="XLRICHVALUE" count="10">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -113,13 +113,27 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="8"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="9"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
   <cellMetadata count="1">
     <bk>
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
-  <valueMetadata count="8">
+  <valueMetadata count="10">
     <bk>
       <rc t="2" v="0"/>
     </bk>
@@ -143,6 +157,12 @@
     </bk>
     <bk>
       <rc t="2" v="7"/>
+    </bk>
+    <bk>
+      <rc t="2" v="8"/>
+    </bk>
+    <bk>
+      <rc t="2" v="9"/>
     </bk>
   </valueMetadata>
 </metadata>
@@ -544,7 +564,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -571,14 +591,23 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -622,47 +651,22 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -915,7 +919,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="8">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="10">
   <rv s="0">
     <v>0</v>
     <v>5</v>
@@ -948,6 +952,14 @@
     <v>7</v>
     <v>5</v>
   </rv>
+  <rv s="0">
+    <v>8</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>9</v>
+    <v>5</v>
+  </rv>
 </rvData>
 </file>
 
@@ -970,6 +982,8 @@
   <rel r:id="rId6"/>
   <rel r:id="rId7"/>
   <rel r:id="rId8"/>
+  <rel r:id="rId9"/>
+  <rel r:id="rId10"/>
 </richValueRels>
 </file>
 
@@ -1311,30 +1325,30 @@
       <c r="B3" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="34" t="s">
+      <c r="C3" s="39" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="33" t="s">
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="J3" s="34"/>
+      <c r="J3" s="39"/>
       <c r="K3" s="8"/>
       <c r="L3" s="8"/>
       <c r="M3" s="8"/>
       <c r="N3" s="8"/>
       <c r="O3" s="8"/>
-      <c r="T3" s="24" t="s">
+      <c r="T3" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="U3" s="24"/>
-      <c r="V3" s="24"/>
-      <c r="W3" s="24"/>
-      <c r="X3" s="24"/>
+      <c r="U3" s="22"/>
+      <c r="V3" s="22"/>
+      <c r="W3" s="22"/>
+      <c r="X3" s="22"/>
     </row>
     <row r="4" spans="1:24" ht="221.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="15" t="s">
@@ -1386,13 +1400,13 @@
       <c r="Q4" s="9" t="str">
         <v>BHN</v>
       </c>
-      <c r="T4" s="22" t="s">
+      <c r="T4" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="U4" s="23"/>
-      <c r="V4" s="23"/>
-      <c r="W4" s="23"/>
-      <c r="X4" s="23"/>
+      <c r="U4" s="29"/>
+      <c r="V4" s="29"/>
+      <c r="W4" s="29"/>
+      <c r="X4" s="29"/>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="B5" s="11" t="str" cm="1">
@@ -2336,23 +2350,23 @@
       <c r="B21" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="35" t="s">
+      <c r="C21" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="D21" s="35"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="35"/>
-      <c r="G21" s="35"/>
-      <c r="H21" s="35"/>
-      <c r="I21" s="35" t="s">
+      <c r="D21" s="40"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="J21" s="35"/>
-      <c r="K21" s="35"/>
-      <c r="L21" s="35"/>
-      <c r="M21" s="35"/>
-      <c r="N21" s="35"/>
-      <c r="O21" s="35"/>
+      <c r="J21" s="40"/>
+      <c r="K21" s="40"/>
+      <c r="L21" s="40"/>
+      <c r="M21" s="40"/>
+      <c r="N21" s="40"/>
+      <c r="O21" s="40"/>
       <c r="Q21" s="1" t="s">
         <v>59</v>
       </c>
@@ -2368,62 +2382,62 @@
         <f t="array" ref="B22:B36">TRANSPOSE(_xlfn.ANCHORARRAY(C4))</f>
         <v>BHN_FWB</v>
       </c>
-      <c r="C22" s="36" t="s">
+      <c r="C22" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="D22" s="36"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="36"/>
-      <c r="I22" s="32"/>
-      <c r="J22" s="32"/>
-      <c r="K22" s="32"/>
-      <c r="L22" s="32"/>
-      <c r="M22" s="32"/>
-      <c r="N22" s="32"/>
-      <c r="O22" s="32"/>
-      <c r="Q22" s="25" t="e" vm="1">
+      <c r="D22" s="41"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="41"/>
+      <c r="H22" s="41"/>
+      <c r="I22" s="37"/>
+      <c r="J22" s="37"/>
+      <c r="K22" s="37"/>
+      <c r="L22" s="37"/>
+      <c r="M22" s="37"/>
+      <c r="N22" s="37"/>
+      <c r="O22" s="37"/>
+      <c r="Q22" s="30" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="R22" s="25"/>
-      <c r="S22" s="25"/>
-      <c r="T22" s="25"/>
-      <c r="U22" s="25"/>
-      <c r="V22" s="25"/>
-      <c r="W22" s="25"/>
-      <c r="X22" s="25"/>
-      <c r="Y22" s="25"/>
-      <c r="Z22" s="25"/>
-      <c r="AA22" s="25"/>
-      <c r="AB22" s="25" t="e" vm="2">
+      <c r="R22" s="30"/>
+      <c r="S22" s="30"/>
+      <c r="T22" s="30"/>
+      <c r="U22" s="30"/>
+      <c r="V22" s="30"/>
+      <c r="W22" s="30"/>
+      <c r="X22" s="30"/>
+      <c r="Y22" s="30"/>
+      <c r="Z22" s="30"/>
+      <c r="AA22" s="30"/>
+      <c r="AB22" s="30" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="AC22" s="25"/>
-      <c r="AD22" s="25"/>
-      <c r="AE22" s="25"/>
-      <c r="AF22" s="25"/>
-      <c r="AG22" s="25"/>
-      <c r="AH22" s="25"/>
-      <c r="AI22" s="25"/>
-      <c r="AJ22" s="25"/>
-      <c r="AK22" s="25"/>
-      <c r="AL22" s="25"/>
-      <c r="AM22" s="25"/>
-      <c r="AN22" s="25"/>
-      <c r="AO22" s="25"/>
-      <c r="AP22" s="25"/>
-      <c r="AQ22" s="25"/>
-      <c r="AR22" s="25" t="e" vm="3">
+      <c r="AC22" s="30"/>
+      <c r="AD22" s="30"/>
+      <c r="AE22" s="30"/>
+      <c r="AF22" s="30"/>
+      <c r="AG22" s="30"/>
+      <c r="AH22" s="30"/>
+      <c r="AI22" s="30"/>
+      <c r="AJ22" s="30"/>
+      <c r="AK22" s="30"/>
+      <c r="AL22" s="30"/>
+      <c r="AM22" s="30"/>
+      <c r="AN22" s="30"/>
+      <c r="AO22" s="30"/>
+      <c r="AP22" s="30"/>
+      <c r="AQ22" s="30"/>
+      <c r="AR22" s="30" t="e" vm="3">
         <v>#VALUE!</v>
       </c>
-      <c r="AS22" s="25"/>
-      <c r="AT22" s="25"/>
-      <c r="AU22" s="25"/>
-      <c r="AV22" s="25"/>
-      <c r="AW22" s="25"/>
-      <c r="AX22" s="25"/>
-      <c r="AY22" s="25"/>
+      <c r="AS22" s="30"/>
+      <c r="AT22" s="30"/>
+      <c r="AU22" s="30"/>
+      <c r="AV22" s="30"/>
+      <c r="AW22" s="30"/>
+      <c r="AX22" s="30"/>
+      <c r="AY22" s="30"/>
     </row>
     <row r="23" spans="1:51" ht="87.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23">
@@ -2432,56 +2446,56 @@
       <c r="B23" s="7" t="str">
         <v>BHN_FWB_AllExt</v>
       </c>
-      <c r="C23" s="36" t="s">
+      <c r="C23" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="D23" s="36"/>
-      <c r="E23" s="36"/>
-      <c r="F23" s="36"/>
-      <c r="G23" s="36"/>
-      <c r="H23" s="36"/>
-      <c r="I23" s="32"/>
-      <c r="J23" s="32"/>
-      <c r="K23" s="32"/>
-      <c r="L23" s="32"/>
-      <c r="M23" s="32"/>
-      <c r="N23" s="32"/>
-      <c r="O23" s="32"/>
-      <c r="Q23" s="25"/>
-      <c r="R23" s="25"/>
-      <c r="S23" s="25"/>
-      <c r="T23" s="25"/>
-      <c r="U23" s="25"/>
-      <c r="V23" s="25"/>
-      <c r="W23" s="25"/>
-      <c r="X23" s="25"/>
-      <c r="Y23" s="25"/>
-      <c r="Z23" s="25"/>
-      <c r="AA23" s="25"/>
-      <c r="AB23" s="25"/>
-      <c r="AC23" s="25"/>
-      <c r="AD23" s="25"/>
-      <c r="AE23" s="25"/>
-      <c r="AF23" s="25"/>
-      <c r="AG23" s="25"/>
-      <c r="AH23" s="25"/>
-      <c r="AI23" s="25"/>
-      <c r="AJ23" s="25"/>
-      <c r="AK23" s="25"/>
-      <c r="AL23" s="25"/>
-      <c r="AM23" s="25"/>
-      <c r="AN23" s="25"/>
-      <c r="AO23" s="25"/>
-      <c r="AP23" s="25"/>
-      <c r="AQ23" s="25"/>
-      <c r="AR23" s="25"/>
-      <c r="AS23" s="25"/>
-      <c r="AT23" s="25"/>
-      <c r="AU23" s="25"/>
-      <c r="AV23" s="25"/>
-      <c r="AW23" s="25"/>
-      <c r="AX23" s="25"/>
-      <c r="AY23" s="25"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="41"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="41"/>
+      <c r="H23" s="41"/>
+      <c r="I23" s="37"/>
+      <c r="J23" s="37"/>
+      <c r="K23" s="37"/>
+      <c r="L23" s="37"/>
+      <c r="M23" s="37"/>
+      <c r="N23" s="37"/>
+      <c r="O23" s="37"/>
+      <c r="Q23" s="30"/>
+      <c r="R23" s="30"/>
+      <c r="S23" s="30"/>
+      <c r="T23" s="30"/>
+      <c r="U23" s="30"/>
+      <c r="V23" s="30"/>
+      <c r="W23" s="30"/>
+      <c r="X23" s="30"/>
+      <c r="Y23" s="30"/>
+      <c r="Z23" s="30"/>
+      <c r="AA23" s="30"/>
+      <c r="AB23" s="30"/>
+      <c r="AC23" s="30"/>
+      <c r="AD23" s="30"/>
+      <c r="AE23" s="30"/>
+      <c r="AF23" s="30"/>
+      <c r="AG23" s="30"/>
+      <c r="AH23" s="30"/>
+      <c r="AI23" s="30"/>
+      <c r="AJ23" s="30"/>
+      <c r="AK23" s="30"/>
+      <c r="AL23" s="30"/>
+      <c r="AM23" s="30"/>
+      <c r="AN23" s="30"/>
+      <c r="AO23" s="30"/>
+      <c r="AP23" s="30"/>
+      <c r="AQ23" s="30"/>
+      <c r="AR23" s="30"/>
+      <c r="AS23" s="30"/>
+      <c r="AT23" s="30"/>
+      <c r="AU23" s="30"/>
+      <c r="AV23" s="30"/>
+      <c r="AW23" s="30"/>
+      <c r="AX23" s="30"/>
+      <c r="AY23" s="30"/>
     </row>
     <row r="24" spans="1:51" ht="108.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24">
@@ -2490,56 +2504,56 @@
       <c r="B24" s="7" t="str">
         <v>Few_indicators_closest_DLS_coverage</v>
       </c>
-      <c r="C24" s="36" t="s">
+      <c r="C24" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="D24" s="36"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="36"/>
-      <c r="H24" s="36"/>
-      <c r="I24" s="32"/>
-      <c r="J24" s="32"/>
-      <c r="K24" s="32"/>
-      <c r="L24" s="32"/>
-      <c r="M24" s="32"/>
-      <c r="N24" s="32"/>
-      <c r="O24" s="32"/>
-      <c r="Q24" s="25"/>
-      <c r="R24" s="25"/>
-      <c r="S24" s="25"/>
-      <c r="T24" s="25"/>
-      <c r="U24" s="25"/>
-      <c r="V24" s="25"/>
-      <c r="W24" s="25"/>
-      <c r="X24" s="25"/>
-      <c r="Y24" s="25"/>
-      <c r="Z24" s="25"/>
-      <c r="AA24" s="25"/>
-      <c r="AB24" s="25"/>
-      <c r="AC24" s="25"/>
-      <c r="AD24" s="25"/>
-      <c r="AE24" s="25"/>
-      <c r="AF24" s="25"/>
-      <c r="AG24" s="25"/>
-      <c r="AH24" s="25"/>
-      <c r="AI24" s="25"/>
-      <c r="AJ24" s="25"/>
-      <c r="AK24" s="25"/>
-      <c r="AL24" s="25"/>
-      <c r="AM24" s="25"/>
-      <c r="AN24" s="25"/>
-      <c r="AO24" s="25"/>
-      <c r="AP24" s="25"/>
-      <c r="AQ24" s="25"/>
-      <c r="AR24" s="25"/>
-      <c r="AS24" s="25"/>
-      <c r="AT24" s="25"/>
-      <c r="AU24" s="25"/>
-      <c r="AV24" s="25"/>
-      <c r="AW24" s="25"/>
-      <c r="AX24" s="25"/>
-      <c r="AY24" s="25"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="41"/>
+      <c r="F24" s="41"/>
+      <c r="G24" s="41"/>
+      <c r="H24" s="41"/>
+      <c r="I24" s="37"/>
+      <c r="J24" s="37"/>
+      <c r="K24" s="37"/>
+      <c r="L24" s="37"/>
+      <c r="M24" s="37"/>
+      <c r="N24" s="37"/>
+      <c r="O24" s="37"/>
+      <c r="Q24" s="30"/>
+      <c r="R24" s="30"/>
+      <c r="S24" s="30"/>
+      <c r="T24" s="30"/>
+      <c r="U24" s="30"/>
+      <c r="V24" s="30"/>
+      <c r="W24" s="30"/>
+      <c r="X24" s="30"/>
+      <c r="Y24" s="30"/>
+      <c r="Z24" s="30"/>
+      <c r="AA24" s="30"/>
+      <c r="AB24" s="30"/>
+      <c r="AC24" s="30"/>
+      <c r="AD24" s="30"/>
+      <c r="AE24" s="30"/>
+      <c r="AF24" s="30"/>
+      <c r="AG24" s="30"/>
+      <c r="AH24" s="30"/>
+      <c r="AI24" s="30"/>
+      <c r="AJ24" s="30"/>
+      <c r="AK24" s="30"/>
+      <c r="AL24" s="30"/>
+      <c r="AM24" s="30"/>
+      <c r="AN24" s="30"/>
+      <c r="AO24" s="30"/>
+      <c r="AP24" s="30"/>
+      <c r="AQ24" s="30"/>
+      <c r="AR24" s="30"/>
+      <c r="AS24" s="30"/>
+      <c r="AT24" s="30"/>
+      <c r="AU24" s="30"/>
+      <c r="AV24" s="30"/>
+      <c r="AW24" s="30"/>
+      <c r="AX24" s="30"/>
+      <c r="AY24" s="30"/>
     </row>
     <row r="25" spans="1:51" ht="81.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25">
@@ -2548,48 +2562,48 @@
       <c r="B25" s="7" t="str">
         <v>Few indicators_SPI_preferred</v>
       </c>
-      <c r="C25" s="36" t="s">
+      <c r="C25" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="D25" s="36"/>
-      <c r="E25" s="36"/>
-      <c r="F25" s="36"/>
-      <c r="G25" s="36"/>
-      <c r="H25" s="36"/>
-      <c r="I25" s="32"/>
-      <c r="J25" s="32"/>
-      <c r="K25" s="32"/>
-      <c r="L25" s="32"/>
-      <c r="M25" s="32"/>
-      <c r="N25" s="32"/>
-      <c r="O25" s="32"/>
-      <c r="Q25" s="25"/>
-      <c r="R25" s="25"/>
-      <c r="S25" s="25"/>
-      <c r="T25" s="25"/>
-      <c r="U25" s="25"/>
-      <c r="V25" s="25"/>
-      <c r="W25" s="25"/>
-      <c r="X25" s="25"/>
-      <c r="Y25" s="25"/>
-      <c r="Z25" s="25"/>
-      <c r="AA25" s="25"/>
-      <c r="AB25" s="25"/>
-      <c r="AC25" s="25"/>
-      <c r="AD25" s="25"/>
-      <c r="AE25" s="25"/>
-      <c r="AF25" s="25"/>
-      <c r="AG25" s="25"/>
-      <c r="AH25" s="25"/>
-      <c r="AI25" s="25"/>
-      <c r="AJ25" s="25"/>
-      <c r="AK25" s="25"/>
-      <c r="AL25" s="25"/>
-      <c r="AM25" s="25"/>
-      <c r="AN25" s="25"/>
-      <c r="AO25" s="25"/>
-      <c r="AP25" s="25"/>
-      <c r="AQ25" s="25"/>
+      <c r="D25" s="41"/>
+      <c r="E25" s="41"/>
+      <c r="F25" s="41"/>
+      <c r="G25" s="41"/>
+      <c r="H25" s="41"/>
+      <c r="I25" s="37"/>
+      <c r="J25" s="37"/>
+      <c r="K25" s="37"/>
+      <c r="L25" s="37"/>
+      <c r="M25" s="37"/>
+      <c r="N25" s="37"/>
+      <c r="O25" s="37"/>
+      <c r="Q25" s="30"/>
+      <c r="R25" s="30"/>
+      <c r="S25" s="30"/>
+      <c r="T25" s="30"/>
+      <c r="U25" s="30"/>
+      <c r="V25" s="30"/>
+      <c r="W25" s="30"/>
+      <c r="X25" s="30"/>
+      <c r="Y25" s="30"/>
+      <c r="Z25" s="30"/>
+      <c r="AA25" s="30"/>
+      <c r="AB25" s="30"/>
+      <c r="AC25" s="30"/>
+      <c r="AD25" s="30"/>
+      <c r="AE25" s="30"/>
+      <c r="AF25" s="30"/>
+      <c r="AG25" s="30"/>
+      <c r="AH25" s="30"/>
+      <c r="AI25" s="30"/>
+      <c r="AJ25" s="30"/>
+      <c r="AK25" s="30"/>
+      <c r="AL25" s="30"/>
+      <c r="AM25" s="30"/>
+      <c r="AN25" s="30"/>
+      <c r="AO25" s="30"/>
+      <c r="AP25" s="30"/>
+      <c r="AQ25" s="30"/>
     </row>
     <row r="26" spans="1:51" ht="69.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26">
@@ -2598,50 +2612,50 @@
       <c r="B26" s="7" t="str">
         <v>No_non_DLS</v>
       </c>
-      <c r="C26" s="38" t="s">
+      <c r="C26" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="D26" s="38"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="38"/>
-      <c r="G26" s="38"/>
-      <c r="H26" s="38"/>
-      <c r="I26" s="32"/>
-      <c r="J26" s="32"/>
-      <c r="K26" s="32"/>
-      <c r="L26" s="32"/>
-      <c r="M26" s="32"/>
-      <c r="N26" s="32"/>
-      <c r="O26" s="32"/>
-      <c r="Q26" s="25" t="e" vm="4">
+      <c r="D26" s="43"/>
+      <c r="E26" s="43"/>
+      <c r="F26" s="43"/>
+      <c r="G26" s="43"/>
+      <c r="H26" s="43"/>
+      <c r="I26" s="37"/>
+      <c r="J26" s="37"/>
+      <c r="K26" s="37"/>
+      <c r="L26" s="37"/>
+      <c r="M26" s="37"/>
+      <c r="N26" s="37"/>
+      <c r="O26" s="37"/>
+      <c r="Q26" s="30" t="e" vm="4">
         <v>#VALUE!</v>
       </c>
-      <c r="R26" s="25"/>
-      <c r="S26" s="25"/>
-      <c r="T26" s="25"/>
-      <c r="U26" s="25"/>
-      <c r="V26" s="25"/>
-      <c r="W26" s="25"/>
-      <c r="X26" s="25"/>
-      <c r="Y26" s="25"/>
-      <c r="Z26" s="25"/>
-      <c r="AA26" s="25"/>
-      <c r="AB26" s="25"/>
-      <c r="AC26" s="25"/>
-      <c r="AD26" s="25"/>
-      <c r="AE26" s="25"/>
-      <c r="AF26" s="25"/>
-      <c r="AG26" s="25"/>
-      <c r="AH26" s="25"/>
-      <c r="AI26" s="25"/>
-      <c r="AJ26" s="25"/>
-      <c r="AK26" s="25"/>
-      <c r="AL26" s="25"/>
-      <c r="AM26" s="25"/>
-      <c r="AN26" s="25"/>
-      <c r="AO26" s="25"/>
-      <c r="AP26" s="25"/>
-      <c r="AQ26" s="25"/>
+      <c r="R26" s="30"/>
+      <c r="S26" s="30"/>
+      <c r="T26" s="30"/>
+      <c r="U26" s="30"/>
+      <c r="V26" s="30"/>
+      <c r="W26" s="30"/>
+      <c r="X26" s="30"/>
+      <c r="Y26" s="30"/>
+      <c r="Z26" s="30"/>
+      <c r="AA26" s="30"/>
+      <c r="AB26" s="30"/>
+      <c r="AC26" s="30"/>
+      <c r="AD26" s="30"/>
+      <c r="AE26" s="30"/>
+      <c r="AF26" s="30"/>
+      <c r="AG26" s="30"/>
+      <c r="AH26" s="30"/>
+      <c r="AI26" s="30"/>
+      <c r="AJ26" s="30"/>
+      <c r="AK26" s="30"/>
+      <c r="AL26" s="30"/>
+      <c r="AM26" s="30"/>
+      <c r="AN26" s="30"/>
+      <c r="AO26" s="30"/>
+      <c r="AP26" s="30"/>
+      <c r="AQ26" s="30"/>
     </row>
     <row r="27" spans="1:51" ht="93" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27">
@@ -2650,48 +2664,48 @@
       <c r="B27" s="7" t="str">
         <v>Only_%_of_pop</v>
       </c>
-      <c r="C27" s="38" t="s">
+      <c r="C27" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="D27" s="38"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="38"/>
-      <c r="H27" s="38"/>
-      <c r="I27" s="32"/>
-      <c r="J27" s="32"/>
-      <c r="K27" s="32"/>
-      <c r="L27" s="32"/>
-      <c r="M27" s="32"/>
-      <c r="N27" s="32"/>
-      <c r="O27" s="32"/>
-      <c r="Q27" s="25"/>
-      <c r="R27" s="25"/>
-      <c r="S27" s="25"/>
-      <c r="T27" s="25"/>
-      <c r="U27" s="25"/>
-      <c r="V27" s="25"/>
-      <c r="W27" s="25"/>
-      <c r="X27" s="25"/>
-      <c r="Y27" s="25"/>
-      <c r="Z27" s="25"/>
-      <c r="AA27" s="25"/>
-      <c r="AB27" s="25"/>
-      <c r="AC27" s="25"/>
-      <c r="AD27" s="25"/>
-      <c r="AE27" s="25"/>
-      <c r="AF27" s="25"/>
-      <c r="AG27" s="25"/>
-      <c r="AH27" s="25"/>
-      <c r="AI27" s="25"/>
-      <c r="AJ27" s="25"/>
-      <c r="AK27" s="25"/>
-      <c r="AL27" s="25"/>
-      <c r="AM27" s="25"/>
-      <c r="AN27" s="25"/>
-      <c r="AO27" s="25"/>
-      <c r="AP27" s="25"/>
-      <c r="AQ27" s="25"/>
+      <c r="D27" s="43"/>
+      <c r="E27" s="43"/>
+      <c r="F27" s="43"/>
+      <c r="G27" s="43"/>
+      <c r="H27" s="43"/>
+      <c r="I27" s="37"/>
+      <c r="J27" s="37"/>
+      <c r="K27" s="37"/>
+      <c r="L27" s="37"/>
+      <c r="M27" s="37"/>
+      <c r="N27" s="37"/>
+      <c r="O27" s="37"/>
+      <c r="Q27" s="30"/>
+      <c r="R27" s="30"/>
+      <c r="S27" s="30"/>
+      <c r="T27" s="30"/>
+      <c r="U27" s="30"/>
+      <c r="V27" s="30"/>
+      <c r="W27" s="30"/>
+      <c r="X27" s="30"/>
+      <c r="Y27" s="30"/>
+      <c r="Z27" s="30"/>
+      <c r="AA27" s="30"/>
+      <c r="AB27" s="30"/>
+      <c r="AC27" s="30"/>
+      <c r="AD27" s="30"/>
+      <c r="AE27" s="30"/>
+      <c r="AF27" s="30"/>
+      <c r="AG27" s="30"/>
+      <c r="AH27" s="30"/>
+      <c r="AI27" s="30"/>
+      <c r="AJ27" s="30"/>
+      <c r="AK27" s="30"/>
+      <c r="AL27" s="30"/>
+      <c r="AM27" s="30"/>
+      <c r="AN27" s="30"/>
+      <c r="AO27" s="30"/>
+      <c r="AP27" s="30"/>
+      <c r="AQ27" s="30"/>
     </row>
     <row r="28" spans="1:51" ht="65.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28">
@@ -2700,50 +2714,50 @@
       <c r="B28" s="17" t="str">
         <v>Few_indicators_closest_DLS_coverage_90</v>
       </c>
-      <c r="C28" s="28" t="s">
+      <c r="C28" s="33" t="s">
         <v>62</v>
       </c>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="28"/>
-      <c r="I28" s="30"/>
-      <c r="J28" s="30"/>
-      <c r="K28" s="30"/>
-      <c r="L28" s="30"/>
-      <c r="M28" s="30"/>
-      <c r="N28" s="30"/>
-      <c r="O28" s="30"/>
-      <c r="Q28" s="25"/>
-      <c r="R28" s="25"/>
-      <c r="S28" s="25"/>
-      <c r="T28" s="25"/>
-      <c r="U28" s="25"/>
-      <c r="V28" s="25"/>
-      <c r="W28" s="25"/>
-      <c r="X28" s="25"/>
-      <c r="Y28" s="25"/>
-      <c r="Z28" s="25"/>
-      <c r="AA28" s="25"/>
-      <c r="AB28" s="25" t="e" vm="5">
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="35"/>
+      <c r="J28" s="35"/>
+      <c r="K28" s="35"/>
+      <c r="L28" s="35"/>
+      <c r="M28" s="35"/>
+      <c r="N28" s="35"/>
+      <c r="O28" s="35"/>
+      <c r="Q28" s="30"/>
+      <c r="R28" s="30"/>
+      <c r="S28" s="30"/>
+      <c r="T28" s="30"/>
+      <c r="U28" s="30"/>
+      <c r="V28" s="30"/>
+      <c r="W28" s="30"/>
+      <c r="X28" s="30"/>
+      <c r="Y28" s="30"/>
+      <c r="Z28" s="30"/>
+      <c r="AA28" s="30"/>
+      <c r="AB28" s="30" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="AC28" s="25"/>
-      <c r="AD28" s="25"/>
-      <c r="AE28" s="25"/>
-      <c r="AF28" s="25"/>
-      <c r="AG28" s="25"/>
-      <c r="AH28" s="25"/>
-      <c r="AI28" s="25"/>
-      <c r="AJ28" s="25"/>
-      <c r="AK28" s="25"/>
-      <c r="AL28" s="25"/>
-      <c r="AM28" s="25"/>
-      <c r="AN28" s="25"/>
-      <c r="AO28" s="25"/>
-      <c r="AP28" s="25"/>
-      <c r="AQ28" s="25"/>
+      <c r="AC28" s="30"/>
+      <c r="AD28" s="30"/>
+      <c r="AE28" s="30"/>
+      <c r="AF28" s="30"/>
+      <c r="AG28" s="30"/>
+      <c r="AH28" s="30"/>
+      <c r="AI28" s="30"/>
+      <c r="AJ28" s="30"/>
+      <c r="AK28" s="30"/>
+      <c r="AL28" s="30"/>
+      <c r="AM28" s="30"/>
+      <c r="AN28" s="30"/>
+      <c r="AO28" s="30"/>
+      <c r="AP28" s="30"/>
+      <c r="AQ28" s="30"/>
     </row>
     <row r="29" spans="1:51" ht="67.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29">
@@ -2752,48 +2766,48 @@
       <c r="B29" s="17" t="str">
         <v>Few indicators_SPI_preferred_90</v>
       </c>
-      <c r="C29" s="28" t="s">
+      <c r="C29" s="33" t="s">
         <v>62</v>
       </c>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="28"/>
-      <c r="I29" s="30"/>
-      <c r="J29" s="30"/>
-      <c r="K29" s="30"/>
-      <c r="L29" s="30"/>
-      <c r="M29" s="30"/>
-      <c r="N29" s="30"/>
-      <c r="O29" s="30"/>
-      <c r="Q29" s="25"/>
-      <c r="R29" s="25"/>
-      <c r="S29" s="25"/>
-      <c r="T29" s="25"/>
-      <c r="U29" s="25"/>
-      <c r="V29" s="25"/>
-      <c r="W29" s="25"/>
-      <c r="X29" s="25"/>
-      <c r="Y29" s="25"/>
-      <c r="Z29" s="25"/>
-      <c r="AA29" s="25"/>
-      <c r="AB29" s="25"/>
-      <c r="AC29" s="25"/>
-      <c r="AD29" s="25"/>
-      <c r="AE29" s="25"/>
-      <c r="AF29" s="25"/>
-      <c r="AG29" s="25"/>
-      <c r="AH29" s="25"/>
-      <c r="AI29" s="25"/>
-      <c r="AJ29" s="25"/>
-      <c r="AK29" s="25"/>
-      <c r="AL29" s="25"/>
-      <c r="AM29" s="25"/>
-      <c r="AN29" s="25"/>
-      <c r="AO29" s="25"/>
-      <c r="AP29" s="25"/>
-      <c r="AQ29" s="25"/>
+      <c r="D29" s="33"/>
+      <c r="E29" s="33"/>
+      <c r="F29" s="33"/>
+      <c r="G29" s="33"/>
+      <c r="H29" s="33"/>
+      <c r="I29" s="35"/>
+      <c r="J29" s="35"/>
+      <c r="K29" s="35"/>
+      <c r="L29" s="35"/>
+      <c r="M29" s="35"/>
+      <c r="N29" s="35"/>
+      <c r="O29" s="35"/>
+      <c r="Q29" s="30"/>
+      <c r="R29" s="30"/>
+      <c r="S29" s="30"/>
+      <c r="T29" s="30"/>
+      <c r="U29" s="30"/>
+      <c r="V29" s="30"/>
+      <c r="W29" s="30"/>
+      <c r="X29" s="30"/>
+      <c r="Y29" s="30"/>
+      <c r="Z29" s="30"/>
+      <c r="AA29" s="30"/>
+      <c r="AB29" s="30"/>
+      <c r="AC29" s="30"/>
+      <c r="AD29" s="30"/>
+      <c r="AE29" s="30"/>
+      <c r="AF29" s="30"/>
+      <c r="AG29" s="30"/>
+      <c r="AH29" s="30"/>
+      <c r="AI29" s="30"/>
+      <c r="AJ29" s="30"/>
+      <c r="AK29" s="30"/>
+      <c r="AL29" s="30"/>
+      <c r="AM29" s="30"/>
+      <c r="AN29" s="30"/>
+      <c r="AO29" s="30"/>
+      <c r="AP29" s="30"/>
+      <c r="AQ29" s="30"/>
     </row>
     <row r="30" spans="1:51" ht="55.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30">
@@ -2802,50 +2816,50 @@
       <c r="B30" s="17" t="str">
         <v>Few_indicators_closeDLS_subPrimSchool</v>
       </c>
-      <c r="C30" s="26" t="s">
+      <c r="C30" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="30"/>
-      <c r="J30" s="30"/>
-      <c r="K30" s="30"/>
-      <c r="L30" s="30"/>
-      <c r="M30" s="30"/>
-      <c r="N30" s="30"/>
-      <c r="O30" s="30"/>
-      <c r="Q30" s="25" t="e" vm="6">
+      <c r="D30" s="31"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="31"/>
+      <c r="G30" s="31"/>
+      <c r="H30" s="31"/>
+      <c r="I30" s="35"/>
+      <c r="J30" s="35"/>
+      <c r="K30" s="35"/>
+      <c r="L30" s="35"/>
+      <c r="M30" s="35"/>
+      <c r="N30" s="35"/>
+      <c r="O30" s="35"/>
+      <c r="Q30" s="30" t="e" vm="6">
         <v>#VALUE!</v>
       </c>
-      <c r="R30" s="25"/>
-      <c r="S30" s="25"/>
-      <c r="T30" s="25"/>
-      <c r="U30" s="25"/>
-      <c r="V30" s="25"/>
-      <c r="W30" s="25"/>
-      <c r="X30" s="25"/>
-      <c r="Y30" s="25"/>
-      <c r="Z30" s="25"/>
-      <c r="AA30" s="25"/>
-      <c r="AB30" s="25"/>
-      <c r="AC30" s="25"/>
-      <c r="AD30" s="25"/>
-      <c r="AE30" s="25"/>
-      <c r="AF30" s="25"/>
-      <c r="AG30" s="25"/>
-      <c r="AH30" s="25"/>
-      <c r="AI30" s="25"/>
-      <c r="AJ30" s="25"/>
-      <c r="AK30" s="25"/>
-      <c r="AL30" s="25"/>
-      <c r="AM30" s="25"/>
-      <c r="AN30" s="25"/>
-      <c r="AO30" s="25"/>
-      <c r="AP30" s="25"/>
-      <c r="AQ30" s="25"/>
+      <c r="R30" s="30"/>
+      <c r="S30" s="30"/>
+      <c r="T30" s="30"/>
+      <c r="U30" s="30"/>
+      <c r="V30" s="30"/>
+      <c r="W30" s="30"/>
+      <c r="X30" s="30"/>
+      <c r="Y30" s="30"/>
+      <c r="Z30" s="30"/>
+      <c r="AA30" s="30"/>
+      <c r="AB30" s="30"/>
+      <c r="AC30" s="30"/>
+      <c r="AD30" s="30"/>
+      <c r="AE30" s="30"/>
+      <c r="AF30" s="30"/>
+      <c r="AG30" s="30"/>
+      <c r="AH30" s="30"/>
+      <c r="AI30" s="30"/>
+      <c r="AJ30" s="30"/>
+      <c r="AK30" s="30"/>
+      <c r="AL30" s="30"/>
+      <c r="AM30" s="30"/>
+      <c r="AN30" s="30"/>
+      <c r="AO30" s="30"/>
+      <c r="AP30" s="30"/>
+      <c r="AQ30" s="30"/>
     </row>
     <row r="31" spans="1:51" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31">
@@ -2854,48 +2868,48 @@
       <c r="B31" s="17" t="str">
         <v>No_non_DLS_90</v>
       </c>
-      <c r="C31" s="28" t="s">
+      <c r="C31" s="33" t="s">
         <v>62</v>
       </c>
-      <c r="D31" s="28"/>
-      <c r="E31" s="28"/>
-      <c r="F31" s="28"/>
-      <c r="G31" s="28"/>
-      <c r="H31" s="28"/>
-      <c r="I31" s="30"/>
-      <c r="J31" s="30"/>
-      <c r="K31" s="30"/>
-      <c r="L31" s="30"/>
-      <c r="M31" s="30"/>
-      <c r="N31" s="30"/>
-      <c r="O31" s="30"/>
-      <c r="Q31" s="25"/>
-      <c r="R31" s="25"/>
-      <c r="S31" s="25"/>
-      <c r="T31" s="25"/>
-      <c r="U31" s="25"/>
-      <c r="V31" s="25"/>
-      <c r="W31" s="25"/>
-      <c r="X31" s="25"/>
-      <c r="Y31" s="25"/>
-      <c r="Z31" s="25"/>
-      <c r="AA31" s="25"/>
-      <c r="AB31" s="25"/>
-      <c r="AC31" s="25"/>
-      <c r="AD31" s="25"/>
-      <c r="AE31" s="25"/>
-      <c r="AF31" s="25"/>
-      <c r="AG31" s="25"/>
-      <c r="AH31" s="25"/>
-      <c r="AI31" s="25"/>
-      <c r="AJ31" s="25"/>
-      <c r="AK31" s="25"/>
-      <c r="AL31" s="25"/>
-      <c r="AM31" s="25"/>
-      <c r="AN31" s="25"/>
-      <c r="AO31" s="25"/>
-      <c r="AP31" s="25"/>
-      <c r="AQ31" s="25"/>
+      <c r="D31" s="33"/>
+      <c r="E31" s="33"/>
+      <c r="F31" s="33"/>
+      <c r="G31" s="33"/>
+      <c r="H31" s="33"/>
+      <c r="I31" s="35"/>
+      <c r="J31" s="35"/>
+      <c r="K31" s="35"/>
+      <c r="L31" s="35"/>
+      <c r="M31" s="35"/>
+      <c r="N31" s="35"/>
+      <c r="O31" s="35"/>
+      <c r="Q31" s="30"/>
+      <c r="R31" s="30"/>
+      <c r="S31" s="30"/>
+      <c r="T31" s="30"/>
+      <c r="U31" s="30"/>
+      <c r="V31" s="30"/>
+      <c r="W31" s="30"/>
+      <c r="X31" s="30"/>
+      <c r="Y31" s="30"/>
+      <c r="Z31" s="30"/>
+      <c r="AA31" s="30"/>
+      <c r="AB31" s="30"/>
+      <c r="AC31" s="30"/>
+      <c r="AD31" s="30"/>
+      <c r="AE31" s="30"/>
+      <c r="AF31" s="30"/>
+      <c r="AG31" s="30"/>
+      <c r="AH31" s="30"/>
+      <c r="AI31" s="30"/>
+      <c r="AJ31" s="30"/>
+      <c r="AK31" s="30"/>
+      <c r="AL31" s="30"/>
+      <c r="AM31" s="30"/>
+      <c r="AN31" s="30"/>
+      <c r="AO31" s="30"/>
+      <c r="AP31" s="30"/>
+      <c r="AQ31" s="30"/>
     </row>
     <row r="32" spans="1:51" ht="103.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32">
@@ -2904,50 +2918,50 @@
       <c r="B32" s="17" t="str">
         <v>Few_Indicators_subWatSani</v>
       </c>
-      <c r="C32" s="28" t="s">
+      <c r="C32" s="33" t="s">
         <v>67</v>
       </c>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
-      <c r="I32" s="30"/>
-      <c r="J32" s="30"/>
-      <c r="K32" s="30"/>
-      <c r="L32" s="30"/>
-      <c r="M32" s="30"/>
-      <c r="N32" s="30"/>
-      <c r="O32" s="30"/>
-      <c r="Q32" s="25"/>
-      <c r="R32" s="25"/>
-      <c r="S32" s="25"/>
-      <c r="T32" s="25"/>
-      <c r="U32" s="25"/>
-      <c r="V32" s="25"/>
-      <c r="W32" s="25"/>
-      <c r="X32" s="25"/>
-      <c r="Y32" s="25"/>
-      <c r="Z32" s="25"/>
-      <c r="AA32" s="25"/>
-      <c r="AB32" s="25" t="e" vm="7">
+      <c r="D32" s="33"/>
+      <c r="E32" s="33"/>
+      <c r="F32" s="33"/>
+      <c r="G32" s="33"/>
+      <c r="H32" s="33"/>
+      <c r="I32" s="35"/>
+      <c r="J32" s="35"/>
+      <c r="K32" s="35"/>
+      <c r="L32" s="35"/>
+      <c r="M32" s="35"/>
+      <c r="N32" s="35"/>
+      <c r="O32" s="35"/>
+      <c r="Q32" s="30"/>
+      <c r="R32" s="30"/>
+      <c r="S32" s="30"/>
+      <c r="T32" s="30"/>
+      <c r="U32" s="30"/>
+      <c r="V32" s="30"/>
+      <c r="W32" s="30"/>
+      <c r="X32" s="30"/>
+      <c r="Y32" s="30"/>
+      <c r="Z32" s="30"/>
+      <c r="AA32" s="30"/>
+      <c r="AB32" s="30" t="e" vm="7">
         <v>#VALUE!</v>
       </c>
-      <c r="AC32" s="25"/>
-      <c r="AD32" s="25"/>
-      <c r="AE32" s="25"/>
-      <c r="AF32" s="25"/>
-      <c r="AG32" s="25"/>
-      <c r="AH32" s="25"/>
-      <c r="AI32" s="25"/>
-      <c r="AJ32" s="25"/>
-      <c r="AK32" s="25"/>
-      <c r="AL32" s="25"/>
-      <c r="AM32" s="25"/>
-      <c r="AN32" s="25"/>
-      <c r="AO32" s="25"/>
-      <c r="AP32" s="25"/>
-      <c r="AQ32" s="25"/>
+      <c r="AC32" s="30"/>
+      <c r="AD32" s="30"/>
+      <c r="AE32" s="30"/>
+      <c r="AF32" s="30"/>
+      <c r="AG32" s="30"/>
+      <c r="AH32" s="30"/>
+      <c r="AI32" s="30"/>
+      <c r="AJ32" s="30"/>
+      <c r="AK32" s="30"/>
+      <c r="AL32" s="30"/>
+      <c r="AM32" s="30"/>
+      <c r="AN32" s="30"/>
+      <c r="AO32" s="30"/>
+      <c r="AP32" s="30"/>
+      <c r="AQ32" s="30"/>
     </row>
     <row r="33" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A33">
@@ -2956,501 +2970,498 @@
       <c r="B33" s="6" t="str">
         <v>Only_OPP</v>
       </c>
-      <c r="C33" s="29" t="s">
+      <c r="C33" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="D33" s="29"/>
-      <c r="E33" s="29"/>
-      <c r="F33" s="29"/>
-      <c r="G33" s="29"/>
-      <c r="H33" s="29"/>
-      <c r="I33" s="27"/>
-      <c r="J33" s="27"/>
-      <c r="K33" s="27"/>
-      <c r="L33" s="27"/>
-      <c r="M33" s="27"/>
-      <c r="N33" s="27"/>
-      <c r="O33" s="27"/>
-      <c r="Q33" s="25"/>
-      <c r="R33" s="25"/>
-      <c r="S33" s="25"/>
-      <c r="T33" s="25"/>
-      <c r="U33" s="25"/>
-      <c r="V33" s="25"/>
-      <c r="W33" s="25"/>
-      <c r="X33" s="25"/>
-      <c r="Y33" s="25"/>
-      <c r="Z33" s="25"/>
-      <c r="AA33" s="25"/>
-      <c r="AB33" s="25"/>
-      <c r="AC33" s="25"/>
-      <c r="AD33" s="25"/>
-      <c r="AE33" s="25"/>
-      <c r="AF33" s="25"/>
-      <c r="AG33" s="25"/>
-      <c r="AH33" s="25"/>
-      <c r="AI33" s="25"/>
-      <c r="AJ33" s="25"/>
-      <c r="AK33" s="25"/>
-      <c r="AL33" s="25"/>
-      <c r="AM33" s="25"/>
-      <c r="AN33" s="25"/>
-      <c r="AO33" s="25"/>
-      <c r="AP33" s="25"/>
-      <c r="AQ33" s="25"/>
+      <c r="D33" s="34"/>
+      <c r="E33" s="34"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="34"/>
+      <c r="H33" s="34"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="32"/>
+      <c r="K33" s="32"/>
+      <c r="L33" s="32"/>
+      <c r="M33" s="32"/>
+      <c r="N33" s="32"/>
+      <c r="O33" s="32"/>
+      <c r="Q33" s="30"/>
+      <c r="R33" s="30"/>
+      <c r="S33" s="30"/>
+      <c r="T33" s="30"/>
+      <c r="U33" s="30"/>
+      <c r="V33" s="30"/>
+      <c r="W33" s="30"/>
+      <c r="X33" s="30"/>
+      <c r="Y33" s="30"/>
+      <c r="Z33" s="30"/>
+      <c r="AA33" s="30"/>
+      <c r="AB33" s="30"/>
+      <c r="AC33" s="30"/>
+      <c r="AD33" s="30"/>
+      <c r="AE33" s="30"/>
+      <c r="AF33" s="30"/>
+      <c r="AG33" s="30"/>
+      <c r="AH33" s="30"/>
+      <c r="AI33" s="30"/>
+      <c r="AJ33" s="30"/>
+      <c r="AK33" s="30"/>
+      <c r="AL33" s="30"/>
+      <c r="AM33" s="30"/>
+      <c r="AN33" s="30"/>
+      <c r="AO33" s="30"/>
+      <c r="AP33" s="30"/>
+      <c r="AQ33" s="30"/>
     </row>
     <row r="34" spans="1:43" x14ac:dyDescent="0.3">
       <c r="B34" s="6" t="str">
         <v>Baseline</v>
       </c>
-      <c r="C34" s="27"/>
-      <c r="D34" s="27"/>
-      <c r="E34" s="27"/>
-      <c r="F34" s="27"/>
-      <c r="G34" s="27"/>
-      <c r="H34" s="27"/>
-      <c r="I34" s="27"/>
-      <c r="J34" s="27"/>
-      <c r="K34" s="27"/>
-      <c r="L34" s="27"/>
-      <c r="M34" s="27"/>
-      <c r="N34" s="27"/>
-      <c r="O34" s="27"/>
-      <c r="Q34" s="25"/>
-      <c r="R34" s="25"/>
-      <c r="S34" s="25"/>
-      <c r="T34" s="25"/>
-      <c r="U34" s="25"/>
-      <c r="V34" s="25"/>
-      <c r="W34" s="25"/>
-      <c r="X34" s="25"/>
-      <c r="Y34" s="25"/>
-      <c r="Z34" s="25"/>
-      <c r="AA34" s="25"/>
-      <c r="AB34" s="25"/>
-      <c r="AC34" s="25"/>
-      <c r="AD34" s="25"/>
-      <c r="AE34" s="25"/>
-      <c r="AF34" s="25"/>
-      <c r="AG34" s="25"/>
-      <c r="AH34" s="25"/>
-      <c r="AI34" s="25"/>
-      <c r="AJ34" s="25"/>
-      <c r="AK34" s="25"/>
-      <c r="AL34" s="25"/>
-      <c r="AM34" s="25"/>
-      <c r="AN34" s="25"/>
-      <c r="AO34" s="25"/>
-      <c r="AP34" s="25"/>
-      <c r="AQ34" s="25"/>
+      <c r="C34" s="32"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="32"/>
+      <c r="K34" s="32"/>
+      <c r="L34" s="32"/>
+      <c r="M34" s="32"/>
+      <c r="N34" s="32"/>
+      <c r="O34" s="32"/>
+      <c r="Q34" s="30"/>
+      <c r="R34" s="30"/>
+      <c r="S34" s="30"/>
+      <c r="T34" s="30"/>
+      <c r="U34" s="30"/>
+      <c r="V34" s="30"/>
+      <c r="W34" s="30"/>
+      <c r="X34" s="30"/>
+      <c r="Y34" s="30"/>
+      <c r="Z34" s="30"/>
+      <c r="AA34" s="30"/>
+      <c r="AB34" s="30"/>
+      <c r="AC34" s="30"/>
+      <c r="AD34" s="30"/>
+      <c r="AE34" s="30"/>
+      <c r="AF34" s="30"/>
+      <c r="AG34" s="30"/>
+      <c r="AH34" s="30"/>
+      <c r="AI34" s="30"/>
+      <c r="AJ34" s="30"/>
+      <c r="AK34" s="30"/>
+      <c r="AL34" s="30"/>
+      <c r="AM34" s="30"/>
+      <c r="AN34" s="30"/>
+      <c r="AO34" s="30"/>
+      <c r="AP34" s="30"/>
+      <c r="AQ34" s="30"/>
     </row>
     <row r="35" spans="1:43" x14ac:dyDescent="0.3">
       <c r="B35" s="6" t="str">
         <v>No_nonDLS_limExt</v>
       </c>
-      <c r="C35" s="27"/>
-      <c r="D35" s="27"/>
-      <c r="E35" s="27"/>
-      <c r="F35" s="27"/>
-      <c r="G35" s="27"/>
-      <c r="H35" s="27"/>
-      <c r="I35" s="27" t="s">
+      <c r="C35" s="32"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="32"/>
+      <c r="G35" s="32"/>
+      <c r="H35" s="32"/>
+      <c r="I35" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="J35" s="27"/>
-      <c r="K35" s="27"/>
-      <c r="L35" s="27"/>
-      <c r="M35" s="27"/>
-      <c r="N35" s="27"/>
-      <c r="O35" s="27"/>
-      <c r="Q35" s="25"/>
-      <c r="R35" s="25"/>
-      <c r="S35" s="25"/>
-      <c r="T35" s="25"/>
-      <c r="U35" s="25"/>
-      <c r="V35" s="25"/>
-      <c r="W35" s="25"/>
-      <c r="X35" s="25"/>
-      <c r="Y35" s="25"/>
-      <c r="Z35" s="25"/>
-      <c r="AA35" s="25"/>
-      <c r="AB35" s="25"/>
-      <c r="AC35" s="25"/>
-      <c r="AD35" s="25"/>
-      <c r="AE35" s="25"/>
-      <c r="AF35" s="25"/>
-      <c r="AG35" s="25"/>
-      <c r="AH35" s="25"/>
-      <c r="AI35" s="25"/>
-      <c r="AJ35" s="25"/>
-      <c r="AK35" s="25"/>
-      <c r="AL35" s="25"/>
-      <c r="AM35" s="25"/>
-      <c r="AN35" s="25"/>
-      <c r="AO35" s="25"/>
-      <c r="AP35" s="25"/>
-      <c r="AQ35" s="25"/>
+      <c r="J35" s="32"/>
+      <c r="K35" s="32"/>
+      <c r="L35" s="32"/>
+      <c r="M35" s="32"/>
+      <c r="N35" s="32"/>
+      <c r="O35" s="32"/>
+      <c r="Q35" s="30"/>
+      <c r="R35" s="30"/>
+      <c r="S35" s="30"/>
+      <c r="T35" s="30"/>
+      <c r="U35" s="30"/>
+      <c r="V35" s="30"/>
+      <c r="W35" s="30"/>
+      <c r="X35" s="30"/>
+      <c r="Y35" s="30"/>
+      <c r="Z35" s="30"/>
+      <c r="AA35" s="30"/>
+      <c r="AB35" s="30"/>
+      <c r="AC35" s="30"/>
+      <c r="AD35" s="30"/>
+      <c r="AE35" s="30"/>
+      <c r="AF35" s="30"/>
+      <c r="AG35" s="30"/>
+      <c r="AH35" s="30"/>
+      <c r="AI35" s="30"/>
+      <c r="AJ35" s="30"/>
+      <c r="AK35" s="30"/>
+      <c r="AL35" s="30"/>
+      <c r="AM35" s="30"/>
+      <c r="AN35" s="30"/>
+      <c r="AO35" s="30"/>
+      <c r="AP35" s="30"/>
+      <c r="AQ35" s="30"/>
     </row>
     <row r="36" spans="1:43" ht="99" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="6" t="str">
         <v>BHN</v>
       </c>
-      <c r="C36" s="31" t="s">
+      <c r="C36" s="36" t="s">
         <v>74</v>
       </c>
-      <c r="D36" s="31"/>
-      <c r="E36" s="31"/>
-      <c r="F36" s="31"/>
-      <c r="G36" s="31"/>
-      <c r="H36" s="31"/>
-      <c r="I36" s="27"/>
-      <c r="J36" s="27"/>
-      <c r="K36" s="27"/>
-      <c r="L36" s="27"/>
-      <c r="M36" s="27"/>
-      <c r="N36" s="27"/>
-      <c r="O36" s="27"/>
-      <c r="Q36" s="25"/>
-      <c r="R36" s="25"/>
-      <c r="S36" s="25"/>
-      <c r="T36" s="25"/>
-      <c r="U36" s="25"/>
-      <c r="V36" s="25"/>
-      <c r="W36" s="25"/>
-      <c r="X36" s="25"/>
-      <c r="Y36" s="25"/>
-      <c r="Z36" s="25"/>
-      <c r="AA36" s="25"/>
-      <c r="AB36" s="25"/>
-      <c r="AC36" s="25"/>
-      <c r="AD36" s="25"/>
-      <c r="AE36" s="25"/>
-      <c r="AF36" s="25"/>
-      <c r="AG36" s="25"/>
-      <c r="AH36" s="25"/>
-      <c r="AI36" s="25"/>
-      <c r="AJ36" s="25"/>
-      <c r="AK36" s="25"/>
-      <c r="AL36" s="25"/>
-      <c r="AM36" s="25"/>
-      <c r="AN36" s="25"/>
-      <c r="AO36" s="25"/>
-      <c r="AP36" s="25"/>
-      <c r="AQ36" s="25"/>
+      <c r="D36" s="36"/>
+      <c r="E36" s="36"/>
+      <c r="F36" s="36"/>
+      <c r="G36" s="36"/>
+      <c r="H36" s="36"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="32"/>
+      <c r="K36" s="32"/>
+      <c r="L36" s="32"/>
+      <c r="M36" s="32"/>
+      <c r="N36" s="32"/>
+      <c r="O36" s="32"/>
+      <c r="Q36" s="30"/>
+      <c r="R36" s="30"/>
+      <c r="S36" s="30"/>
+      <c r="T36" s="30"/>
+      <c r="U36" s="30"/>
+      <c r="V36" s="30"/>
+      <c r="W36" s="30"/>
+      <c r="X36" s="30"/>
+      <c r="Y36" s="30"/>
+      <c r="Z36" s="30"/>
+      <c r="AA36" s="30"/>
+      <c r="AB36" s="30"/>
+      <c r="AC36" s="30"/>
+      <c r="AD36" s="30"/>
+      <c r="AE36" s="30"/>
+      <c r="AF36" s="30"/>
+      <c r="AG36" s="30"/>
+      <c r="AH36" s="30"/>
+      <c r="AI36" s="30"/>
+      <c r="AJ36" s="30"/>
+      <c r="AK36" s="30"/>
+      <c r="AL36" s="30"/>
+      <c r="AM36" s="30"/>
+      <c r="AN36" s="30"/>
+      <c r="AO36" s="30"/>
+      <c r="AP36" s="30"/>
+      <c r="AQ36" s="30"/>
     </row>
     <row r="37" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB37" s="25"/>
-      <c r="AC37" s="25"/>
-      <c r="AD37" s="25"/>
-      <c r="AE37" s="25"/>
-      <c r="AF37" s="25"/>
-      <c r="AG37" s="25"/>
-      <c r="AH37" s="25"/>
-      <c r="AI37" s="25"/>
-      <c r="AJ37" s="25"/>
-      <c r="AK37" s="25"/>
-      <c r="AL37" s="25"/>
-      <c r="AM37" s="25"/>
-      <c r="AN37" s="25"/>
-      <c r="AO37" s="25"/>
-      <c r="AP37" s="25"/>
-      <c r="AQ37" s="25"/>
+      <c r="AB37" s="30"/>
+      <c r="AC37" s="30"/>
+      <c r="AD37" s="30"/>
+      <c r="AE37" s="30"/>
+      <c r="AF37" s="30"/>
+      <c r="AG37" s="30"/>
+      <c r="AH37" s="30"/>
+      <c r="AI37" s="30"/>
+      <c r="AJ37" s="30"/>
+      <c r="AK37" s="30"/>
+      <c r="AL37" s="30"/>
+      <c r="AM37" s="30"/>
+      <c r="AN37" s="30"/>
+      <c r="AO37" s="30"/>
+      <c r="AP37" s="30"/>
+      <c r="AQ37" s="30"/>
     </row>
     <row r="38" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB38" s="25"/>
-      <c r="AC38" s="25"/>
-      <c r="AD38" s="25"/>
-      <c r="AE38" s="25"/>
-      <c r="AF38" s="25"/>
-      <c r="AG38" s="25"/>
-      <c r="AH38" s="25"/>
-      <c r="AI38" s="25"/>
-      <c r="AJ38" s="25"/>
-      <c r="AK38" s="25"/>
-      <c r="AL38" s="25"/>
-      <c r="AM38" s="25"/>
-      <c r="AN38" s="25"/>
-      <c r="AO38" s="25"/>
-      <c r="AP38" s="25"/>
-      <c r="AQ38" s="25"/>
+      <c r="AB38" s="30"/>
+      <c r="AC38" s="30"/>
+      <c r="AD38" s="30"/>
+      <c r="AE38" s="30"/>
+      <c r="AF38" s="30"/>
+      <c r="AG38" s="30"/>
+      <c r="AH38" s="30"/>
+      <c r="AI38" s="30"/>
+      <c r="AJ38" s="30"/>
+      <c r="AK38" s="30"/>
+      <c r="AL38" s="30"/>
+      <c r="AM38" s="30"/>
+      <c r="AN38" s="30"/>
+      <c r="AO38" s="30"/>
+      <c r="AP38" s="30"/>
+      <c r="AQ38" s="30"/>
     </row>
     <row r="39" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB39" s="25"/>
-      <c r="AC39" s="25"/>
-      <c r="AD39" s="25"/>
-      <c r="AE39" s="25"/>
-      <c r="AF39" s="25"/>
-      <c r="AG39" s="25"/>
-      <c r="AH39" s="25"/>
-      <c r="AI39" s="25"/>
-      <c r="AJ39" s="25"/>
-      <c r="AK39" s="25"/>
-      <c r="AL39" s="25"/>
-      <c r="AM39" s="25"/>
-      <c r="AN39" s="25"/>
-      <c r="AO39" s="25"/>
-      <c r="AP39" s="25"/>
-      <c r="AQ39" s="25"/>
+      <c r="AB39" s="30"/>
+      <c r="AC39" s="30"/>
+      <c r="AD39" s="30"/>
+      <c r="AE39" s="30"/>
+      <c r="AF39" s="30"/>
+      <c r="AG39" s="30"/>
+      <c r="AH39" s="30"/>
+      <c r="AI39" s="30"/>
+      <c r="AJ39" s="30"/>
+      <c r="AK39" s="30"/>
+      <c r="AL39" s="30"/>
+      <c r="AM39" s="30"/>
+      <c r="AN39" s="30"/>
+      <c r="AO39" s="30"/>
+      <c r="AP39" s="30"/>
+      <c r="AQ39" s="30"/>
     </row>
     <row r="40" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB40" s="25"/>
-      <c r="AC40" s="25"/>
-      <c r="AD40" s="25"/>
-      <c r="AE40" s="25"/>
-      <c r="AF40" s="25"/>
-      <c r="AG40" s="25"/>
-      <c r="AH40" s="25"/>
-      <c r="AI40" s="25"/>
-      <c r="AJ40" s="25"/>
-      <c r="AK40" s="25"/>
-      <c r="AL40" s="25"/>
-      <c r="AM40" s="25"/>
-      <c r="AN40" s="25"/>
-      <c r="AO40" s="25"/>
-      <c r="AP40" s="25"/>
-      <c r="AQ40" s="25"/>
+      <c r="AB40" s="30"/>
+      <c r="AC40" s="30"/>
+      <c r="AD40" s="30"/>
+      <c r="AE40" s="30"/>
+      <c r="AF40" s="30"/>
+      <c r="AG40" s="30"/>
+      <c r="AH40" s="30"/>
+      <c r="AI40" s="30"/>
+      <c r="AJ40" s="30"/>
+      <c r="AK40" s="30"/>
+      <c r="AL40" s="30"/>
+      <c r="AM40" s="30"/>
+      <c r="AN40" s="30"/>
+      <c r="AO40" s="30"/>
+      <c r="AP40" s="30"/>
+      <c r="AQ40" s="30"/>
     </row>
     <row r="41" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB41" s="25"/>
-      <c r="AC41" s="25"/>
-      <c r="AD41" s="25"/>
-      <c r="AE41" s="25"/>
-      <c r="AF41" s="25"/>
-      <c r="AG41" s="25"/>
-      <c r="AH41" s="25"/>
-      <c r="AI41" s="25"/>
-      <c r="AJ41" s="25"/>
-      <c r="AK41" s="25"/>
-      <c r="AL41" s="25"/>
-      <c r="AM41" s="25"/>
-      <c r="AN41" s="25"/>
-      <c r="AO41" s="25"/>
-      <c r="AP41" s="25"/>
-      <c r="AQ41" s="25"/>
+      <c r="AB41" s="30"/>
+      <c r="AC41" s="30"/>
+      <c r="AD41" s="30"/>
+      <c r="AE41" s="30"/>
+      <c r="AF41" s="30"/>
+      <c r="AG41" s="30"/>
+      <c r="AH41" s="30"/>
+      <c r="AI41" s="30"/>
+      <c r="AJ41" s="30"/>
+      <c r="AK41" s="30"/>
+      <c r="AL41" s="30"/>
+      <c r="AM41" s="30"/>
+      <c r="AN41" s="30"/>
+      <c r="AO41" s="30"/>
+      <c r="AP41" s="30"/>
+      <c r="AQ41" s="30"/>
     </row>
     <row r="42" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB42" s="25" t="e" vm="8">
+      <c r="AB42" s="30" t="e" vm="8">
         <v>#VALUE!</v>
       </c>
-      <c r="AC42" s="25"/>
-      <c r="AD42" s="25"/>
-      <c r="AE42" s="25"/>
-      <c r="AF42" s="25"/>
-      <c r="AG42" s="25"/>
-      <c r="AH42" s="25"/>
-      <c r="AI42" s="25"/>
-      <c r="AJ42" s="25"/>
-      <c r="AK42" s="25"/>
-      <c r="AL42" s="25"/>
-      <c r="AM42" s="25"/>
-      <c r="AN42" s="25"/>
-      <c r="AO42" s="25"/>
-      <c r="AP42" s="25"/>
-      <c r="AQ42" s="25"/>
+      <c r="AC42" s="30"/>
+      <c r="AD42" s="30"/>
+      <c r="AE42" s="30"/>
+      <c r="AF42" s="30"/>
+      <c r="AG42" s="30"/>
+      <c r="AH42" s="30"/>
+      <c r="AI42" s="30"/>
+      <c r="AJ42" s="30"/>
+      <c r="AK42" s="30"/>
+      <c r="AL42" s="30"/>
+      <c r="AM42" s="30"/>
+      <c r="AN42" s="30"/>
+      <c r="AO42" s="30"/>
+      <c r="AP42" s="30"/>
+      <c r="AQ42" s="30"/>
     </row>
     <row r="43" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB43" s="25"/>
-      <c r="AC43" s="25"/>
-      <c r="AD43" s="25"/>
-      <c r="AE43" s="25"/>
-      <c r="AF43" s="25"/>
-      <c r="AG43" s="25"/>
-      <c r="AH43" s="25"/>
-      <c r="AI43" s="25"/>
-      <c r="AJ43" s="25"/>
-      <c r="AK43" s="25"/>
-      <c r="AL43" s="25"/>
-      <c r="AM43" s="25"/>
-      <c r="AN43" s="25"/>
-      <c r="AO43" s="25"/>
-      <c r="AP43" s="25"/>
-      <c r="AQ43" s="25"/>
+      <c r="AB43" s="30"/>
+      <c r="AC43" s="30"/>
+      <c r="AD43" s="30"/>
+      <c r="AE43" s="30"/>
+      <c r="AF43" s="30"/>
+      <c r="AG43" s="30"/>
+      <c r="AH43" s="30"/>
+      <c r="AI43" s="30"/>
+      <c r="AJ43" s="30"/>
+      <c r="AK43" s="30"/>
+      <c r="AL43" s="30"/>
+      <c r="AM43" s="30"/>
+      <c r="AN43" s="30"/>
+      <c r="AO43" s="30"/>
+      <c r="AP43" s="30"/>
+      <c r="AQ43" s="30"/>
     </row>
     <row r="44" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB44" s="25"/>
-      <c r="AC44" s="25"/>
-      <c r="AD44" s="25"/>
-      <c r="AE44" s="25"/>
-      <c r="AF44" s="25"/>
-      <c r="AG44" s="25"/>
-      <c r="AH44" s="25"/>
-      <c r="AI44" s="25"/>
-      <c r="AJ44" s="25"/>
-      <c r="AK44" s="25"/>
-      <c r="AL44" s="25"/>
-      <c r="AM44" s="25"/>
-      <c r="AN44" s="25"/>
-      <c r="AO44" s="25"/>
-      <c r="AP44" s="25"/>
-      <c r="AQ44" s="25"/>
+      <c r="AB44" s="30"/>
+      <c r="AC44" s="30"/>
+      <c r="AD44" s="30"/>
+      <c r="AE44" s="30"/>
+      <c r="AF44" s="30"/>
+      <c r="AG44" s="30"/>
+      <c r="AH44" s="30"/>
+      <c r="AI44" s="30"/>
+      <c r="AJ44" s="30"/>
+      <c r="AK44" s="30"/>
+      <c r="AL44" s="30"/>
+      <c r="AM44" s="30"/>
+      <c r="AN44" s="30"/>
+      <c r="AO44" s="30"/>
+      <c r="AP44" s="30"/>
+      <c r="AQ44" s="30"/>
     </row>
     <row r="45" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB45" s="25"/>
-      <c r="AC45" s="25"/>
-      <c r="AD45" s="25"/>
-      <c r="AE45" s="25"/>
-      <c r="AF45" s="25"/>
-      <c r="AG45" s="25"/>
-      <c r="AH45" s="25"/>
-      <c r="AI45" s="25"/>
-      <c r="AJ45" s="25"/>
-      <c r="AK45" s="25"/>
-      <c r="AL45" s="25"/>
-      <c r="AM45" s="25"/>
-      <c r="AN45" s="25"/>
-      <c r="AO45" s="25"/>
-      <c r="AP45" s="25"/>
-      <c r="AQ45" s="25"/>
+      <c r="AB45" s="30"/>
+      <c r="AC45" s="30"/>
+      <c r="AD45" s="30"/>
+      <c r="AE45" s="30"/>
+      <c r="AF45" s="30"/>
+      <c r="AG45" s="30"/>
+      <c r="AH45" s="30"/>
+      <c r="AI45" s="30"/>
+      <c r="AJ45" s="30"/>
+      <c r="AK45" s="30"/>
+      <c r="AL45" s="30"/>
+      <c r="AM45" s="30"/>
+      <c r="AN45" s="30"/>
+      <c r="AO45" s="30"/>
+      <c r="AP45" s="30"/>
+      <c r="AQ45" s="30"/>
     </row>
     <row r="46" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB46" s="25"/>
-      <c r="AC46" s="25"/>
-      <c r="AD46" s="25"/>
-      <c r="AE46" s="25"/>
-      <c r="AF46" s="25"/>
-      <c r="AG46" s="25"/>
-      <c r="AH46" s="25"/>
-      <c r="AI46" s="25"/>
-      <c r="AJ46" s="25"/>
-      <c r="AK46" s="25"/>
-      <c r="AL46" s="25"/>
-      <c r="AM46" s="25"/>
-      <c r="AN46" s="25"/>
-      <c r="AO46" s="25"/>
-      <c r="AP46" s="25"/>
-      <c r="AQ46" s="25"/>
+      <c r="AB46" s="30"/>
+      <c r="AC46" s="30"/>
+      <c r="AD46" s="30"/>
+      <c r="AE46" s="30"/>
+      <c r="AF46" s="30"/>
+      <c r="AG46" s="30"/>
+      <c r="AH46" s="30"/>
+      <c r="AI46" s="30"/>
+      <c r="AJ46" s="30"/>
+      <c r="AK46" s="30"/>
+      <c r="AL46" s="30"/>
+      <c r="AM46" s="30"/>
+      <c r="AN46" s="30"/>
+      <c r="AO46" s="30"/>
+      <c r="AP46" s="30"/>
+      <c r="AQ46" s="30"/>
     </row>
     <row r="47" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB47" s="25"/>
-      <c r="AC47" s="25"/>
-      <c r="AD47" s="25"/>
-      <c r="AE47" s="25"/>
-      <c r="AF47" s="25"/>
-      <c r="AG47" s="25"/>
-      <c r="AH47" s="25"/>
-      <c r="AI47" s="25"/>
-      <c r="AJ47" s="25"/>
-      <c r="AK47" s="25"/>
-      <c r="AL47" s="25"/>
-      <c r="AM47" s="25"/>
-      <c r="AN47" s="25"/>
-      <c r="AO47" s="25"/>
-      <c r="AP47" s="25"/>
-      <c r="AQ47" s="25"/>
+      <c r="AB47" s="30"/>
+      <c r="AC47" s="30"/>
+      <c r="AD47" s="30"/>
+      <c r="AE47" s="30"/>
+      <c r="AF47" s="30"/>
+      <c r="AG47" s="30"/>
+      <c r="AH47" s="30"/>
+      <c r="AI47" s="30"/>
+      <c r="AJ47" s="30"/>
+      <c r="AK47" s="30"/>
+      <c r="AL47" s="30"/>
+      <c r="AM47" s="30"/>
+      <c r="AN47" s="30"/>
+      <c r="AO47" s="30"/>
+      <c r="AP47" s="30"/>
+      <c r="AQ47" s="30"/>
     </row>
     <row r="48" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB48" s="25"/>
-      <c r="AC48" s="25"/>
-      <c r="AD48" s="25"/>
-      <c r="AE48" s="25"/>
-      <c r="AF48" s="25"/>
-      <c r="AG48" s="25"/>
-      <c r="AH48" s="25"/>
-      <c r="AI48" s="25"/>
-      <c r="AJ48" s="25"/>
-      <c r="AK48" s="25"/>
-      <c r="AL48" s="25"/>
-      <c r="AM48" s="25"/>
-      <c r="AN48" s="25"/>
-      <c r="AO48" s="25"/>
-      <c r="AP48" s="25"/>
-      <c r="AQ48" s="25"/>
+      <c r="AB48" s="30"/>
+      <c r="AC48" s="30"/>
+      <c r="AD48" s="30"/>
+      <c r="AE48" s="30"/>
+      <c r="AF48" s="30"/>
+      <c r="AG48" s="30"/>
+      <c r="AH48" s="30"/>
+      <c r="AI48" s="30"/>
+      <c r="AJ48" s="30"/>
+      <c r="AK48" s="30"/>
+      <c r="AL48" s="30"/>
+      <c r="AM48" s="30"/>
+      <c r="AN48" s="30"/>
+      <c r="AO48" s="30"/>
+      <c r="AP48" s="30"/>
+      <c r="AQ48" s="30"/>
     </row>
     <row r="49" spans="28:43" x14ac:dyDescent="0.3">
-      <c r="AB49" s="25"/>
-      <c r="AC49" s="25"/>
-      <c r="AD49" s="25"/>
-      <c r="AE49" s="25"/>
-      <c r="AF49" s="25"/>
-      <c r="AG49" s="25"/>
-      <c r="AH49" s="25"/>
-      <c r="AI49" s="25"/>
-      <c r="AJ49" s="25"/>
-      <c r="AK49" s="25"/>
-      <c r="AL49" s="25"/>
-      <c r="AM49" s="25"/>
-      <c r="AN49" s="25"/>
-      <c r="AO49" s="25"/>
-      <c r="AP49" s="25"/>
-      <c r="AQ49" s="25"/>
+      <c r="AB49" s="30"/>
+      <c r="AC49" s="30"/>
+      <c r="AD49" s="30"/>
+      <c r="AE49" s="30"/>
+      <c r="AF49" s="30"/>
+      <c r="AG49" s="30"/>
+      <c r="AH49" s="30"/>
+      <c r="AI49" s="30"/>
+      <c r="AJ49" s="30"/>
+      <c r="AK49" s="30"/>
+      <c r="AL49" s="30"/>
+      <c r="AM49" s="30"/>
+      <c r="AN49" s="30"/>
+      <c r="AO49" s="30"/>
+      <c r="AP49" s="30"/>
+      <c r="AQ49" s="30"/>
     </row>
     <row r="50" spans="28:43" x14ac:dyDescent="0.3">
-      <c r="AB50" s="25"/>
-      <c r="AC50" s="25"/>
-      <c r="AD50" s="25"/>
-      <c r="AE50" s="25"/>
-      <c r="AF50" s="25"/>
-      <c r="AG50" s="25"/>
-      <c r="AH50" s="25"/>
-      <c r="AI50" s="25"/>
-      <c r="AJ50" s="25"/>
-      <c r="AK50" s="25"/>
-      <c r="AL50" s="25"/>
-      <c r="AM50" s="25"/>
-      <c r="AN50" s="25"/>
-      <c r="AO50" s="25"/>
-      <c r="AP50" s="25"/>
-      <c r="AQ50" s="25"/>
+      <c r="AB50" s="30"/>
+      <c r="AC50" s="30"/>
+      <c r="AD50" s="30"/>
+      <c r="AE50" s="30"/>
+      <c r="AF50" s="30"/>
+      <c r="AG50" s="30"/>
+      <c r="AH50" s="30"/>
+      <c r="AI50" s="30"/>
+      <c r="AJ50" s="30"/>
+      <c r="AK50" s="30"/>
+      <c r="AL50" s="30"/>
+      <c r="AM50" s="30"/>
+      <c r="AN50" s="30"/>
+      <c r="AO50" s="30"/>
+      <c r="AP50" s="30"/>
+      <c r="AQ50" s="30"/>
     </row>
     <row r="51" spans="28:43" x14ac:dyDescent="0.3">
-      <c r="AB51" s="25"/>
-      <c r="AC51" s="25"/>
-      <c r="AD51" s="25"/>
-      <c r="AE51" s="25"/>
-      <c r="AF51" s="25"/>
-      <c r="AG51" s="25"/>
-      <c r="AH51" s="25"/>
-      <c r="AI51" s="25"/>
-      <c r="AJ51" s="25"/>
-      <c r="AK51" s="25"/>
-      <c r="AL51" s="25"/>
-      <c r="AM51" s="25"/>
-      <c r="AN51" s="25"/>
-      <c r="AO51" s="25"/>
-      <c r="AP51" s="25"/>
-      <c r="AQ51" s="25"/>
+      <c r="AB51" s="30"/>
+      <c r="AC51" s="30"/>
+      <c r="AD51" s="30"/>
+      <c r="AE51" s="30"/>
+      <c r="AF51" s="30"/>
+      <c r="AG51" s="30"/>
+      <c r="AH51" s="30"/>
+      <c r="AI51" s="30"/>
+      <c r="AJ51" s="30"/>
+      <c r="AK51" s="30"/>
+      <c r="AL51" s="30"/>
+      <c r="AM51" s="30"/>
+      <c r="AN51" s="30"/>
+      <c r="AO51" s="30"/>
+      <c r="AP51" s="30"/>
+      <c r="AQ51" s="30"/>
     </row>
     <row r="52" spans="28:43" x14ac:dyDescent="0.3">
-      <c r="AB52" s="25"/>
-      <c r="AC52" s="25"/>
-      <c r="AD52" s="25"/>
-      <c r="AE52" s="25"/>
-      <c r="AF52" s="25"/>
-      <c r="AG52" s="25"/>
-      <c r="AH52" s="25"/>
-      <c r="AI52" s="25"/>
-      <c r="AJ52" s="25"/>
-      <c r="AK52" s="25"/>
-      <c r="AL52" s="25"/>
-      <c r="AM52" s="25"/>
-      <c r="AN52" s="25"/>
-      <c r="AO52" s="25"/>
-      <c r="AP52" s="25"/>
-      <c r="AQ52" s="25"/>
+      <c r="AB52" s="30"/>
+      <c r="AC52" s="30"/>
+      <c r="AD52" s="30"/>
+      <c r="AE52" s="30"/>
+      <c r="AF52" s="30"/>
+      <c r="AG52" s="30"/>
+      <c r="AH52" s="30"/>
+      <c r="AI52" s="30"/>
+      <c r="AJ52" s="30"/>
+      <c r="AK52" s="30"/>
+      <c r="AL52" s="30"/>
+      <c r="AM52" s="30"/>
+      <c r="AN52" s="30"/>
+      <c r="AO52" s="30"/>
+      <c r="AP52" s="30"/>
+      <c r="AQ52" s="30"/>
     </row>
     <row r="53" spans="28:43" x14ac:dyDescent="0.3">
-      <c r="AB53" s="25"/>
-      <c r="AC53" s="25"/>
-      <c r="AD53" s="25"/>
-      <c r="AE53" s="25"/>
-      <c r="AF53" s="25"/>
-      <c r="AG53" s="25"/>
-      <c r="AH53" s="25"/>
-      <c r="AI53" s="25"/>
-      <c r="AJ53" s="25"/>
-      <c r="AK53" s="25"/>
-      <c r="AL53" s="25"/>
-      <c r="AM53" s="25"/>
-      <c r="AN53" s="25"/>
-      <c r="AO53" s="25"/>
-      <c r="AP53" s="25"/>
-      <c r="AQ53" s="25"/>
+      <c r="AB53" s="30"/>
+      <c r="AC53" s="30"/>
+      <c r="AD53" s="30"/>
+      <c r="AE53" s="30"/>
+      <c r="AF53" s="30"/>
+      <c r="AG53" s="30"/>
+      <c r="AH53" s="30"/>
+      <c r="AI53" s="30"/>
+      <c r="AJ53" s="30"/>
+      <c r="AK53" s="30"/>
+      <c r="AL53" s="30"/>
+      <c r="AM53" s="30"/>
+      <c r="AN53" s="30"/>
+      <c r="AO53" s="30"/>
+      <c r="AP53" s="30"/>
+      <c r="AQ53" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="42">
-    <mergeCell ref="C24:H24"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C26:H26"/>
+  <mergeCells count="43">
     <mergeCell ref="C27:H27"/>
     <mergeCell ref="I24:O24"/>
     <mergeCell ref="I25:O25"/>
@@ -3462,6 +3473,7 @@
     <mergeCell ref="I23:O23"/>
     <mergeCell ref="C3:H3"/>
     <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C28:H28"/>
     <mergeCell ref="I28:O28"/>
     <mergeCell ref="I29:O29"/>
     <mergeCell ref="AR22:AY24"/>
@@ -3474,6 +3486,10 @@
     <mergeCell ref="I34:O34"/>
     <mergeCell ref="AB22:AQ27"/>
     <mergeCell ref="Q22:AA25"/>
+    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C26:H26"/>
+    <mergeCell ref="T4:X4"/>
     <mergeCell ref="AB42:AQ53"/>
     <mergeCell ref="C30:H30"/>
     <mergeCell ref="AB28:AQ31"/>
@@ -3489,7 +3505,6 @@
     <mergeCell ref="I31:O31"/>
     <mergeCell ref="C36:H36"/>
     <mergeCell ref="I36:O36"/>
-    <mergeCell ref="C28:H28"/>
   </mergeCells>
   <conditionalFormatting sqref="C5:Q15">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
@@ -3523,84 +3538,84 @@
       <c r="B3" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="33"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="33"/>
-      <c r="J3" s="41"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="38"/>
+      <c r="J3" s="39"/>
       <c r="K3" s="8"/>
       <c r="L3" s="8"/>
       <c r="M3" s="8"/>
       <c r="N3" s="8"/>
       <c r="O3" s="8"/>
-      <c r="T3" s="24" t="s">
+      <c r="T3" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="U3" s="24"/>
-      <c r="V3" s="24"/>
-      <c r="W3" s="24"/>
-      <c r="X3" s="24"/>
+      <c r="U3" s="22"/>
+      <c r="V3" s="22"/>
+      <c r="W3" s="22"/>
+      <c r="X3" s="22"/>
     </row>
     <row r="4" spans="1:24" ht="221.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="42" t="str" cm="1">
+      <c r="C4" s="25" t="str" cm="1">
         <f t="array" ref="C4:Q4">Experiments!C1:Q1</f>
         <v>BHN_FWB</v>
       </c>
-      <c r="D4" s="46" t="str">
+      <c r="D4" s="23" t="str">
         <v>BHN_FWB_AllExt</v>
       </c>
-      <c r="E4" s="43" t="str">
+      <c r="E4" s="9" t="str">
         <v>Few_indicators_closest_DLS_coverage</v>
       </c>
-      <c r="F4" s="43" t="str">
+      <c r="F4" s="9" t="str">
         <v>Few indicators_SPI_preferred</v>
       </c>
-      <c r="G4" s="43" t="str">
+      <c r="G4" s="9" t="str">
         <v>No_non_DLS</v>
       </c>
-      <c r="H4" s="40" t="str">
+      <c r="H4" s="24" t="str">
         <v>Only_%_of_pop</v>
       </c>
-      <c r="I4" s="42" t="str">
+      <c r="I4" s="25" t="str">
         <v>Few_indicators_closest_DLS_coverage_90</v>
       </c>
-      <c r="J4" s="43" t="str">
+      <c r="J4" s="9" t="str">
         <v>Few indicators_SPI_preferred_90</v>
       </c>
-      <c r="K4" s="39" t="str">
+      <c r="K4" s="23" t="str">
         <v>Few_indicators_closeDLS_subPrimSchool</v>
       </c>
-      <c r="L4" s="39" t="str">
+      <c r="L4" s="23" t="str">
         <v>No_non_DLS_90</v>
       </c>
-      <c r="M4" s="39" t="str">
+      <c r="M4" s="23" t="str">
         <v>Few_Indicators_subWatSani</v>
       </c>
-      <c r="N4" s="39" t="str">
+      <c r="N4" s="23" t="str">
         <v>Only_OPP</v>
       </c>
       <c r="O4" s="9" t="str">
         <v>Baseline</v>
       </c>
-      <c r="P4" s="39" t="str">
+      <c r="P4" s="23" t="str">
         <v>No_nonDLS_limExt</v>
       </c>
-      <c r="Q4" s="39" t="str">
+      <c r="Q4" s="23" t="str">
         <v>BHN</v>
       </c>
-      <c r="T4" s="47" t="s">
+      <c r="T4" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="U4" s="47"/>
-      <c r="V4" s="47"/>
-      <c r="W4" s="47"/>
-      <c r="X4" s="47"/>
+      <c r="U4" s="29"/>
+      <c r="V4" s="29"/>
+      <c r="W4" s="29"/>
+      <c r="X4" s="29"/>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="B5" s="11" t="str" cm="1">
@@ -3611,19 +3626,19 @@
         <f t="array" ref="C5">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B5)*(Experiments!C$2:C$64=1))</f>
         <v>3</v>
       </c>
-      <c r="D5" s="44" cm="1">
+      <c r="D5" s="8" cm="1">
         <f t="array" ref="D5">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B5)*(Experiments!D$2:D$64=1))</f>
         <v>5</v>
       </c>
-      <c r="E5" s="44" cm="1">
+      <c r="E5" s="8" cm="1">
         <f t="array" ref="E5">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B5)*(Experiments!E$2:E$64=1))</f>
         <v>1</v>
       </c>
-      <c r="F5" s="44" cm="1">
+      <c r="F5" s="8" cm="1">
         <f t="array" ref="F5">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B5)*(Experiments!F$2:F$64=1))</f>
         <v>1</v>
       </c>
-      <c r="G5" s="44" cm="1">
+      <c r="G5" s="8" cm="1">
         <f t="array" ref="G5">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B5)*(Experiments!G$2:G$64=1))</f>
         <v>5</v>
       </c>
@@ -3635,7 +3650,7 @@
         <f t="array" ref="I5">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B5)*(Experiments!I$2:I$64=1))</f>
         <v>1</v>
       </c>
-      <c r="J5" s="44" cm="1">
+      <c r="J5" s="8" cm="1">
         <f t="array" ref="J5">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B5)*(Experiments!J$2:J$64=1))</f>
         <v>1</v>
       </c>
@@ -3679,19 +3694,19 @@
         <f t="array" ref="C6">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B6)*(Experiments!C$2:C$64=1))</f>
         <v>7</v>
       </c>
-      <c r="D6" s="44" cm="1">
+      <c r="D6" s="8" cm="1">
         <f t="array" ref="D6">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B6)*(Experiments!D$2:D$64=1))</f>
         <v>10</v>
       </c>
-      <c r="E6" s="44" cm="1">
+      <c r="E6" s="8" cm="1">
         <f t="array" ref="E6">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B6)*(Experiments!E$2:E$64=1))</f>
         <v>1</v>
       </c>
-      <c r="F6" s="44" cm="1">
+      <c r="F6" s="8" cm="1">
         <f t="array" ref="F6">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B6)*(Experiments!F$2:F$64=1))</f>
         <v>1</v>
       </c>
-      <c r="G6" s="44" cm="1">
+      <c r="G6" s="8" cm="1">
         <f t="array" ref="G6">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B6)*(Experiments!G$2:G$64=1))</f>
         <v>10</v>
       </c>
@@ -3703,7 +3718,7 @@
         <f t="array" ref="I6">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B6)*(Experiments!I$2:I$64=1))</f>
         <v>1</v>
       </c>
-      <c r="J6" s="44" cm="1">
+      <c r="J6" s="8" cm="1">
         <f t="array" ref="J6">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B6)*(Experiments!J$2:J$64=1))</f>
         <v>1</v>
       </c>
@@ -3744,19 +3759,19 @@
         <f t="array" ref="C7">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B7)*(Experiments!C$2:C$64=1))</f>
         <v>3</v>
       </c>
-      <c r="D7" s="44" cm="1">
+      <c r="D7" s="8" cm="1">
         <f t="array" ref="D7">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B7)*(Experiments!D$2:D$64=1))</f>
         <v>4</v>
       </c>
-      <c r="E7" s="44" cm="1">
+      <c r="E7" s="8" cm="1">
         <f t="array" ref="E7">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B7)*(Experiments!E$2:E$64=1))</f>
         <v>2</v>
       </c>
-      <c r="F7" s="44" cm="1">
+      <c r="F7" s="8" cm="1">
         <f t="array" ref="F7">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B7)*(Experiments!F$2:F$64=1))</f>
         <v>2</v>
       </c>
-      <c r="G7" s="44" cm="1">
+      <c r="G7" s="8" cm="1">
         <f t="array" ref="G7">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B7)*(Experiments!G$2:G$64=1))</f>
         <v>4</v>
       </c>
@@ -3768,7 +3783,7 @@
         <f t="array" ref="I7">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B7)*(Experiments!I$2:I$64=1))</f>
         <v>2</v>
       </c>
-      <c r="J7" s="44" cm="1">
+      <c r="J7" s="8" cm="1">
         <f t="array" ref="J7">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B7)*(Experiments!J$2:J$64=1))</f>
         <v>2</v>
       </c>
@@ -3809,19 +3824,19 @@
         <f t="array" ref="C8">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B8)*(Experiments!C$2:C$64=1))</f>
         <v>1</v>
       </c>
-      <c r="D8" s="44" cm="1">
+      <c r="D8" s="8" cm="1">
         <f t="array" ref="D8">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B8)*(Experiments!D$2:D$64=1))</f>
         <v>2</v>
       </c>
-      <c r="E8" s="44" cm="1">
+      <c r="E8" s="8" cm="1">
         <f t="array" ref="E8">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B8)*(Experiments!E$2:E$64=1))</f>
         <v>1</v>
       </c>
-      <c r="F8" s="44" cm="1">
+      <c r="F8" s="8" cm="1">
         <f t="array" ref="F8">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B8)*(Experiments!F$2:F$64=1))</f>
         <v>1</v>
       </c>
-      <c r="G8" s="44" cm="1">
+      <c r="G8" s="8" cm="1">
         <f t="array" ref="G8">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B8)*(Experiments!G$2:G$64=1))</f>
         <v>2</v>
       </c>
@@ -3833,7 +3848,7 @@
         <f t="array" ref="I8">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B8)*(Experiments!I$2:I$64=1))</f>
         <v>1</v>
       </c>
-      <c r="J8" s="44" cm="1">
+      <c r="J8" s="8" cm="1">
         <f t="array" ref="J8">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B8)*(Experiments!J$2:J$64=1))</f>
         <v>1</v>
       </c>
@@ -3874,19 +3889,19 @@
         <f t="array" ref="C9">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B9)*(Experiments!C$2:C$64=1))</f>
         <v>2</v>
       </c>
-      <c r="D9" s="44" cm="1">
+      <c r="D9" s="8" cm="1">
         <f t="array" ref="D9">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B9)*(Experiments!D$2:D$64=1))</f>
         <v>3</v>
       </c>
-      <c r="E9" s="44" cm="1">
+      <c r="E9" s="8" cm="1">
         <f t="array" ref="E9">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B9)*(Experiments!E$2:E$64=1))</f>
         <v>1</v>
       </c>
-      <c r="F9" s="44" cm="1">
+      <c r="F9" s="8" cm="1">
         <f t="array" ref="F9">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B9)*(Experiments!F$2:F$64=1))</f>
         <v>1</v>
       </c>
-      <c r="G9" s="44" cm="1">
+      <c r="G9" s="8" cm="1">
         <f t="array" ref="G9">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B9)*(Experiments!G$2:G$64=1))</f>
         <v>3</v>
       </c>
@@ -3898,7 +3913,7 @@
         <f t="array" ref="I9">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B9)*(Experiments!I$2:I$64=1))</f>
         <v>1</v>
       </c>
-      <c r="J9" s="44" cm="1">
+      <c r="J9" s="8" cm="1">
         <f t="array" ref="J9">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B9)*(Experiments!J$2:J$64=1))</f>
         <v>1</v>
       </c>
@@ -3939,19 +3954,19 @@
         <f t="array" ref="C10">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B10)*(Experiments!C$2:C$64=1))</f>
         <v>1</v>
       </c>
-      <c r="D10" s="44" cm="1">
+      <c r="D10" s="8" cm="1">
         <f t="array" ref="D10">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B10)*(Experiments!D$2:D$64=1))</f>
         <v>1</v>
       </c>
-      <c r="E10" s="44" cm="1">
+      <c r="E10" s="8" cm="1">
         <f t="array" ref="E10">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B10)*(Experiments!E$2:E$64=1))</f>
         <v>1</v>
       </c>
-      <c r="F10" s="44" cm="1">
+      <c r="F10" s="8" cm="1">
         <f t="array" ref="F10">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B10)*(Experiments!F$2:F$64=1))</f>
         <v>1</v>
       </c>
-      <c r="G10" s="44" cm="1">
+      <c r="G10" s="8" cm="1">
         <f t="array" ref="G10">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B10)*(Experiments!G$2:G$64=1))</f>
         <v>1</v>
       </c>
@@ -3963,7 +3978,7 @@
         <f t="array" ref="I10">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B10)*(Experiments!I$2:I$64=1))</f>
         <v>1</v>
       </c>
-      <c r="J10" s="44" cm="1">
+      <c r="J10" s="8" cm="1">
         <f t="array" ref="J10">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B10)*(Experiments!J$2:J$64=1))</f>
         <v>1</v>
       </c>
@@ -4004,19 +4019,19 @@
         <f t="array" ref="C11">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B11)*(Experiments!C$2:C$64=1))</f>
         <v>9</v>
       </c>
-      <c r="D11" s="44" cm="1">
+      <c r="D11" s="8" cm="1">
         <f t="array" ref="D11">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B11)*(Experiments!D$2:D$64=1))</f>
         <v>10</v>
       </c>
-      <c r="E11" s="44" cm="1">
+      <c r="E11" s="8" cm="1">
         <f t="array" ref="E11">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B11)*(Experiments!E$2:E$64=1))</f>
         <v>0</v>
       </c>
-      <c r="F11" s="44" cm="1">
+      <c r="F11" s="8" cm="1">
         <f t="array" ref="F11">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B11)*(Experiments!F$2:F$64=1))</f>
         <v>0</v>
       </c>
-      <c r="G11" s="44" cm="1">
+      <c r="G11" s="8" cm="1">
         <f t="array" ref="G11">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B11)*(Experiments!G$2:G$64=1))</f>
         <v>0</v>
       </c>
@@ -4028,7 +4043,7 @@
         <f t="array" ref="I11">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B11)*(Experiments!I$2:I$64=1))</f>
         <v>0</v>
       </c>
-      <c r="J11" s="44" cm="1">
+      <c r="J11" s="8" cm="1">
         <f t="array" ref="J11">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B11)*(Experiments!J$2:J$64=1))</f>
         <v>0</v>
       </c>
@@ -4069,19 +4084,19 @@
         <f t="array" ref="C12">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B12)*(Experiments!C$2:C$64=1))</f>
         <v>4</v>
       </c>
-      <c r="D12" s="44" cm="1">
+      <c r="D12" s="8" cm="1">
         <f t="array" ref="D12">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B12)*(Experiments!D$2:D$64=1))</f>
         <v>5</v>
       </c>
-      <c r="E12" s="44" cm="1">
+      <c r="E12" s="8" cm="1">
         <f t="array" ref="E12">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B12)*(Experiments!E$2:E$64=1))</f>
         <v>1</v>
       </c>
-      <c r="F12" s="44" cm="1">
+      <c r="F12" s="8" cm="1">
         <f t="array" ref="F12">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B12)*(Experiments!F$2:F$64=1))</f>
         <v>1</v>
       </c>
-      <c r="G12" s="44" cm="1">
+      <c r="G12" s="8" cm="1">
         <f t="array" ref="G12">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B12)*(Experiments!G$2:G$64=1))</f>
         <v>9</v>
       </c>
@@ -4093,7 +4108,7 @@
         <f t="array" ref="I12">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B12)*(Experiments!I$2:I$64=1))</f>
         <v>1</v>
       </c>
-      <c r="J12" s="44" cm="1">
+      <c r="J12" s="8" cm="1">
         <f t="array" ref="J12">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B12)*(Experiments!J$2:J$64=1))</f>
         <v>1</v>
       </c>
@@ -4134,19 +4149,19 @@
         <f t="array" ref="C13">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B13)*(Experiments!C$2:C$64=1))</f>
         <v>3</v>
       </c>
-      <c r="D13" s="44" cm="1">
+      <c r="D13" s="8" cm="1">
         <f t="array" ref="D13">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B13)*(Experiments!D$2:D$64=1))</f>
         <v>3</v>
       </c>
-      <c r="E13" s="44" cm="1">
+      <c r="E13" s="8" cm="1">
         <f t="array" ref="E13">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B13)*(Experiments!E$2:E$64=1))</f>
         <v>2</v>
       </c>
-      <c r="F13" s="44" cm="1">
+      <c r="F13" s="8" cm="1">
         <f t="array" ref="F13">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B13)*(Experiments!F$2:F$64=1))</f>
         <v>2</v>
       </c>
-      <c r="G13" s="44" cm="1">
+      <c r="G13" s="8" cm="1">
         <f t="array" ref="G13">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B13)*(Experiments!G$2:G$64=1))</f>
         <v>3</v>
       </c>
@@ -4158,7 +4173,7 @@
         <f t="array" ref="I13">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B13)*(Experiments!I$2:I$64=1))</f>
         <v>2</v>
       </c>
-      <c r="J13" s="44" cm="1">
+      <c r="J13" s="8" cm="1">
         <f t="array" ref="J13">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B13)*(Experiments!J$2:J$64=1))</f>
         <v>2</v>
       </c>
@@ -4199,19 +4214,19 @@
         <f t="array" ref="C14">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B14)*(Experiments!C$2:C$64=1))</f>
         <v>0</v>
       </c>
-      <c r="D14" s="44" cm="1">
+      <c r="D14" s="8" cm="1">
         <f t="array" ref="D14">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B14)*(Experiments!D$2:D$64=1))</f>
         <v>1</v>
       </c>
-      <c r="E14" s="44" cm="1">
+      <c r="E14" s="8" cm="1">
         <f t="array" ref="E14">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B14)*(Experiments!E$2:E$64=1))</f>
         <v>1</v>
       </c>
-      <c r="F14" s="44" cm="1">
+      <c r="F14" s="8" cm="1">
         <f t="array" ref="F14">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B14)*(Experiments!F$2:F$64=1))</f>
         <v>1</v>
       </c>
-      <c r="G14" s="44" cm="1">
+      <c r="G14" s="8" cm="1">
         <f t="array" ref="G14">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B14)*(Experiments!G$2:G$64=1))</f>
         <v>1</v>
       </c>
@@ -4223,7 +4238,7 @@
         <f t="array" ref="I14">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B14)*(Experiments!I$2:I$64=1))</f>
         <v>1</v>
       </c>
-      <c r="J14" s="44" cm="1">
+      <c r="J14" s="8" cm="1">
         <f t="array" ref="J14">SUMPRODUCT(('Overview of indicators and DLS'!$C$4:$C$66=$B14)*(Experiments!J$2:J$64=1))</f>
         <v>1</v>
       </c>
@@ -4327,13 +4342,13 @@
     <row r="16" spans="1:24" x14ac:dyDescent="0.3">
       <c r="B16" s="11"/>
       <c r="C16" s="20"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="44"/>
-      <c r="F16" s="44"/>
-      <c r="G16" s="44"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
       <c r="H16" s="11"/>
       <c r="I16" s="18"/>
-      <c r="J16" s="44"/>
+      <c r="J16" s="8"/>
       <c r="K16" s="8"/>
       <c r="L16" s="8"/>
       <c r="M16" s="8"/>
@@ -4350,19 +4365,19 @@
         <f>SUM(C5:C15)</f>
         <v>33</v>
       </c>
-      <c r="D17" s="45">
+      <c r="D17" s="14">
         <f>SUM(D5:D15)</f>
         <v>44</v>
       </c>
-      <c r="E17" s="45">
+      <c r="E17" s="14">
         <f t="shared" ref="E17:Q17" si="0">SUM(E5:E15)</f>
         <v>11</v>
       </c>
-      <c r="F17" s="45">
+      <c r="F17" s="14">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="G17" s="45">
+      <c r="G17" s="14">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
@@ -4374,7 +4389,7 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="J17" s="45">
+      <c r="J17" s="14">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
@@ -4415,19 +4430,19 @@
         <f>SUM(Experiments!C2:C53)</f>
         <v>33</v>
       </c>
-      <c r="D18" s="44">
+      <c r="D18" s="8">
         <f>SUM(Experiments!D2:D53)</f>
         <v>33</v>
       </c>
-      <c r="E18" s="44">
+      <c r="E18" s="8">
         <f>SUM(Experiments!E2:E53)</f>
         <v>7</v>
       </c>
-      <c r="F18" s="44">
+      <c r="F18" s="8">
         <f>SUM(Experiments!F2:F53)</f>
         <v>10</v>
       </c>
-      <c r="G18" s="44">
+      <c r="G18" s="8">
         <f>SUM(Experiments!G2:G53)</f>
         <v>28</v>
       </c>
@@ -4439,7 +4454,7 @@
         <f>SUM(Experiments!I2:I53)</f>
         <v>7</v>
       </c>
-      <c r="J18" s="44">
+      <c r="J18" s="8">
         <f>SUM(Experiments!J2:J53)</f>
         <v>10</v>
       </c>
@@ -4480,19 +4495,19 @@
         <f>SUM(Experiments!C54:C64)</f>
         <v>0</v>
       </c>
-      <c r="D19" s="44">
+      <c r="D19" s="8">
         <f>SUM(Experiments!D54:D64)</f>
         <v>11</v>
       </c>
-      <c r="E19" s="44">
+      <c r="E19" s="8">
         <f>SUM(Experiments!E54:E64)</f>
         <v>4</v>
       </c>
-      <c r="F19" s="44">
+      <c r="F19" s="8">
         <f>SUM(Experiments!F54:F64)</f>
         <v>1</v>
       </c>
-      <c r="G19" s="44">
+      <c r="G19" s="8">
         <f>SUM(Experiments!G54:G64)</f>
         <v>10</v>
       </c>
@@ -4504,7 +4519,7 @@
         <f>SUM(Experiments!I54:I64)</f>
         <v>4</v>
       </c>
-      <c r="J19" s="44">
+      <c r="J19" s="8">
         <f>SUM(Experiments!J54:J64)</f>
         <v>1</v>
       </c>
@@ -4544,23 +4559,23 @@
       <c r="B21" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="35" t="s">
+      <c r="C21" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="D21" s="35"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="35"/>
-      <c r="G21" s="35"/>
-      <c r="H21" s="35"/>
-      <c r="I21" s="35" t="s">
+      <c r="D21" s="40"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="J21" s="35"/>
-      <c r="K21" s="35"/>
-      <c r="L21" s="35"/>
-      <c r="M21" s="35"/>
-      <c r="N21" s="35"/>
-      <c r="O21" s="35"/>
+      <c r="J21" s="40"/>
+      <c r="K21" s="40"/>
+      <c r="L21" s="40"/>
+      <c r="M21" s="40"/>
+      <c r="N21" s="40"/>
+      <c r="O21" s="40"/>
       <c r="Q21" s="1" t="s">
         <v>59</v>
       </c>
@@ -4576,116 +4591,120 @@
         <f t="array" ref="B22:B36">TRANSPOSE(_xlfn.ANCHORARRAY(C4))</f>
         <v>BHN_FWB</v>
       </c>
-      <c r="C22" s="36" t="s">
+      <c r="C22" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="D22" s="36"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="36"/>
-      <c r="I22" s="32"/>
-      <c r="J22" s="32"/>
-      <c r="K22" s="32"/>
-      <c r="L22" s="32"/>
-      <c r="M22" s="32"/>
-      <c r="N22" s="32"/>
-      <c r="O22" s="32"/>
-      <c r="Q22" s="25"/>
-      <c r="R22" s="25"/>
-      <c r="S22" s="25"/>
-      <c r="T22" s="25"/>
-      <c r="U22" s="25"/>
-      <c r="V22" s="25"/>
-      <c r="W22" s="25"/>
-      <c r="X22" s="25"/>
-      <c r="Y22" s="25"/>
-      <c r="Z22" s="25"/>
-      <c r="AA22" s="25"/>
-      <c r="AB22" s="25"/>
-      <c r="AC22" s="25"/>
-      <c r="AD22" s="25"/>
-      <c r="AE22" s="25"/>
-      <c r="AF22" s="25"/>
-      <c r="AG22" s="25"/>
-      <c r="AH22" s="25"/>
-      <c r="AI22" s="25"/>
-      <c r="AJ22" s="25"/>
-      <c r="AK22" s="25"/>
-      <c r="AL22" s="25"/>
-      <c r="AM22" s="25"/>
-      <c r="AN22" s="25"/>
-      <c r="AO22" s="25"/>
-      <c r="AP22" s="25"/>
-      <c r="AQ22" s="25"/>
-      <c r="AR22" s="25" t="e" vm="3">
+      <c r="D22" s="41"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="41"/>
+      <c r="H22" s="41"/>
+      <c r="I22" s="37"/>
+      <c r="J22" s="37"/>
+      <c r="K22" s="37"/>
+      <c r="L22" s="37"/>
+      <c r="M22" s="37"/>
+      <c r="N22" s="37"/>
+      <c r="O22" s="37"/>
+      <c r="Q22" s="30" t="e" vm="9">
         <v>#VALUE!</v>
       </c>
-      <c r="AS22" s="25"/>
-      <c r="AT22" s="25"/>
-      <c r="AU22" s="25"/>
-      <c r="AV22" s="25"/>
-      <c r="AW22" s="25"/>
-      <c r="AX22" s="25"/>
-      <c r="AY22" s="25"/>
+      <c r="R22" s="30"/>
+      <c r="S22" s="30"/>
+      <c r="T22" s="30"/>
+      <c r="U22" s="30"/>
+      <c r="V22" s="30"/>
+      <c r="W22" s="30"/>
+      <c r="X22" s="30"/>
+      <c r="Y22" s="30"/>
+      <c r="Z22" s="30"/>
+      <c r="AA22" s="30"/>
+      <c r="AB22" s="30" t="e" vm="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="AC22" s="30"/>
+      <c r="AD22" s="30"/>
+      <c r="AE22" s="30"/>
+      <c r="AF22" s="30"/>
+      <c r="AG22" s="30"/>
+      <c r="AH22" s="30"/>
+      <c r="AI22" s="30"/>
+      <c r="AJ22" s="30"/>
+      <c r="AK22" s="30"/>
+      <c r="AL22" s="30"/>
+      <c r="AM22" s="30"/>
+      <c r="AN22" s="30"/>
+      <c r="AO22" s="30"/>
+      <c r="AP22" s="30"/>
+      <c r="AQ22" s="30"/>
+      <c r="AR22" s="30" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
+      <c r="AS22" s="30"/>
+      <c r="AT22" s="30"/>
+      <c r="AU22" s="30"/>
+      <c r="AV22" s="30"/>
+      <c r="AW22" s="30"/>
+      <c r="AX22" s="30"/>
+      <c r="AY22" s="30"/>
     </row>
     <row r="23" spans="1:51" ht="87.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>1</v>
       </c>
-      <c r="B23" s="48" t="str">
+      <c r="B23" s="26" t="str">
         <v>BHN_FWB_AllExt</v>
       </c>
-      <c r="C23" s="49" t="s">
+      <c r="C23" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="D23" s="49"/>
-      <c r="E23" s="49"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="49"/>
-      <c r="H23" s="49"/>
-      <c r="I23" s="32"/>
-      <c r="J23" s="32"/>
-      <c r="K23" s="32"/>
-      <c r="L23" s="32"/>
-      <c r="M23" s="32"/>
-      <c r="N23" s="32"/>
-      <c r="O23" s="32"/>
-      <c r="Q23" s="25"/>
-      <c r="R23" s="25"/>
-      <c r="S23" s="25"/>
-      <c r="T23" s="25"/>
-      <c r="U23" s="25"/>
-      <c r="V23" s="25"/>
-      <c r="W23" s="25"/>
-      <c r="X23" s="25"/>
-      <c r="Y23" s="25"/>
-      <c r="Z23" s="25"/>
-      <c r="AA23" s="25"/>
-      <c r="AB23" s="25"/>
-      <c r="AC23" s="25"/>
-      <c r="AD23" s="25"/>
-      <c r="AE23" s="25"/>
-      <c r="AF23" s="25"/>
-      <c r="AG23" s="25"/>
-      <c r="AH23" s="25"/>
-      <c r="AI23" s="25"/>
-      <c r="AJ23" s="25"/>
-      <c r="AK23" s="25"/>
-      <c r="AL23" s="25"/>
-      <c r="AM23" s="25"/>
-      <c r="AN23" s="25"/>
-      <c r="AO23" s="25"/>
-      <c r="AP23" s="25"/>
-      <c r="AQ23" s="25"/>
-      <c r="AR23" s="25"/>
-      <c r="AS23" s="25"/>
-      <c r="AT23" s="25"/>
-      <c r="AU23" s="25"/>
-      <c r="AV23" s="25"/>
-      <c r="AW23" s="25"/>
-      <c r="AX23" s="25"/>
-      <c r="AY23" s="25"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="44"/>
+      <c r="F23" s="44"/>
+      <c r="G23" s="44"/>
+      <c r="H23" s="44"/>
+      <c r="I23" s="37"/>
+      <c r="J23" s="37"/>
+      <c r="K23" s="37"/>
+      <c r="L23" s="37"/>
+      <c r="M23" s="37"/>
+      <c r="N23" s="37"/>
+      <c r="O23" s="37"/>
+      <c r="Q23" s="30"/>
+      <c r="R23" s="30"/>
+      <c r="S23" s="30"/>
+      <c r="T23" s="30"/>
+      <c r="U23" s="30"/>
+      <c r="V23" s="30"/>
+      <c r="W23" s="30"/>
+      <c r="X23" s="30"/>
+      <c r="Y23" s="30"/>
+      <c r="Z23" s="30"/>
+      <c r="AA23" s="30"/>
+      <c r="AB23" s="30"/>
+      <c r="AC23" s="30"/>
+      <c r="AD23" s="30"/>
+      <c r="AE23" s="30"/>
+      <c r="AF23" s="30"/>
+      <c r="AG23" s="30"/>
+      <c r="AH23" s="30"/>
+      <c r="AI23" s="30"/>
+      <c r="AJ23" s="30"/>
+      <c r="AK23" s="30"/>
+      <c r="AL23" s="30"/>
+      <c r="AM23" s="30"/>
+      <c r="AN23" s="30"/>
+      <c r="AO23" s="30"/>
+      <c r="AP23" s="30"/>
+      <c r="AQ23" s="30"/>
+      <c r="AR23" s="30"/>
+      <c r="AS23" s="30"/>
+      <c r="AT23" s="30"/>
+      <c r="AU23" s="30"/>
+      <c r="AV23" s="30"/>
+      <c r="AW23" s="30"/>
+      <c r="AX23" s="30"/>
+      <c r="AY23" s="30"/>
     </row>
     <row r="24" spans="1:51" ht="108.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24">
@@ -4694,56 +4713,56 @@
       <c r="B24" s="7" t="str">
         <v>Few_indicators_closest_DLS_coverage</v>
       </c>
-      <c r="C24" s="36" t="s">
+      <c r="C24" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="D24" s="36"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="36"/>
-      <c r="H24" s="36"/>
-      <c r="I24" s="32"/>
-      <c r="J24" s="32"/>
-      <c r="K24" s="32"/>
-      <c r="L24" s="32"/>
-      <c r="M24" s="32"/>
-      <c r="N24" s="32"/>
-      <c r="O24" s="32"/>
-      <c r="Q24" s="25"/>
-      <c r="R24" s="25"/>
-      <c r="S24" s="25"/>
-      <c r="T24" s="25"/>
-      <c r="U24" s="25"/>
-      <c r="V24" s="25"/>
-      <c r="W24" s="25"/>
-      <c r="X24" s="25"/>
-      <c r="Y24" s="25"/>
-      <c r="Z24" s="25"/>
-      <c r="AA24" s="25"/>
-      <c r="AB24" s="25"/>
-      <c r="AC24" s="25"/>
-      <c r="AD24" s="25"/>
-      <c r="AE24" s="25"/>
-      <c r="AF24" s="25"/>
-      <c r="AG24" s="25"/>
-      <c r="AH24" s="25"/>
-      <c r="AI24" s="25"/>
-      <c r="AJ24" s="25"/>
-      <c r="AK24" s="25"/>
-      <c r="AL24" s="25"/>
-      <c r="AM24" s="25"/>
-      <c r="AN24" s="25"/>
-      <c r="AO24" s="25"/>
-      <c r="AP24" s="25"/>
-      <c r="AQ24" s="25"/>
-      <c r="AR24" s="25"/>
-      <c r="AS24" s="25"/>
-      <c r="AT24" s="25"/>
-      <c r="AU24" s="25"/>
-      <c r="AV24" s="25"/>
-      <c r="AW24" s="25"/>
-      <c r="AX24" s="25"/>
-      <c r="AY24" s="25"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="41"/>
+      <c r="F24" s="41"/>
+      <c r="G24" s="41"/>
+      <c r="H24" s="41"/>
+      <c r="I24" s="37"/>
+      <c r="J24" s="37"/>
+      <c r="K24" s="37"/>
+      <c r="L24" s="37"/>
+      <c r="M24" s="37"/>
+      <c r="N24" s="37"/>
+      <c r="O24" s="37"/>
+      <c r="Q24" s="30"/>
+      <c r="R24" s="30"/>
+      <c r="S24" s="30"/>
+      <c r="T24" s="30"/>
+      <c r="U24" s="30"/>
+      <c r="V24" s="30"/>
+      <c r="W24" s="30"/>
+      <c r="X24" s="30"/>
+      <c r="Y24" s="30"/>
+      <c r="Z24" s="30"/>
+      <c r="AA24" s="30"/>
+      <c r="AB24" s="30"/>
+      <c r="AC24" s="30"/>
+      <c r="AD24" s="30"/>
+      <c r="AE24" s="30"/>
+      <c r="AF24" s="30"/>
+      <c r="AG24" s="30"/>
+      <c r="AH24" s="30"/>
+      <c r="AI24" s="30"/>
+      <c r="AJ24" s="30"/>
+      <c r="AK24" s="30"/>
+      <c r="AL24" s="30"/>
+      <c r="AM24" s="30"/>
+      <c r="AN24" s="30"/>
+      <c r="AO24" s="30"/>
+      <c r="AP24" s="30"/>
+      <c r="AQ24" s="30"/>
+      <c r="AR24" s="30"/>
+      <c r="AS24" s="30"/>
+      <c r="AT24" s="30"/>
+      <c r="AU24" s="30"/>
+      <c r="AV24" s="30"/>
+      <c r="AW24" s="30"/>
+      <c r="AX24" s="30"/>
+      <c r="AY24" s="30"/>
     </row>
     <row r="25" spans="1:51" ht="81.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25">
@@ -4752,48 +4771,48 @@
       <c r="B25" s="7" t="str">
         <v>Few indicators_SPI_preferred</v>
       </c>
-      <c r="C25" s="36" t="s">
+      <c r="C25" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="D25" s="36"/>
-      <c r="E25" s="36"/>
-      <c r="F25" s="36"/>
-      <c r="G25" s="36"/>
-      <c r="H25" s="36"/>
-      <c r="I25" s="32"/>
-      <c r="J25" s="32"/>
-      <c r="K25" s="32"/>
-      <c r="L25" s="32"/>
-      <c r="M25" s="32"/>
-      <c r="N25" s="32"/>
-      <c r="O25" s="32"/>
-      <c r="Q25" s="25"/>
-      <c r="R25" s="25"/>
-      <c r="S25" s="25"/>
-      <c r="T25" s="25"/>
-      <c r="U25" s="25"/>
-      <c r="V25" s="25"/>
-      <c r="W25" s="25"/>
-      <c r="X25" s="25"/>
-      <c r="Y25" s="25"/>
-      <c r="Z25" s="25"/>
-      <c r="AA25" s="25"/>
-      <c r="AB25" s="25"/>
-      <c r="AC25" s="25"/>
-      <c r="AD25" s="25"/>
-      <c r="AE25" s="25"/>
-      <c r="AF25" s="25"/>
-      <c r="AG25" s="25"/>
-      <c r="AH25" s="25"/>
-      <c r="AI25" s="25"/>
-      <c r="AJ25" s="25"/>
-      <c r="AK25" s="25"/>
-      <c r="AL25" s="25"/>
-      <c r="AM25" s="25"/>
-      <c r="AN25" s="25"/>
-      <c r="AO25" s="25"/>
-      <c r="AP25" s="25"/>
-      <c r="AQ25" s="25"/>
+      <c r="D25" s="41"/>
+      <c r="E25" s="41"/>
+      <c r="F25" s="41"/>
+      <c r="G25" s="41"/>
+      <c r="H25" s="41"/>
+      <c r="I25" s="37"/>
+      <c r="J25" s="37"/>
+      <c r="K25" s="37"/>
+      <c r="L25" s="37"/>
+      <c r="M25" s="37"/>
+      <c r="N25" s="37"/>
+      <c r="O25" s="37"/>
+      <c r="Q25" s="49"/>
+      <c r="R25" s="49"/>
+      <c r="S25" s="49"/>
+      <c r="T25" s="49"/>
+      <c r="U25" s="49"/>
+      <c r="V25" s="49"/>
+      <c r="W25" s="49"/>
+      <c r="X25" s="49"/>
+      <c r="Y25" s="49"/>
+      <c r="Z25" s="49"/>
+      <c r="AA25" s="49"/>
+      <c r="AB25" s="30"/>
+      <c r="AC25" s="30"/>
+      <c r="AD25" s="30"/>
+      <c r="AE25" s="30"/>
+      <c r="AF25" s="30"/>
+      <c r="AG25" s="30"/>
+      <c r="AH25" s="30"/>
+      <c r="AI25" s="30"/>
+      <c r="AJ25" s="30"/>
+      <c r="AK25" s="30"/>
+      <c r="AL25" s="30"/>
+      <c r="AM25" s="30"/>
+      <c r="AN25" s="30"/>
+      <c r="AO25" s="30"/>
+      <c r="AP25" s="30"/>
+      <c r="AQ25" s="30"/>
     </row>
     <row r="26" spans="1:51" ht="69.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26">
@@ -4802,98 +4821,98 @@
       <c r="B26" s="7" t="str">
         <v>No_non_DLS</v>
       </c>
-      <c r="C26" s="38" t="s">
+      <c r="C26" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="D26" s="38"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="38"/>
-      <c r="G26" s="38"/>
-      <c r="H26" s="38"/>
-      <c r="I26" s="32"/>
-      <c r="J26" s="32"/>
-      <c r="K26" s="32"/>
-      <c r="L26" s="32"/>
-      <c r="M26" s="32"/>
-      <c r="N26" s="32"/>
-      <c r="O26" s="32"/>
-      <c r="Q26" s="25"/>
-      <c r="R26" s="25"/>
-      <c r="S26" s="25"/>
-      <c r="T26" s="25"/>
-      <c r="U26" s="25"/>
-      <c r="V26" s="25"/>
-      <c r="W26" s="25"/>
-      <c r="X26" s="25"/>
-      <c r="Y26" s="25"/>
-      <c r="Z26" s="25"/>
-      <c r="AA26" s="25"/>
-      <c r="AB26" s="25"/>
-      <c r="AC26" s="25"/>
-      <c r="AD26" s="25"/>
-      <c r="AE26" s="25"/>
-      <c r="AF26" s="25"/>
-      <c r="AG26" s="25"/>
-      <c r="AH26" s="25"/>
-      <c r="AI26" s="25"/>
-      <c r="AJ26" s="25"/>
-      <c r="AK26" s="25"/>
-      <c r="AL26" s="25"/>
-      <c r="AM26" s="25"/>
-      <c r="AN26" s="25"/>
-      <c r="AO26" s="25"/>
-      <c r="AP26" s="25"/>
-      <c r="AQ26" s="25"/>
+      <c r="D26" s="43"/>
+      <c r="E26" s="43"/>
+      <c r="F26" s="43"/>
+      <c r="G26" s="43"/>
+      <c r="H26" s="43"/>
+      <c r="I26" s="37"/>
+      <c r="J26" s="37"/>
+      <c r="K26" s="37"/>
+      <c r="L26" s="37"/>
+      <c r="M26" s="37"/>
+      <c r="N26" s="37"/>
+      <c r="O26" s="37"/>
+      <c r="Q26" s="30"/>
+      <c r="R26" s="30"/>
+      <c r="S26" s="30"/>
+      <c r="T26" s="30"/>
+      <c r="U26" s="30"/>
+      <c r="V26" s="30"/>
+      <c r="W26" s="30"/>
+      <c r="X26" s="30"/>
+      <c r="Y26" s="30"/>
+      <c r="Z26" s="30"/>
+      <c r="AA26" s="30"/>
+      <c r="AB26" s="30"/>
+      <c r="AC26" s="30"/>
+      <c r="AD26" s="30"/>
+      <c r="AE26" s="30"/>
+      <c r="AF26" s="30"/>
+      <c r="AG26" s="30"/>
+      <c r="AH26" s="30"/>
+      <c r="AI26" s="30"/>
+      <c r="AJ26" s="30"/>
+      <c r="AK26" s="30"/>
+      <c r="AL26" s="30"/>
+      <c r="AM26" s="30"/>
+      <c r="AN26" s="30"/>
+      <c r="AO26" s="30"/>
+      <c r="AP26" s="30"/>
+      <c r="AQ26" s="30"/>
     </row>
     <row r="27" spans="1:51" ht="93" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>1</v>
       </c>
-      <c r="B27" s="48" t="str">
+      <c r="B27" s="26" t="str">
         <v>Only_%_of_pop</v>
       </c>
-      <c r="C27" s="50" t="s">
+      <c r="C27" s="45" t="s">
         <v>51</v>
       </c>
-      <c r="D27" s="50"/>
-      <c r="E27" s="50"/>
-      <c r="F27" s="50"/>
-      <c r="G27" s="50"/>
-      <c r="H27" s="50"/>
-      <c r="I27" s="32"/>
-      <c r="J27" s="32"/>
-      <c r="K27" s="32"/>
-      <c r="L27" s="32"/>
-      <c r="M27" s="32"/>
-      <c r="N27" s="32"/>
-      <c r="O27" s="32"/>
-      <c r="Q27" s="25"/>
-      <c r="R27" s="25"/>
-      <c r="S27" s="25"/>
-      <c r="T27" s="25"/>
-      <c r="U27" s="25"/>
-      <c r="V27" s="25"/>
-      <c r="W27" s="25"/>
-      <c r="X27" s="25"/>
-      <c r="Y27" s="25"/>
-      <c r="Z27" s="25"/>
-      <c r="AA27" s="25"/>
-      <c r="AB27" s="25"/>
-      <c r="AC27" s="25"/>
-      <c r="AD27" s="25"/>
-      <c r="AE27" s="25"/>
-      <c r="AF27" s="25"/>
-      <c r="AG27" s="25"/>
-      <c r="AH27" s="25"/>
-      <c r="AI27" s="25"/>
-      <c r="AJ27" s="25"/>
-      <c r="AK27" s="25"/>
-      <c r="AL27" s="25"/>
-      <c r="AM27" s="25"/>
-      <c r="AN27" s="25"/>
-      <c r="AO27" s="25"/>
-      <c r="AP27" s="25"/>
-      <c r="AQ27" s="25"/>
+      <c r="D27" s="45"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="45"/>
+      <c r="G27" s="45"/>
+      <c r="H27" s="45"/>
+      <c r="I27" s="37"/>
+      <c r="J27" s="37"/>
+      <c r="K27" s="37"/>
+      <c r="L27" s="37"/>
+      <c r="M27" s="37"/>
+      <c r="N27" s="37"/>
+      <c r="O27" s="37"/>
+      <c r="Q27" s="30"/>
+      <c r="R27" s="30"/>
+      <c r="S27" s="30"/>
+      <c r="T27" s="30"/>
+      <c r="U27" s="30"/>
+      <c r="V27" s="30"/>
+      <c r="W27" s="30"/>
+      <c r="X27" s="30"/>
+      <c r="Y27" s="30"/>
+      <c r="Z27" s="30"/>
+      <c r="AA27" s="30"/>
+      <c r="AB27" s="30"/>
+      <c r="AC27" s="30"/>
+      <c r="AD27" s="30"/>
+      <c r="AE27" s="30"/>
+      <c r="AF27" s="30"/>
+      <c r="AG27" s="30"/>
+      <c r="AH27" s="30"/>
+      <c r="AI27" s="30"/>
+      <c r="AJ27" s="30"/>
+      <c r="AK27" s="30"/>
+      <c r="AL27" s="30"/>
+      <c r="AM27" s="30"/>
+      <c r="AN27" s="30"/>
+      <c r="AO27" s="30"/>
+      <c r="AP27" s="30"/>
+      <c r="AQ27" s="30"/>
     </row>
     <row r="28" spans="1:51" ht="65.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28">
@@ -4902,48 +4921,48 @@
       <c r="B28" s="17" t="str">
         <v>Few_indicators_closest_DLS_coverage_90</v>
       </c>
-      <c r="C28" s="28" t="s">
+      <c r="C28" s="33" t="s">
         <v>62</v>
       </c>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="28"/>
-      <c r="I28" s="30"/>
-      <c r="J28" s="30"/>
-      <c r="K28" s="30"/>
-      <c r="L28" s="30"/>
-      <c r="M28" s="30"/>
-      <c r="N28" s="30"/>
-      <c r="O28" s="30"/>
-      <c r="Q28" s="25"/>
-      <c r="R28" s="25"/>
-      <c r="S28" s="25"/>
-      <c r="T28" s="25"/>
-      <c r="U28" s="25"/>
-      <c r="V28" s="25"/>
-      <c r="W28" s="25"/>
-      <c r="X28" s="25"/>
-      <c r="Y28" s="25"/>
-      <c r="Z28" s="25"/>
-      <c r="AA28" s="25"/>
-      <c r="AB28" s="25"/>
-      <c r="AC28" s="25"/>
-      <c r="AD28" s="25"/>
-      <c r="AE28" s="25"/>
-      <c r="AF28" s="25"/>
-      <c r="AG28" s="25"/>
-      <c r="AH28" s="25"/>
-      <c r="AI28" s="25"/>
-      <c r="AJ28" s="25"/>
-      <c r="AK28" s="25"/>
-      <c r="AL28" s="25"/>
-      <c r="AM28" s="25"/>
-      <c r="AN28" s="25"/>
-      <c r="AO28" s="25"/>
-      <c r="AP28" s="25"/>
-      <c r="AQ28" s="25"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="35"/>
+      <c r="J28" s="35"/>
+      <c r="K28" s="35"/>
+      <c r="L28" s="35"/>
+      <c r="M28" s="35"/>
+      <c r="N28" s="35"/>
+      <c r="O28" s="35"/>
+      <c r="Q28" s="30"/>
+      <c r="R28" s="30"/>
+      <c r="S28" s="30"/>
+      <c r="T28" s="30"/>
+      <c r="U28" s="30"/>
+      <c r="V28" s="30"/>
+      <c r="W28" s="30"/>
+      <c r="X28" s="30"/>
+      <c r="Y28" s="30"/>
+      <c r="Z28" s="30"/>
+      <c r="AA28" s="30"/>
+      <c r="AB28" s="30"/>
+      <c r="AC28" s="30"/>
+      <c r="AD28" s="30"/>
+      <c r="AE28" s="30"/>
+      <c r="AF28" s="30"/>
+      <c r="AG28" s="30"/>
+      <c r="AH28" s="30"/>
+      <c r="AI28" s="30"/>
+      <c r="AJ28" s="30"/>
+      <c r="AK28" s="30"/>
+      <c r="AL28" s="30"/>
+      <c r="AM28" s="30"/>
+      <c r="AN28" s="30"/>
+      <c r="AO28" s="30"/>
+      <c r="AP28" s="30"/>
+      <c r="AQ28" s="30"/>
     </row>
     <row r="29" spans="1:51" ht="67.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29">
@@ -4952,48 +4971,48 @@
       <c r="B29" s="17" t="str">
         <v>Few indicators_SPI_preferred_90</v>
       </c>
-      <c r="C29" s="28" t="s">
+      <c r="C29" s="33" t="s">
         <v>62</v>
       </c>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="28"/>
-      <c r="I29" s="30"/>
-      <c r="J29" s="30"/>
-      <c r="K29" s="30"/>
-      <c r="L29" s="30"/>
-      <c r="M29" s="30"/>
-      <c r="N29" s="30"/>
-      <c r="O29" s="30"/>
-      <c r="Q29" s="25"/>
-      <c r="R29" s="25"/>
-      <c r="S29" s="25"/>
-      <c r="T29" s="25"/>
-      <c r="U29" s="25"/>
-      <c r="V29" s="25"/>
-      <c r="W29" s="25"/>
-      <c r="X29" s="25"/>
-      <c r="Y29" s="25"/>
-      <c r="Z29" s="25"/>
-      <c r="AA29" s="25"/>
-      <c r="AB29" s="25"/>
-      <c r="AC29" s="25"/>
-      <c r="AD29" s="25"/>
-      <c r="AE29" s="25"/>
-      <c r="AF29" s="25"/>
-      <c r="AG29" s="25"/>
-      <c r="AH29" s="25"/>
-      <c r="AI29" s="25"/>
-      <c r="AJ29" s="25"/>
-      <c r="AK29" s="25"/>
-      <c r="AL29" s="25"/>
-      <c r="AM29" s="25"/>
-      <c r="AN29" s="25"/>
-      <c r="AO29" s="25"/>
-      <c r="AP29" s="25"/>
-      <c r="AQ29" s="25"/>
+      <c r="D29" s="33"/>
+      <c r="E29" s="33"/>
+      <c r="F29" s="33"/>
+      <c r="G29" s="33"/>
+      <c r="H29" s="33"/>
+      <c r="I29" s="35"/>
+      <c r="J29" s="35"/>
+      <c r="K29" s="35"/>
+      <c r="L29" s="35"/>
+      <c r="M29" s="35"/>
+      <c r="N29" s="35"/>
+      <c r="O29" s="35"/>
+      <c r="Q29" s="30"/>
+      <c r="R29" s="30"/>
+      <c r="S29" s="30"/>
+      <c r="T29" s="30"/>
+      <c r="U29" s="30"/>
+      <c r="V29" s="30"/>
+      <c r="W29" s="30"/>
+      <c r="X29" s="30"/>
+      <c r="Y29" s="30"/>
+      <c r="Z29" s="30"/>
+      <c r="AA29" s="30"/>
+      <c r="AB29" s="30"/>
+      <c r="AC29" s="30"/>
+      <c r="AD29" s="30"/>
+      <c r="AE29" s="30"/>
+      <c r="AF29" s="30"/>
+      <c r="AG29" s="30"/>
+      <c r="AH29" s="30"/>
+      <c r="AI29" s="30"/>
+      <c r="AJ29" s="30"/>
+      <c r="AK29" s="30"/>
+      <c r="AL29" s="30"/>
+      <c r="AM29" s="30"/>
+      <c r="AN29" s="30"/>
+      <c r="AO29" s="30"/>
+      <c r="AP29" s="30"/>
+      <c r="AQ29" s="30"/>
     </row>
     <row r="30" spans="1:51" ht="55.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30">
@@ -5002,650 +5021,652 @@
       <c r="B30" s="17" t="str">
         <v>Few_indicators_closeDLS_subPrimSchool</v>
       </c>
-      <c r="C30" s="26" t="s">
+      <c r="C30" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="30"/>
-      <c r="J30" s="30"/>
-      <c r="K30" s="30"/>
-      <c r="L30" s="30"/>
-      <c r="M30" s="30"/>
-      <c r="N30" s="30"/>
-      <c r="O30" s="30"/>
-      <c r="Q30" s="25"/>
-      <c r="R30" s="25"/>
-      <c r="S30" s="25"/>
-      <c r="T30" s="25"/>
-      <c r="U30" s="25"/>
-      <c r="V30" s="25"/>
-      <c r="W30" s="25"/>
-      <c r="X30" s="25"/>
-      <c r="Y30" s="25"/>
-      <c r="Z30" s="25"/>
-      <c r="AA30" s="25"/>
-      <c r="AB30" s="25"/>
-      <c r="AC30" s="25"/>
-      <c r="AD30" s="25"/>
-      <c r="AE30" s="25"/>
-      <c r="AF30" s="25"/>
-      <c r="AG30" s="25"/>
-      <c r="AH30" s="25"/>
-      <c r="AI30" s="25"/>
-      <c r="AJ30" s="25"/>
-      <c r="AK30" s="25"/>
-      <c r="AL30" s="25"/>
-      <c r="AM30" s="25"/>
-      <c r="AN30" s="25"/>
-      <c r="AO30" s="25"/>
-      <c r="AP30" s="25"/>
-      <c r="AQ30" s="25"/>
+      <c r="D30" s="31"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="31"/>
+      <c r="G30" s="31"/>
+      <c r="H30" s="31"/>
+      <c r="I30" s="35"/>
+      <c r="J30" s="35"/>
+      <c r="K30" s="35"/>
+      <c r="L30" s="35"/>
+      <c r="M30" s="35"/>
+      <c r="N30" s="35"/>
+      <c r="O30" s="35"/>
+      <c r="Q30" s="30"/>
+      <c r="R30" s="30"/>
+      <c r="S30" s="30"/>
+      <c r="T30" s="30"/>
+      <c r="U30" s="30"/>
+      <c r="V30" s="30"/>
+      <c r="W30" s="30"/>
+      <c r="X30" s="30"/>
+      <c r="Y30" s="30"/>
+      <c r="Z30" s="30"/>
+      <c r="AA30" s="30"/>
+      <c r="AB30" s="30"/>
+      <c r="AC30" s="30"/>
+      <c r="AD30" s="30"/>
+      <c r="AE30" s="30"/>
+      <c r="AF30" s="30"/>
+      <c r="AG30" s="30"/>
+      <c r="AH30" s="30"/>
+      <c r="AI30" s="30"/>
+      <c r="AJ30" s="30"/>
+      <c r="AK30" s="30"/>
+      <c r="AL30" s="30"/>
+      <c r="AM30" s="30"/>
+      <c r="AN30" s="30"/>
+      <c r="AO30" s="30"/>
+      <c r="AP30" s="30"/>
+      <c r="AQ30" s="30"/>
     </row>
     <row r="31" spans="1:51" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>3</v>
       </c>
-      <c r="B31" s="51" t="str">
+      <c r="B31" s="27" t="str">
         <v>No_non_DLS_90</v>
       </c>
-      <c r="C31" s="52" t="s">
+      <c r="C31" s="46" t="s">
         <v>62</v>
       </c>
-      <c r="D31" s="52"/>
-      <c r="E31" s="52"/>
-      <c r="F31" s="52"/>
-      <c r="G31" s="52"/>
-      <c r="H31" s="52"/>
-      <c r="I31" s="52" t="s">
+      <c r="D31" s="46"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="46"/>
+      <c r="G31" s="46"/>
+      <c r="H31" s="46"/>
+      <c r="I31" s="46" t="s">
         <v>76</v>
       </c>
-      <c r="J31" s="52"/>
-      <c r="K31" s="52"/>
-      <c r="L31" s="52"/>
-      <c r="M31" s="52"/>
-      <c r="N31" s="52"/>
-      <c r="O31" s="52"/>
-      <c r="Q31" s="25"/>
-      <c r="R31" s="25"/>
-      <c r="S31" s="25"/>
-      <c r="T31" s="25"/>
-      <c r="U31" s="25"/>
-      <c r="V31" s="25"/>
-      <c r="W31" s="25"/>
-      <c r="X31" s="25"/>
-      <c r="Y31" s="25"/>
-      <c r="Z31" s="25"/>
-      <c r="AA31" s="25"/>
-      <c r="AB31" s="25"/>
-      <c r="AC31" s="25"/>
-      <c r="AD31" s="25"/>
-      <c r="AE31" s="25"/>
-      <c r="AF31" s="25"/>
-      <c r="AG31" s="25"/>
-      <c r="AH31" s="25"/>
-      <c r="AI31" s="25"/>
-      <c r="AJ31" s="25"/>
-      <c r="AK31" s="25"/>
-      <c r="AL31" s="25"/>
-      <c r="AM31" s="25"/>
-      <c r="AN31" s="25"/>
-      <c r="AO31" s="25"/>
-      <c r="AP31" s="25"/>
-      <c r="AQ31" s="25"/>
+      <c r="J31" s="46"/>
+      <c r="K31" s="46"/>
+      <c r="L31" s="46"/>
+      <c r="M31" s="46"/>
+      <c r="N31" s="46"/>
+      <c r="O31" s="46"/>
+      <c r="Q31" s="30"/>
+      <c r="R31" s="30"/>
+      <c r="S31" s="30"/>
+      <c r="T31" s="30"/>
+      <c r="U31" s="30"/>
+      <c r="V31" s="30"/>
+      <c r="W31" s="30"/>
+      <c r="X31" s="30"/>
+      <c r="Y31" s="30"/>
+      <c r="Z31" s="30"/>
+      <c r="AA31" s="30"/>
+      <c r="AB31" s="30"/>
+      <c r="AC31" s="30"/>
+      <c r="AD31" s="30"/>
+      <c r="AE31" s="30"/>
+      <c r="AF31" s="30"/>
+      <c r="AG31" s="30"/>
+      <c r="AH31" s="30"/>
+      <c r="AI31" s="30"/>
+      <c r="AJ31" s="30"/>
+      <c r="AK31" s="30"/>
+      <c r="AL31" s="30"/>
+      <c r="AM31" s="30"/>
+      <c r="AN31" s="30"/>
+      <c r="AO31" s="30"/>
+      <c r="AP31" s="30"/>
+      <c r="AQ31" s="30"/>
     </row>
     <row r="32" spans="1:51" ht="103.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>3</v>
       </c>
-      <c r="B32" s="51" t="str">
+      <c r="B32" s="27" t="str">
         <v>Few_Indicators_subWatSani</v>
       </c>
-      <c r="C32" s="52" t="s">
+      <c r="C32" s="46" t="s">
         <v>67</v>
       </c>
-      <c r="D32" s="52"/>
-      <c r="E32" s="52"/>
-      <c r="F32" s="52"/>
-      <c r="G32" s="52"/>
-      <c r="H32" s="52"/>
-      <c r="I32" s="30"/>
-      <c r="J32" s="30"/>
-      <c r="K32" s="30"/>
-      <c r="L32" s="30"/>
-      <c r="M32" s="30"/>
-      <c r="N32" s="30"/>
-      <c r="O32" s="30"/>
-      <c r="Q32" s="25"/>
-      <c r="R32" s="25"/>
-      <c r="S32" s="25"/>
-      <c r="T32" s="25"/>
-      <c r="U32" s="25"/>
-      <c r="V32" s="25"/>
-      <c r="W32" s="25"/>
-      <c r="X32" s="25"/>
-      <c r="Y32" s="25"/>
-      <c r="Z32" s="25"/>
-      <c r="AA32" s="25"/>
-      <c r="AB32" s="25"/>
-      <c r="AC32" s="25"/>
-      <c r="AD32" s="25"/>
-      <c r="AE32" s="25"/>
-      <c r="AF32" s="25"/>
-      <c r="AG32" s="25"/>
-      <c r="AH32" s="25"/>
-      <c r="AI32" s="25"/>
-      <c r="AJ32" s="25"/>
-      <c r="AK32" s="25"/>
-      <c r="AL32" s="25"/>
-      <c r="AM32" s="25"/>
-      <c r="AN32" s="25"/>
-      <c r="AO32" s="25"/>
-      <c r="AP32" s="25"/>
-      <c r="AQ32" s="25"/>
+      <c r="D32" s="46"/>
+      <c r="E32" s="46"/>
+      <c r="F32" s="46"/>
+      <c r="G32" s="46"/>
+      <c r="H32" s="46"/>
+      <c r="I32" s="35"/>
+      <c r="J32" s="35"/>
+      <c r="K32" s="35"/>
+      <c r="L32" s="35"/>
+      <c r="M32" s="35"/>
+      <c r="N32" s="35"/>
+      <c r="O32" s="35"/>
+      <c r="Q32" s="30"/>
+      <c r="R32" s="30"/>
+      <c r="S32" s="30"/>
+      <c r="T32" s="30"/>
+      <c r="U32" s="30"/>
+      <c r="V32" s="30"/>
+      <c r="W32" s="30"/>
+      <c r="X32" s="30"/>
+      <c r="Y32" s="30"/>
+      <c r="Z32" s="30"/>
+      <c r="AA32" s="30"/>
+      <c r="AB32" s="30"/>
+      <c r="AC32" s="30"/>
+      <c r="AD32" s="30"/>
+      <c r="AE32" s="30"/>
+      <c r="AF32" s="30"/>
+      <c r="AG32" s="30"/>
+      <c r="AH32" s="30"/>
+      <c r="AI32" s="30"/>
+      <c r="AJ32" s="30"/>
+      <c r="AK32" s="30"/>
+      <c r="AL32" s="30"/>
+      <c r="AM32" s="30"/>
+      <c r="AN32" s="30"/>
+      <c r="AO32" s="30"/>
+      <c r="AP32" s="30"/>
+      <c r="AQ32" s="30"/>
     </row>
     <row r="33" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>4</v>
       </c>
-      <c r="B33" s="53" t="str">
+      <c r="B33" s="28" t="str">
         <v>Only_OPP</v>
       </c>
-      <c r="C33" s="54" t="s">
+      <c r="C33" s="47" t="s">
         <v>70</v>
       </c>
-      <c r="D33" s="54"/>
-      <c r="E33" s="54"/>
-      <c r="F33" s="54"/>
-      <c r="G33" s="54"/>
-      <c r="H33" s="54"/>
-      <c r="I33" s="27"/>
-      <c r="J33" s="27"/>
-      <c r="K33" s="27"/>
-      <c r="L33" s="27"/>
-      <c r="M33" s="27"/>
-      <c r="N33" s="27"/>
-      <c r="O33" s="27"/>
-      <c r="Q33" s="25"/>
-      <c r="R33" s="25"/>
-      <c r="S33" s="25"/>
-      <c r="T33" s="25"/>
-      <c r="U33" s="25"/>
-      <c r="V33" s="25"/>
-      <c r="W33" s="25"/>
-      <c r="X33" s="25"/>
-      <c r="Y33" s="25"/>
-      <c r="Z33" s="25"/>
-      <c r="AA33" s="25"/>
-      <c r="AB33" s="25"/>
-      <c r="AC33" s="25"/>
-      <c r="AD33" s="25"/>
-      <c r="AE33" s="25"/>
-      <c r="AF33" s="25"/>
-      <c r="AG33" s="25"/>
-      <c r="AH33" s="25"/>
-      <c r="AI33" s="25"/>
-      <c r="AJ33" s="25"/>
-      <c r="AK33" s="25"/>
-      <c r="AL33" s="25"/>
-      <c r="AM33" s="25"/>
-      <c r="AN33" s="25"/>
-      <c r="AO33" s="25"/>
-      <c r="AP33" s="25"/>
-      <c r="AQ33" s="25"/>
+      <c r="D33" s="47"/>
+      <c r="E33" s="47"/>
+      <c r="F33" s="47"/>
+      <c r="G33" s="47"/>
+      <c r="H33" s="47"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="32"/>
+      <c r="K33" s="32"/>
+      <c r="L33" s="32"/>
+      <c r="M33" s="32"/>
+      <c r="N33" s="32"/>
+      <c r="O33" s="32"/>
+      <c r="Q33" s="30"/>
+      <c r="R33" s="30"/>
+      <c r="S33" s="30"/>
+      <c r="T33" s="30"/>
+      <c r="U33" s="30"/>
+      <c r="V33" s="30"/>
+      <c r="W33" s="30"/>
+      <c r="X33" s="30"/>
+      <c r="Y33" s="30"/>
+      <c r="Z33" s="30"/>
+      <c r="AA33" s="30"/>
+      <c r="AB33" s="30"/>
+      <c r="AC33" s="30"/>
+      <c r="AD33" s="30"/>
+      <c r="AE33" s="30"/>
+      <c r="AF33" s="30"/>
+      <c r="AG33" s="30"/>
+      <c r="AH33" s="30"/>
+      <c r="AI33" s="30"/>
+      <c r="AJ33" s="30"/>
+      <c r="AK33" s="30"/>
+      <c r="AL33" s="30"/>
+      <c r="AM33" s="30"/>
+      <c r="AN33" s="30"/>
+      <c r="AO33" s="30"/>
+      <c r="AP33" s="30"/>
+      <c r="AQ33" s="30"/>
     </row>
     <row r="34" spans="1:43" x14ac:dyDescent="0.3">
       <c r="B34" s="6" t="str">
         <v>Baseline</v>
       </c>
-      <c r="C34" s="27"/>
-      <c r="D34" s="27"/>
-      <c r="E34" s="27"/>
-      <c r="F34" s="27"/>
-      <c r="G34" s="27"/>
-      <c r="H34" s="27"/>
-      <c r="I34" s="27"/>
-      <c r="J34" s="27"/>
-      <c r="K34" s="27"/>
-      <c r="L34" s="27"/>
-      <c r="M34" s="27"/>
-      <c r="N34" s="27"/>
-      <c r="O34" s="27"/>
-      <c r="Q34" s="25"/>
-      <c r="R34" s="25"/>
-      <c r="S34" s="25"/>
-      <c r="T34" s="25"/>
-      <c r="U34" s="25"/>
-      <c r="V34" s="25"/>
-      <c r="W34" s="25"/>
-      <c r="X34" s="25"/>
-      <c r="Y34" s="25"/>
-      <c r="Z34" s="25"/>
-      <c r="AA34" s="25"/>
-      <c r="AB34" s="25"/>
-      <c r="AC34" s="25"/>
-      <c r="AD34" s="25"/>
-      <c r="AE34" s="25"/>
-      <c r="AF34" s="25"/>
-      <c r="AG34" s="25"/>
-      <c r="AH34" s="25"/>
-      <c r="AI34" s="25"/>
-      <c r="AJ34" s="25"/>
-      <c r="AK34" s="25"/>
-      <c r="AL34" s="25"/>
-      <c r="AM34" s="25"/>
-      <c r="AN34" s="25"/>
-      <c r="AO34" s="25"/>
-      <c r="AP34" s="25"/>
-      <c r="AQ34" s="25"/>
+      <c r="C34" s="32"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="32"/>
+      <c r="K34" s="32"/>
+      <c r="L34" s="32"/>
+      <c r="M34" s="32"/>
+      <c r="N34" s="32"/>
+      <c r="O34" s="32"/>
+      <c r="Q34" s="30"/>
+      <c r="R34" s="30"/>
+      <c r="S34" s="30"/>
+      <c r="T34" s="30"/>
+      <c r="U34" s="30"/>
+      <c r="V34" s="30"/>
+      <c r="W34" s="30"/>
+      <c r="X34" s="30"/>
+      <c r="Y34" s="30"/>
+      <c r="Z34" s="30"/>
+      <c r="AA34" s="30"/>
+      <c r="AB34" s="30"/>
+      <c r="AC34" s="30"/>
+      <c r="AD34" s="30"/>
+      <c r="AE34" s="30"/>
+      <c r="AF34" s="30"/>
+      <c r="AG34" s="30"/>
+      <c r="AH34" s="30"/>
+      <c r="AI34" s="30"/>
+      <c r="AJ34" s="30"/>
+      <c r="AK34" s="30"/>
+      <c r="AL34" s="30"/>
+      <c r="AM34" s="30"/>
+      <c r="AN34" s="30"/>
+      <c r="AO34" s="30"/>
+      <c r="AP34" s="30"/>
+      <c r="AQ34" s="30"/>
     </row>
     <row r="35" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="B35" s="53" t="str">
+      <c r="B35" s="28" t="str">
         <v>No_nonDLS_limExt</v>
       </c>
-      <c r="C35" s="55"/>
-      <c r="D35" s="55"/>
-      <c r="E35" s="55"/>
-      <c r="F35" s="55"/>
-      <c r="G35" s="55"/>
-      <c r="H35" s="55"/>
-      <c r="I35" s="55" t="s">
+      <c r="C35" s="48"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="48"/>
+      <c r="F35" s="48"/>
+      <c r="G35" s="48"/>
+      <c r="H35" s="48"/>
+      <c r="I35" s="48" t="s">
         <v>73</v>
       </c>
-      <c r="J35" s="55"/>
-      <c r="K35" s="55"/>
-      <c r="L35" s="55"/>
-      <c r="M35" s="55"/>
-      <c r="N35" s="55"/>
-      <c r="O35" s="55"/>
-      <c r="Q35" s="25"/>
-      <c r="R35" s="25"/>
-      <c r="S35" s="25"/>
-      <c r="T35" s="25"/>
-      <c r="U35" s="25"/>
-      <c r="V35" s="25"/>
-      <c r="W35" s="25"/>
-      <c r="X35" s="25"/>
-      <c r="Y35" s="25"/>
-      <c r="Z35" s="25"/>
-      <c r="AA35" s="25"/>
-      <c r="AB35" s="25"/>
-      <c r="AC35" s="25"/>
-      <c r="AD35" s="25"/>
-      <c r="AE35" s="25"/>
-      <c r="AF35" s="25"/>
-      <c r="AG35" s="25"/>
-      <c r="AH35" s="25"/>
-      <c r="AI35" s="25"/>
-      <c r="AJ35" s="25"/>
-      <c r="AK35" s="25"/>
-      <c r="AL35" s="25"/>
-      <c r="AM35" s="25"/>
-      <c r="AN35" s="25"/>
-      <c r="AO35" s="25"/>
-      <c r="AP35" s="25"/>
-      <c r="AQ35" s="25"/>
+      <c r="J35" s="48"/>
+      <c r="K35" s="48"/>
+      <c r="L35" s="48"/>
+      <c r="M35" s="48"/>
+      <c r="N35" s="48"/>
+      <c r="O35" s="48"/>
+      <c r="Q35" s="30"/>
+      <c r="R35" s="30"/>
+      <c r="S35" s="30"/>
+      <c r="T35" s="30"/>
+      <c r="U35" s="30"/>
+      <c r="V35" s="30"/>
+      <c r="W35" s="30"/>
+      <c r="X35" s="30"/>
+      <c r="Y35" s="30"/>
+      <c r="Z35" s="30"/>
+      <c r="AA35" s="30"/>
+      <c r="AB35" s="30"/>
+      <c r="AC35" s="30"/>
+      <c r="AD35" s="30"/>
+      <c r="AE35" s="30"/>
+      <c r="AF35" s="30"/>
+      <c r="AG35" s="30"/>
+      <c r="AH35" s="30"/>
+      <c r="AI35" s="30"/>
+      <c r="AJ35" s="30"/>
+      <c r="AK35" s="30"/>
+      <c r="AL35" s="30"/>
+      <c r="AM35" s="30"/>
+      <c r="AN35" s="30"/>
+      <c r="AO35" s="30"/>
+      <c r="AP35" s="30"/>
+      <c r="AQ35" s="30"/>
     </row>
     <row r="36" spans="1:43" ht="76.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="6" t="str">
         <v>BHN</v>
       </c>
-      <c r="C36" s="31" t="s">
+      <c r="C36" s="36" t="s">
         <v>74</v>
       </c>
-      <c r="D36" s="31"/>
-      <c r="E36" s="31"/>
-      <c r="F36" s="31"/>
-      <c r="G36" s="31"/>
-      <c r="H36" s="31"/>
-      <c r="I36" s="27"/>
-      <c r="J36" s="27"/>
-      <c r="K36" s="27"/>
-      <c r="L36" s="27"/>
-      <c r="M36" s="27"/>
-      <c r="N36" s="27"/>
-      <c r="O36" s="27"/>
-      <c r="Q36" s="25"/>
-      <c r="R36" s="25"/>
-      <c r="S36" s="25"/>
-      <c r="T36" s="25"/>
-      <c r="U36" s="25"/>
-      <c r="V36" s="25"/>
-      <c r="W36" s="25"/>
-      <c r="X36" s="25"/>
-      <c r="Y36" s="25"/>
-      <c r="Z36" s="25"/>
-      <c r="AA36" s="25"/>
-      <c r="AB36" s="25"/>
-      <c r="AC36" s="25"/>
-      <c r="AD36" s="25"/>
-      <c r="AE36" s="25"/>
-      <c r="AF36" s="25"/>
-      <c r="AG36" s="25"/>
-      <c r="AH36" s="25"/>
-      <c r="AI36" s="25"/>
-      <c r="AJ36" s="25"/>
-      <c r="AK36" s="25"/>
-      <c r="AL36" s="25"/>
-      <c r="AM36" s="25"/>
-      <c r="AN36" s="25"/>
-      <c r="AO36" s="25"/>
-      <c r="AP36" s="25"/>
-      <c r="AQ36" s="25"/>
+      <c r="D36" s="36"/>
+      <c r="E36" s="36"/>
+      <c r="F36" s="36"/>
+      <c r="G36" s="36"/>
+      <c r="H36" s="36"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="32"/>
+      <c r="K36" s="32"/>
+      <c r="L36" s="32"/>
+      <c r="M36" s="32"/>
+      <c r="N36" s="32"/>
+      <c r="O36" s="32"/>
+      <c r="Q36" s="30"/>
+      <c r="R36" s="30"/>
+      <c r="S36" s="30"/>
+      <c r="T36" s="30"/>
+      <c r="U36" s="30"/>
+      <c r="V36" s="30"/>
+      <c r="W36" s="30"/>
+      <c r="X36" s="30"/>
+      <c r="Y36" s="30"/>
+      <c r="Z36" s="30"/>
+      <c r="AA36" s="30"/>
+      <c r="AB36" s="30"/>
+      <c r="AC36" s="30"/>
+      <c r="AD36" s="30"/>
+      <c r="AE36" s="30"/>
+      <c r="AF36" s="30"/>
+      <c r="AG36" s="30"/>
+      <c r="AH36" s="30"/>
+      <c r="AI36" s="30"/>
+      <c r="AJ36" s="30"/>
+      <c r="AK36" s="30"/>
+      <c r="AL36" s="30"/>
+      <c r="AM36" s="30"/>
+      <c r="AN36" s="30"/>
+      <c r="AO36" s="30"/>
+      <c r="AP36" s="30"/>
+      <c r="AQ36" s="30"/>
     </row>
     <row r="37" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB37" s="25"/>
-      <c r="AC37" s="25"/>
-      <c r="AD37" s="25"/>
-      <c r="AE37" s="25"/>
-      <c r="AF37" s="25"/>
-      <c r="AG37" s="25"/>
-      <c r="AH37" s="25"/>
-      <c r="AI37" s="25"/>
-      <c r="AJ37" s="25"/>
-      <c r="AK37" s="25"/>
-      <c r="AL37" s="25"/>
-      <c r="AM37" s="25"/>
-      <c r="AN37" s="25"/>
-      <c r="AO37" s="25"/>
-      <c r="AP37" s="25"/>
-      <c r="AQ37" s="25"/>
+      <c r="AB37" s="30"/>
+      <c r="AC37" s="30"/>
+      <c r="AD37" s="30"/>
+      <c r="AE37" s="30"/>
+      <c r="AF37" s="30"/>
+      <c r="AG37" s="30"/>
+      <c r="AH37" s="30"/>
+      <c r="AI37" s="30"/>
+      <c r="AJ37" s="30"/>
+      <c r="AK37" s="30"/>
+      <c r="AL37" s="30"/>
+      <c r="AM37" s="30"/>
+      <c r="AN37" s="30"/>
+      <c r="AO37" s="30"/>
+      <c r="AP37" s="30"/>
+      <c r="AQ37" s="30"/>
     </row>
     <row r="38" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB38" s="25"/>
-      <c r="AC38" s="25"/>
-      <c r="AD38" s="25"/>
-      <c r="AE38" s="25"/>
-      <c r="AF38" s="25"/>
-      <c r="AG38" s="25"/>
-      <c r="AH38" s="25"/>
-      <c r="AI38" s="25"/>
-      <c r="AJ38" s="25"/>
-      <c r="AK38" s="25"/>
-      <c r="AL38" s="25"/>
-      <c r="AM38" s="25"/>
-      <c r="AN38" s="25"/>
-      <c r="AO38" s="25"/>
-      <c r="AP38" s="25"/>
-      <c r="AQ38" s="25"/>
+      <c r="AB38" s="30"/>
+      <c r="AC38" s="30"/>
+      <c r="AD38" s="30"/>
+      <c r="AE38" s="30"/>
+      <c r="AF38" s="30"/>
+      <c r="AG38" s="30"/>
+      <c r="AH38" s="30"/>
+      <c r="AI38" s="30"/>
+      <c r="AJ38" s="30"/>
+      <c r="AK38" s="30"/>
+      <c r="AL38" s="30"/>
+      <c r="AM38" s="30"/>
+      <c r="AN38" s="30"/>
+      <c r="AO38" s="30"/>
+      <c r="AP38" s="30"/>
+      <c r="AQ38" s="30"/>
     </row>
     <row r="39" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB39" s="25"/>
-      <c r="AC39" s="25"/>
-      <c r="AD39" s="25"/>
-      <c r="AE39" s="25"/>
-      <c r="AF39" s="25"/>
-      <c r="AG39" s="25"/>
-      <c r="AH39" s="25"/>
-      <c r="AI39" s="25"/>
-      <c r="AJ39" s="25"/>
-      <c r="AK39" s="25"/>
-      <c r="AL39" s="25"/>
-      <c r="AM39" s="25"/>
-      <c r="AN39" s="25"/>
-      <c r="AO39" s="25"/>
-      <c r="AP39" s="25"/>
-      <c r="AQ39" s="25"/>
+      <c r="AB39" s="30"/>
+      <c r="AC39" s="30"/>
+      <c r="AD39" s="30"/>
+      <c r="AE39" s="30"/>
+      <c r="AF39" s="30"/>
+      <c r="AG39" s="30"/>
+      <c r="AH39" s="30"/>
+      <c r="AI39" s="30"/>
+      <c r="AJ39" s="30"/>
+      <c r="AK39" s="30"/>
+      <c r="AL39" s="30"/>
+      <c r="AM39" s="30"/>
+      <c r="AN39" s="30"/>
+      <c r="AO39" s="30"/>
+      <c r="AP39" s="30"/>
+      <c r="AQ39" s="30"/>
     </row>
     <row r="40" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB40" s="25"/>
-      <c r="AC40" s="25"/>
-      <c r="AD40" s="25"/>
-      <c r="AE40" s="25"/>
-      <c r="AF40" s="25"/>
-      <c r="AG40" s="25"/>
-      <c r="AH40" s="25"/>
-      <c r="AI40" s="25"/>
-      <c r="AJ40" s="25"/>
-      <c r="AK40" s="25"/>
-      <c r="AL40" s="25"/>
-      <c r="AM40" s="25"/>
-      <c r="AN40" s="25"/>
-      <c r="AO40" s="25"/>
-      <c r="AP40" s="25"/>
-      <c r="AQ40" s="25"/>
+      <c r="AB40" s="30"/>
+      <c r="AC40" s="30"/>
+      <c r="AD40" s="30"/>
+      <c r="AE40" s="30"/>
+      <c r="AF40" s="30"/>
+      <c r="AG40" s="30"/>
+      <c r="AH40" s="30"/>
+      <c r="AI40" s="30"/>
+      <c r="AJ40" s="30"/>
+      <c r="AK40" s="30"/>
+      <c r="AL40" s="30"/>
+      <c r="AM40" s="30"/>
+      <c r="AN40" s="30"/>
+      <c r="AO40" s="30"/>
+      <c r="AP40" s="30"/>
+      <c r="AQ40" s="30"/>
     </row>
     <row r="41" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB41" s="25"/>
-      <c r="AC41" s="25"/>
-      <c r="AD41" s="25"/>
-      <c r="AE41" s="25"/>
-      <c r="AF41" s="25"/>
-      <c r="AG41" s="25"/>
-      <c r="AH41" s="25"/>
-      <c r="AI41" s="25"/>
-      <c r="AJ41" s="25"/>
-      <c r="AK41" s="25"/>
-      <c r="AL41" s="25"/>
-      <c r="AM41" s="25"/>
-      <c r="AN41" s="25"/>
-      <c r="AO41" s="25"/>
-      <c r="AP41" s="25"/>
-      <c r="AQ41" s="25"/>
+      <c r="AB41" s="30"/>
+      <c r="AC41" s="30"/>
+      <c r="AD41" s="30"/>
+      <c r="AE41" s="30"/>
+      <c r="AF41" s="30"/>
+      <c r="AG41" s="30"/>
+      <c r="AH41" s="30"/>
+      <c r="AI41" s="30"/>
+      <c r="AJ41" s="30"/>
+      <c r="AK41" s="30"/>
+      <c r="AL41" s="30"/>
+      <c r="AM41" s="30"/>
+      <c r="AN41" s="30"/>
+      <c r="AO41" s="30"/>
+      <c r="AP41" s="30"/>
+      <c r="AQ41" s="30"/>
     </row>
     <row r="42" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB42" s="25" t="e" vm="8">
+      <c r="AB42" s="30" t="e" vm="8">
         <v>#VALUE!</v>
       </c>
-      <c r="AC42" s="25"/>
-      <c r="AD42" s="25"/>
-      <c r="AE42" s="25"/>
-      <c r="AF42" s="25"/>
-      <c r="AG42" s="25"/>
-      <c r="AH42" s="25"/>
-      <c r="AI42" s="25"/>
-      <c r="AJ42" s="25"/>
-      <c r="AK42" s="25"/>
-      <c r="AL42" s="25"/>
-      <c r="AM42" s="25"/>
-      <c r="AN42" s="25"/>
-      <c r="AO42" s="25"/>
-      <c r="AP42" s="25"/>
-      <c r="AQ42" s="25"/>
+      <c r="AC42" s="30"/>
+      <c r="AD42" s="30"/>
+      <c r="AE42" s="30"/>
+      <c r="AF42" s="30"/>
+      <c r="AG42" s="30"/>
+      <c r="AH42" s="30"/>
+      <c r="AI42" s="30"/>
+      <c r="AJ42" s="30"/>
+      <c r="AK42" s="30"/>
+      <c r="AL42" s="30"/>
+      <c r="AM42" s="30"/>
+      <c r="AN42" s="30"/>
+      <c r="AO42" s="30"/>
+      <c r="AP42" s="30"/>
+      <c r="AQ42" s="30"/>
     </row>
     <row r="43" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB43" s="25"/>
-      <c r="AC43" s="25"/>
-      <c r="AD43" s="25"/>
-      <c r="AE43" s="25"/>
-      <c r="AF43" s="25"/>
-      <c r="AG43" s="25"/>
-      <c r="AH43" s="25"/>
-      <c r="AI43" s="25"/>
-      <c r="AJ43" s="25"/>
-      <c r="AK43" s="25"/>
-      <c r="AL43" s="25"/>
-      <c r="AM43" s="25"/>
-      <c r="AN43" s="25"/>
-      <c r="AO43" s="25"/>
-      <c r="AP43" s="25"/>
-      <c r="AQ43" s="25"/>
+      <c r="AB43" s="30"/>
+      <c r="AC43" s="30"/>
+      <c r="AD43" s="30"/>
+      <c r="AE43" s="30"/>
+      <c r="AF43" s="30"/>
+      <c r="AG43" s="30"/>
+      <c r="AH43" s="30"/>
+      <c r="AI43" s="30"/>
+      <c r="AJ43" s="30"/>
+      <c r="AK43" s="30"/>
+      <c r="AL43" s="30"/>
+      <c r="AM43" s="30"/>
+      <c r="AN43" s="30"/>
+      <c r="AO43" s="30"/>
+      <c r="AP43" s="30"/>
+      <c r="AQ43" s="30"/>
     </row>
     <row r="44" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB44" s="25"/>
-      <c r="AC44" s="25"/>
-      <c r="AD44" s="25"/>
-      <c r="AE44" s="25"/>
-      <c r="AF44" s="25"/>
-      <c r="AG44" s="25"/>
-      <c r="AH44" s="25"/>
-      <c r="AI44" s="25"/>
-      <c r="AJ44" s="25"/>
-      <c r="AK44" s="25"/>
-      <c r="AL44" s="25"/>
-      <c r="AM44" s="25"/>
-      <c r="AN44" s="25"/>
-      <c r="AO44" s="25"/>
-      <c r="AP44" s="25"/>
-      <c r="AQ44" s="25"/>
+      <c r="AB44" s="30"/>
+      <c r="AC44" s="30"/>
+      <c r="AD44" s="30"/>
+      <c r="AE44" s="30"/>
+      <c r="AF44" s="30"/>
+      <c r="AG44" s="30"/>
+      <c r="AH44" s="30"/>
+      <c r="AI44" s="30"/>
+      <c r="AJ44" s="30"/>
+      <c r="AK44" s="30"/>
+      <c r="AL44" s="30"/>
+      <c r="AM44" s="30"/>
+      <c r="AN44" s="30"/>
+      <c r="AO44" s="30"/>
+      <c r="AP44" s="30"/>
+      <c r="AQ44" s="30"/>
     </row>
     <row r="45" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB45" s="25"/>
-      <c r="AC45" s="25"/>
-      <c r="AD45" s="25"/>
-      <c r="AE45" s="25"/>
-      <c r="AF45" s="25"/>
-      <c r="AG45" s="25"/>
-      <c r="AH45" s="25"/>
-      <c r="AI45" s="25"/>
-      <c r="AJ45" s="25"/>
-      <c r="AK45" s="25"/>
-      <c r="AL45" s="25"/>
-      <c r="AM45" s="25"/>
-      <c r="AN45" s="25"/>
-      <c r="AO45" s="25"/>
-      <c r="AP45" s="25"/>
-      <c r="AQ45" s="25"/>
+      <c r="AB45" s="30"/>
+      <c r="AC45" s="30"/>
+      <c r="AD45" s="30"/>
+      <c r="AE45" s="30"/>
+      <c r="AF45" s="30"/>
+      <c r="AG45" s="30"/>
+      <c r="AH45" s="30"/>
+      <c r="AI45" s="30"/>
+      <c r="AJ45" s="30"/>
+      <c r="AK45" s="30"/>
+      <c r="AL45" s="30"/>
+      <c r="AM45" s="30"/>
+      <c r="AN45" s="30"/>
+      <c r="AO45" s="30"/>
+      <c r="AP45" s="30"/>
+      <c r="AQ45" s="30"/>
     </row>
     <row r="46" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB46" s="25"/>
-      <c r="AC46" s="25"/>
-      <c r="AD46" s="25"/>
-      <c r="AE46" s="25"/>
-      <c r="AF46" s="25"/>
-      <c r="AG46" s="25"/>
-      <c r="AH46" s="25"/>
-      <c r="AI46" s="25"/>
-      <c r="AJ46" s="25"/>
-      <c r="AK46" s="25"/>
-      <c r="AL46" s="25"/>
-      <c r="AM46" s="25"/>
-      <c r="AN46" s="25"/>
-      <c r="AO46" s="25"/>
-      <c r="AP46" s="25"/>
-      <c r="AQ46" s="25"/>
+      <c r="AB46" s="30"/>
+      <c r="AC46" s="30"/>
+      <c r="AD46" s="30"/>
+      <c r="AE46" s="30"/>
+      <c r="AF46" s="30"/>
+      <c r="AG46" s="30"/>
+      <c r="AH46" s="30"/>
+      <c r="AI46" s="30"/>
+      <c r="AJ46" s="30"/>
+      <c r="AK46" s="30"/>
+      <c r="AL46" s="30"/>
+      <c r="AM46" s="30"/>
+      <c r="AN46" s="30"/>
+      <c r="AO46" s="30"/>
+      <c r="AP46" s="30"/>
+      <c r="AQ46" s="30"/>
     </row>
     <row r="47" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB47" s="25"/>
-      <c r="AC47" s="25"/>
-      <c r="AD47" s="25"/>
-      <c r="AE47" s="25"/>
-      <c r="AF47" s="25"/>
-      <c r="AG47" s="25"/>
-      <c r="AH47" s="25"/>
-      <c r="AI47" s="25"/>
-      <c r="AJ47" s="25"/>
-      <c r="AK47" s="25"/>
-      <c r="AL47" s="25"/>
-      <c r="AM47" s="25"/>
-      <c r="AN47" s="25"/>
-      <c r="AO47" s="25"/>
-      <c r="AP47" s="25"/>
-      <c r="AQ47" s="25"/>
+      <c r="AB47" s="30"/>
+      <c r="AC47" s="30"/>
+      <c r="AD47" s="30"/>
+      <c r="AE47" s="30"/>
+      <c r="AF47" s="30"/>
+      <c r="AG47" s="30"/>
+      <c r="AH47" s="30"/>
+      <c r="AI47" s="30"/>
+      <c r="AJ47" s="30"/>
+      <c r="AK47" s="30"/>
+      <c r="AL47" s="30"/>
+      <c r="AM47" s="30"/>
+      <c r="AN47" s="30"/>
+      <c r="AO47" s="30"/>
+      <c r="AP47" s="30"/>
+      <c r="AQ47" s="30"/>
     </row>
     <row r="48" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="AB48" s="25"/>
-      <c r="AC48" s="25"/>
-      <c r="AD48" s="25"/>
-      <c r="AE48" s="25"/>
-      <c r="AF48" s="25"/>
-      <c r="AG48" s="25"/>
-      <c r="AH48" s="25"/>
-      <c r="AI48" s="25"/>
-      <c r="AJ48" s="25"/>
-      <c r="AK48" s="25"/>
-      <c r="AL48" s="25"/>
-      <c r="AM48" s="25"/>
-      <c r="AN48" s="25"/>
-      <c r="AO48" s="25"/>
-      <c r="AP48" s="25"/>
-      <c r="AQ48" s="25"/>
+      <c r="AB48" s="30"/>
+      <c r="AC48" s="30"/>
+      <c r="AD48" s="30"/>
+      <c r="AE48" s="30"/>
+      <c r="AF48" s="30"/>
+      <c r="AG48" s="30"/>
+      <c r="AH48" s="30"/>
+      <c r="AI48" s="30"/>
+      <c r="AJ48" s="30"/>
+      <c r="AK48" s="30"/>
+      <c r="AL48" s="30"/>
+      <c r="AM48" s="30"/>
+      <c r="AN48" s="30"/>
+      <c r="AO48" s="30"/>
+      <c r="AP48" s="30"/>
+      <c r="AQ48" s="30"/>
     </row>
     <row r="49" spans="28:43" x14ac:dyDescent="0.3">
-      <c r="AB49" s="25"/>
-      <c r="AC49" s="25"/>
-      <c r="AD49" s="25"/>
-      <c r="AE49" s="25"/>
-      <c r="AF49" s="25"/>
-      <c r="AG49" s="25"/>
-      <c r="AH49" s="25"/>
-      <c r="AI49" s="25"/>
-      <c r="AJ49" s="25"/>
-      <c r="AK49" s="25"/>
-      <c r="AL49" s="25"/>
-      <c r="AM49" s="25"/>
-      <c r="AN49" s="25"/>
-      <c r="AO49" s="25"/>
-      <c r="AP49" s="25"/>
-      <c r="AQ49" s="25"/>
+      <c r="AB49" s="30"/>
+      <c r="AC49" s="30"/>
+      <c r="AD49" s="30"/>
+      <c r="AE49" s="30"/>
+      <c r="AF49" s="30"/>
+      <c r="AG49" s="30"/>
+      <c r="AH49" s="30"/>
+      <c r="AI49" s="30"/>
+      <c r="AJ49" s="30"/>
+      <c r="AK49" s="30"/>
+      <c r="AL49" s="30"/>
+      <c r="AM49" s="30"/>
+      <c r="AN49" s="30"/>
+      <c r="AO49" s="30"/>
+      <c r="AP49" s="30"/>
+      <c r="AQ49" s="30"/>
     </row>
     <row r="50" spans="28:43" x14ac:dyDescent="0.3">
-      <c r="AB50" s="25"/>
-      <c r="AC50" s="25"/>
-      <c r="AD50" s="25"/>
-      <c r="AE50" s="25"/>
-      <c r="AF50" s="25"/>
-      <c r="AG50" s="25"/>
-      <c r="AH50" s="25"/>
-      <c r="AI50" s="25"/>
-      <c r="AJ50" s="25"/>
-      <c r="AK50" s="25"/>
-      <c r="AL50" s="25"/>
-      <c r="AM50" s="25"/>
-      <c r="AN50" s="25"/>
-      <c r="AO50" s="25"/>
-      <c r="AP50" s="25"/>
-      <c r="AQ50" s="25"/>
+      <c r="AB50" s="30"/>
+      <c r="AC50" s="30"/>
+      <c r="AD50" s="30"/>
+      <c r="AE50" s="30"/>
+      <c r="AF50" s="30"/>
+      <c r="AG50" s="30"/>
+      <c r="AH50" s="30"/>
+      <c r="AI50" s="30"/>
+      <c r="AJ50" s="30"/>
+      <c r="AK50" s="30"/>
+      <c r="AL50" s="30"/>
+      <c r="AM50" s="30"/>
+      <c r="AN50" s="30"/>
+      <c r="AO50" s="30"/>
+      <c r="AP50" s="30"/>
+      <c r="AQ50" s="30"/>
     </row>
     <row r="51" spans="28:43" x14ac:dyDescent="0.3">
-      <c r="AB51" s="25"/>
-      <c r="AC51" s="25"/>
-      <c r="AD51" s="25"/>
-      <c r="AE51" s="25"/>
-      <c r="AF51" s="25"/>
-      <c r="AG51" s="25"/>
-      <c r="AH51" s="25"/>
-      <c r="AI51" s="25"/>
-      <c r="AJ51" s="25"/>
-      <c r="AK51" s="25"/>
-      <c r="AL51" s="25"/>
-      <c r="AM51" s="25"/>
-      <c r="AN51" s="25"/>
-      <c r="AO51" s="25"/>
-      <c r="AP51" s="25"/>
-      <c r="AQ51" s="25"/>
+      <c r="AB51" s="30"/>
+      <c r="AC51" s="30"/>
+      <c r="AD51" s="30"/>
+      <c r="AE51" s="30"/>
+      <c r="AF51" s="30"/>
+      <c r="AG51" s="30"/>
+      <c r="AH51" s="30"/>
+      <c r="AI51" s="30"/>
+      <c r="AJ51" s="30"/>
+      <c r="AK51" s="30"/>
+      <c r="AL51" s="30"/>
+      <c r="AM51" s="30"/>
+      <c r="AN51" s="30"/>
+      <c r="AO51" s="30"/>
+      <c r="AP51" s="30"/>
+      <c r="AQ51" s="30"/>
     </row>
     <row r="52" spans="28:43" x14ac:dyDescent="0.3">
-      <c r="AB52" s="25"/>
-      <c r="AC52" s="25"/>
-      <c r="AD52" s="25"/>
-      <c r="AE52" s="25"/>
-      <c r="AF52" s="25"/>
-      <c r="AG52" s="25"/>
-      <c r="AH52" s="25"/>
-      <c r="AI52" s="25"/>
-      <c r="AJ52" s="25"/>
-      <c r="AK52" s="25"/>
-      <c r="AL52" s="25"/>
-      <c r="AM52" s="25"/>
-      <c r="AN52" s="25"/>
-      <c r="AO52" s="25"/>
-      <c r="AP52" s="25"/>
-      <c r="AQ52" s="25"/>
+      <c r="AB52" s="30"/>
+      <c r="AC52" s="30"/>
+      <c r="AD52" s="30"/>
+      <c r="AE52" s="30"/>
+      <c r="AF52" s="30"/>
+      <c r="AG52" s="30"/>
+      <c r="AH52" s="30"/>
+      <c r="AI52" s="30"/>
+      <c r="AJ52" s="30"/>
+      <c r="AK52" s="30"/>
+      <c r="AL52" s="30"/>
+      <c r="AM52" s="30"/>
+      <c r="AN52" s="30"/>
+      <c r="AO52" s="30"/>
+      <c r="AP52" s="30"/>
+      <c r="AQ52" s="30"/>
     </row>
     <row r="53" spans="28:43" x14ac:dyDescent="0.3">
-      <c r="AB53" s="25"/>
-      <c r="AC53" s="25"/>
-      <c r="AD53" s="25"/>
-      <c r="AE53" s="25"/>
-      <c r="AF53" s="25"/>
-      <c r="AG53" s="25"/>
-      <c r="AH53" s="25"/>
-      <c r="AI53" s="25"/>
-      <c r="AJ53" s="25"/>
-      <c r="AK53" s="25"/>
-      <c r="AL53" s="25"/>
-      <c r="AM53" s="25"/>
-      <c r="AN53" s="25"/>
-      <c r="AO53" s="25"/>
-      <c r="AP53" s="25"/>
-      <c r="AQ53" s="25"/>
+      <c r="AB53" s="30"/>
+      <c r="AC53" s="30"/>
+      <c r="AD53" s="30"/>
+      <c r="AE53" s="30"/>
+      <c r="AF53" s="30"/>
+      <c r="AG53" s="30"/>
+      <c r="AH53" s="30"/>
+      <c r="AI53" s="30"/>
+      <c r="AJ53" s="30"/>
+      <c r="AK53" s="30"/>
+      <c r="AL53" s="30"/>
+      <c r="AM53" s="30"/>
+      <c r="AN53" s="30"/>
+      <c r="AO53" s="30"/>
+      <c r="AP53" s="30"/>
+      <c r="AQ53" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="43">
+  <mergeCells count="42">
+    <mergeCell ref="Q22:AA24"/>
+    <mergeCell ref="AB22:AQ31"/>
     <mergeCell ref="AB42:AQ53"/>
     <mergeCell ref="T4:X4"/>
     <mergeCell ref="AB32:AQ41"/>
@@ -5657,7 +5678,6 @@
     <mergeCell ref="I35:O35"/>
     <mergeCell ref="C36:H36"/>
     <mergeCell ref="I36:O36"/>
-    <mergeCell ref="AB28:AQ31"/>
     <mergeCell ref="C29:H29"/>
     <mergeCell ref="I29:O29"/>
     <mergeCell ref="C30:H30"/>
@@ -5667,14 +5687,6 @@
     <mergeCell ref="I31:O31"/>
     <mergeCell ref="C32:H32"/>
     <mergeCell ref="I32:O32"/>
-    <mergeCell ref="I26:O26"/>
-    <mergeCell ref="Q26:AA29"/>
-    <mergeCell ref="C27:H27"/>
-    <mergeCell ref="I27:O27"/>
-    <mergeCell ref="C28:H28"/>
-    <mergeCell ref="I28:O28"/>
-    <mergeCell ref="Q22:AA25"/>
-    <mergeCell ref="AB22:AQ27"/>
     <mergeCell ref="AR22:AY24"/>
     <mergeCell ref="C23:H23"/>
     <mergeCell ref="I23:O23"/>
@@ -5683,6 +5695,12 @@
     <mergeCell ref="C25:H25"/>
     <mergeCell ref="I25:O25"/>
     <mergeCell ref="C26:H26"/>
+    <mergeCell ref="I26:O26"/>
+    <mergeCell ref="Q26:AA29"/>
+    <mergeCell ref="C27:H27"/>
+    <mergeCell ref="I27:O27"/>
+    <mergeCell ref="C28:H28"/>
+    <mergeCell ref="I28:O28"/>
     <mergeCell ref="C3:H3"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="C21:H21"/>

</xml_diff>

<commit_message>
Revisiting method, and updating some figures
</commit_message>
<xml_diff>
--- a/IndicatorsForClusters.xlsx
+++ b/IndicatorsForClusters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1c3256d208fb6548/Personlig/Aske Banke Consultancy/YALE/Metodeartikel_WorldDevelopmentJournal/WorldDevelopmentArticleGit/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="543" documentId="8_{9856C943-DD01-465B-AD17-0E409E296684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8878DECD-3FB3-4C5B-B7AB-34D399F750D7}"/>
+  <xr:revisionPtr revIDLastSave="741" documentId="8_{9856C943-DD01-465B-AD17-0E409E296684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC687424-937E-4C92-895A-E846DA2EB505}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{726B2859-724A-4801-8E74-5A4E1AFAB973}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{726B2859-724A-4801-8E74-5A4E1AFAB973}"/>
   </bookViews>
   <sheets>
     <sheet name="Unscaled Experiments" sheetId="2" r:id="rId1"/>
@@ -18,9 +18,11 @@
     <sheet name="Experiments" sheetId="3" r:id="rId3"/>
     <sheet name="Overview of indicators and DLS" sheetId="1" r:id="rId4"/>
     <sheet name="Sheet1" sheetId="6" r:id="rId5"/>
+    <sheet name="New table in report" sheetId="7" r:id="rId6"/>
+    <sheet name="Old table in report" sheetId="8" r:id="rId7"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId6"/>
+    <externalReference r:id="rId8"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -170,7 +172,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="198">
   <si>
     <t>SPI</t>
   </si>
@@ -438,13 +440,852 @@
   </si>
   <si>
     <t>DLSFew_bestAlignment_90</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>DLS Indicator</t>
+  </si>
+  <si>
+    <t>DHS Variables with Minimum Thresholds Used to Define DLS</t>
+  </si>
+  <si>
+    <t>Food/Nutrition</t>
+  </si>
+  <si>
+    <t>Food prep/storage</t>
+  </si>
+  <si>
+    <r>
+      <t>Main source of drinking water (hv201):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Household has access to “Safely managed” drinking water as per WASH guidelines</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Type of toilet (hv205):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Household has access to “Safely managed” toilet facility as per WASH guidelines</t>
+    </r>
+  </si>
+  <si>
+    <t>Provision of health care</t>
+  </si>
+  <si>
+    <r>
+      <t>Problems faced in getting healthcare (v467a–v467j):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Binary indicator. If any of v467a–v467j indicates no access, response = 1</t>
+    </r>
+  </si>
+  <si>
+    <t>Social Connectedness</t>
+  </si>
+  <si>
+    <t>Indicators used in this study</t>
+  </si>
+  <si>
+    <t>Access to electricity </t>
+  </si>
+  <si>
+    <t>Child stunting </t>
+  </si>
+  <si>
+    <t>Nutritional deficiencies </t>
+  </si>
+  <si>
+    <t>Diet low in fruits and vegetables </t>
+  </si>
+  <si>
+    <t>Daily Calorie supply </t>
+  </si>
+  <si>
+    <t>Protein supply </t>
+  </si>
+  <si>
+    <t>Deaths from household air pollution </t>
+  </si>
+  <si>
+    <t>Prevalence of cooking with coal/biomass </t>
+  </si>
+  <si>
+    <t>Clean Fuels </t>
+  </si>
+  <si>
+    <t>No access to a handwashing facility </t>
+  </si>
+  <si>
+    <t>Deaths from unsafe water, sanitation and hygiene </t>
+  </si>
+  <si>
+    <t>Improved water source </t>
+  </si>
+  <si>
+    <t>Safely Managed Drinking Water </t>
+  </si>
+  <si>
+    <t>Improved sanitation </t>
+  </si>
+  <si>
+    <t>Safely Managed Sanitation </t>
+  </si>
+  <si>
+    <t>Deaths from infectious diseases </t>
+  </si>
+  <si>
+    <t>Maternal mortality </t>
+  </si>
+  <si>
+    <t>Child mortality  </t>
+  </si>
+  <si>
+    <t>Life expectancy at 60 years </t>
+  </si>
+  <si>
+    <t>Healthy life expectancy </t>
+  </si>
+  <si>
+    <t>Premature deaths from non-communicable diseases </t>
+  </si>
+  <si>
+    <t>Equal access to quality healthcare </t>
+  </si>
+  <si>
+    <t>Universal health coverage </t>
+  </si>
+  <si>
+    <t>Physicians per 1000 </t>
+  </si>
+  <si>
+    <t>Hospital beds per 1000 </t>
+  </si>
+  <si>
+    <t>Primary School Enrollment </t>
+  </si>
+  <si>
+    <t>Gender parity in basic/advanced education (distance from parity)  </t>
+  </si>
+  <si>
+    <t>Equal access to quality education (0=unequal; 4=equal)  </t>
+  </si>
+  <si>
+    <t>Mean years of schooling (years) </t>
+  </si>
+  <si>
+    <t>Population with advanced education (proportion of pop.)  </t>
+  </si>
+  <si>
+    <t>Years of tertiary schooling (years) </t>
+  </si>
+  <si>
+    <t>Respect for academic freedom (0=low; 1=high) </t>
+  </si>
+  <si>
+    <t>Population with no/advanced education (proportion of pop.)  </t>
+  </si>
+  <si>
+    <t>Alternative sources of information (0=low; 1=high) </t>
+  </si>
+  <si>
+    <t>Internet users (% of pop.)  </t>
+  </si>
+  <si>
+    <t>Mobile and landline telephone subscriptions (subscriptions/100 people)  </t>
+  </si>
+  <si>
+    <t>Child stunting</t>
+  </si>
+  <si>
+    <r>
+      <t>Household possesses bicycle (hv210):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> If has bicycle, response = 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Household possesses motorcycle (hv211):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> If has motorcycle, response = 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Household possesses car (hv212):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> If has car, response = 1</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(All Binary Indicators)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Household possesses radio (hv207):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> If has radio, response = 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Household possesses television (hv208):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> If has TV, response = 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Household possesses computer (hv243):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> If has computer, response = 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Household possesses telephone (hv221):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> If has telephone, response = 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Household possesses cell phone (hv243A):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> If has cellphone, response = 1</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(All Binary Indicators)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Is the household member still in school? (hv110):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Binary indicator. If in school and belongs to compulsory schooling age, response = 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Age of household members (hv105):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Compulsory schooling age between 6 and 10</t>
+    </r>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>UN HABITAT</t>
+  </si>
+  <si>
+    <r>
+      <t>BMI (v445):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> If BMI is below 1850, then undernourished.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Height (v438):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> For BMI calculation
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Weight (v437):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> For BMI calculation</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Wall material (hv214):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Finished wall materials (tin, cement, stone, bricks, wood planks)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Roof material (hv215):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Finished roof materials (tin, wood, ceramic tiles, cement, roofing shingles)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access to electricity (hv206):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Binary indicator. If household has access, response = 1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Floor Material (hv213):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Finished floor material (parquet or polished wood, tiles, cement, carpet)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Household size (hv009)/Number of rooms (hv216):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Number of people per room is less than 3</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Household has a refrigerator (hv209):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Binary indicator. If household has refrigerator, response = 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Household uses modern cooking fuel (hv239):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Household has access to at least one of the following types of fuels: gas, LPG, electricity, solar</t>
+    </r>
+  </si>
+  <si>
+    <t>The indicator used is an aggregate indicator measuring lack of one or more of the following: access to improved water, improved sanitation, sufficient living area, housing durability and security of tenure.  Rural population is not considered.</t>
+  </si>
+  <si>
+    <t>FAO</t>
+  </si>
+  <si>
+    <t>World Bank</t>
+  </si>
+  <si>
+    <t>UNESCO</t>
+  </si>
+  <si>
+    <t>https://data.worldbank.org/indicator/SE.PRM.NENR</t>
+  </si>
+  <si>
+    <t>https://databank.worldbank.org/source/world-development-indicators/Series/SH.MED.BEDS.ZS</t>
+  </si>
+  <si>
+    <t>https://databank.worldbank.org/source/health-nutrition-and-population-statistics/Series/SH.MED.PHYS.ZS</t>
+  </si>
+  <si>
+    <t>https://data.unhabitat.org/pages/housing-slums-and-informal-settlements</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>https://data.worldbank.org/indicator/SH.STA.SMSS.ZS</t>
+  </si>
+  <si>
+    <t>WHO / UNICEF JMP</t>
+  </si>
+  <si>
+    <t>https://data.worldbank.org/indicator/SH.H2O.SMDW.ZS</t>
+  </si>
+  <si>
+    <t>https://data.worldbank.org/indicator/EG.CFT.ACCS.ZS</t>
+  </si>
+  <si>
+    <t>IEA</t>
+  </si>
+  <si>
+    <t>https://www.who.int/data/gho/data/indicators/indicator-details/GHO/gho-ghe-hale-healthy-life-expectancy-at-birth</t>
+  </si>
+  <si>
+    <t>WHO</t>
+  </si>
+  <si>
+    <t>DLS answered</t>
+  </si>
+  <si>
+    <t>/</t>
+  </si>
+  <si>
+    <t>+</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Share of urban population living in slums</t>
+  </si>
+  <si>
+    <r>
+      <t>DLS dimension</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <strike/>
+        <sz val="10"/>
+        <color rgb="FF0078D4"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>s</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+  </si>
+  <si>
+    <t>DHS variables </t>
+  </si>
+  <si>
+    <t>Indicator used in this study </t>
+  </si>
+  <si>
+    <t>Source </t>
+  </si>
+  <si>
+    <r>
+      <t>Comment</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+  </si>
+  <si>
+    <t>Housing </t>
+  </si>
+  <si>
+    <t>Floor type </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Share slums </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Share of urban population living in slums </t>
+    </r>
+  </si>
+  <si>
+    <t>Household size </t>
+  </si>
+  <si>
+    <t>Number of rooms </t>
+  </si>
+  <si>
+    <t>Thermal comfort </t>
+  </si>
+  <si>
+    <t>Wall type </t>
+  </si>
+  <si>
+    <t>Roof type </t>
+  </si>
+  <si>
+    <t>Electricity access </t>
+  </si>
+  <si>
+    <t>Food &amp; nutrition </t>
+  </si>
+  <si>
+    <t>Age of household members </t>
+  </si>
+  <si>
+    <t>Weight/heigh of household members </t>
+  </si>
+  <si>
+    <t>Food preparation </t>
+  </si>
+  <si>
+    <t>Use of modern cooking fuels </t>
+  </si>
+  <si>
+    <t>Possession of fridge </t>
+  </si>
+  <si>
+    <t>Water </t>
+  </si>
+  <si>
+    <t>Main water source (based on WASH criteria) </t>
+  </si>
+  <si>
+    <t>Sanitation </t>
+  </si>
+  <si>
+    <t>Type of toilet (based on WASH criteria) </t>
+  </si>
+  <si>
+    <t>Health Care </t>
+  </si>
+  <si>
+    <t>Reason for not using health care related to accessibility issues  </t>
+  </si>
+  <si>
+    <t>Education  </t>
+  </si>
+  <si>
+    <t>Highest level of schooling </t>
+  </si>
+  <si>
+    <t>Social Connectedness </t>
+  </si>
+  <si>
+    <r>
+      <t>House</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="9"/>
+        <color rgb="FF0078D4"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>h</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>ol</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="9"/>
+        <color rgb="FF0078D4"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>d</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>s information assets (e.g. radio, tv, computer) </t>
+    </r>
+  </si>
+  <si>
+    <t>Communication assets (e.g. phone or mobile) </t>
+  </si>
+  <si>
+    <t>Physical Connectedness </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -479,6 +1320,81 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <strike/>
+      <sz val="10"/>
+      <color rgb="FF0078D4"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF0078D4"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="9"/>
+      <color rgb="FF0078D4"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="9"/>
+      <color rgb="FF0078D4"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="9">
@@ -531,7 +1447,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -608,11 +1524,295 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF666666"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF666666"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF666666"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thick">
+        <color rgb="FF666666"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thick">
+        <color rgb="FF666666"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -661,66 +1861,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment textRotation="90"/>
     </xf>
@@ -734,14 +1874,228 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
@@ -1405,18 +2759,18 @@
       <c r="B3" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C3" s="35" t="s">
+      <c r="C3" s="52" t="s">
         <v>57</v>
       </c>
-      <c r="D3" s="35"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="35"/>
-      <c r="G3" s="35"/>
-      <c r="H3" s="38"/>
-      <c r="I3" s="34" t="s">
+      <c r="D3" s="52"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="52"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="51" t="s">
         <v>56</v>
       </c>
-      <c r="J3" s="35"/>
+      <c r="J3" s="52"/>
       <c r="K3" s="8"/>
       <c r="L3" s="8"/>
       <c r="M3" s="8"/>
@@ -1480,13 +2834,13 @@
       <c r="Q4" s="9" t="str">
         <v>BHN</v>
       </c>
-      <c r="T4" s="43" t="s">
+      <c r="T4" s="40" t="s">
         <v>53</v>
       </c>
-      <c r="U4" s="43"/>
-      <c r="V4" s="43"/>
-      <c r="W4" s="43"/>
-      <c r="X4" s="43"/>
+      <c r="U4" s="40"/>
+      <c r="V4" s="40"/>
+      <c r="W4" s="40"/>
+      <c r="X4" s="40"/>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B5" s="11" t="str" cm="1">
@@ -2430,23 +3784,23 @@
       <c r="B21" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="36" t="s">
+      <c r="C21" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="36"/>
-      <c r="I21" s="36" t="s">
+      <c r="D21" s="53"/>
+      <c r="E21" s="53"/>
+      <c r="F21" s="53"/>
+      <c r="G21" s="53"/>
+      <c r="H21" s="53"/>
+      <c r="I21" s="53" t="s">
         <v>41</v>
       </c>
-      <c r="J21" s="36"/>
-      <c r="K21" s="36"/>
-      <c r="L21" s="36"/>
-      <c r="M21" s="36"/>
-      <c r="N21" s="36"/>
-      <c r="O21" s="36"/>
+      <c r="J21" s="53"/>
+      <c r="K21" s="53"/>
+      <c r="L21" s="53"/>
+      <c r="M21" s="53"/>
+      <c r="N21" s="53"/>
+      <c r="O21" s="53"/>
       <c r="Q21" s="1" t="s">
         <v>58</v>
       </c>
@@ -2462,21 +3816,21 @@
         <f t="array" ref="B22:B36">TRANSPOSE(_xlfn.ANCHORARRAY(C4))</f>
         <v>BHN_FWB</v>
       </c>
-      <c r="C22" s="37" t="s">
+      <c r="C22" s="49" t="s">
         <v>43</v>
       </c>
-      <c r="D22" s="37"/>
-      <c r="E22" s="37"/>
-      <c r="F22" s="37"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="37"/>
-      <c r="I22" s="33"/>
-      <c r="J22" s="33"/>
-      <c r="K22" s="33"/>
-      <c r="L22" s="33"/>
-      <c r="M22" s="33"/>
-      <c r="N22" s="33"/>
-      <c r="O22" s="33"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="49"/>
+      <c r="I22" s="48"/>
+      <c r="J22" s="48"/>
+      <c r="K22" s="48"/>
+      <c r="L22" s="48"/>
+      <c r="M22" s="48"/>
+      <c r="N22" s="48"/>
+      <c r="O22" s="48"/>
       <c r="Q22" s="41" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
@@ -2526,21 +3880,21 @@
       <c r="B23" s="7" t="str">
         <v>BHN_FWB_AllExt</v>
       </c>
-      <c r="C23" s="37" t="s">
+      <c r="C23" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="D23" s="37"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="37"/>
-      <c r="G23" s="37"/>
-      <c r="H23" s="37"/>
-      <c r="I23" s="33"/>
-      <c r="J23" s="33"/>
-      <c r="K23" s="33"/>
-      <c r="L23" s="33"/>
-      <c r="M23" s="33"/>
-      <c r="N23" s="33"/>
-      <c r="O23" s="33"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="49"/>
+      <c r="I23" s="48"/>
+      <c r="J23" s="48"/>
+      <c r="K23" s="48"/>
+      <c r="L23" s="48"/>
+      <c r="M23" s="48"/>
+      <c r="N23" s="48"/>
+      <c r="O23" s="48"/>
       <c r="Q23" s="41"/>
       <c r="R23" s="41"/>
       <c r="S23" s="41"/>
@@ -2584,21 +3938,21 @@
       <c r="B24" s="7" t="str">
         <v>Few_indicators_closest_DLS_coverage</v>
       </c>
-      <c r="C24" s="37" t="s">
+      <c r="C24" s="49" t="s">
         <v>46</v>
       </c>
-      <c r="D24" s="37"/>
-      <c r="E24" s="37"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="37"/>
-      <c r="I24" s="33"/>
-      <c r="J24" s="33"/>
-      <c r="K24" s="33"/>
-      <c r="L24" s="33"/>
-      <c r="M24" s="33"/>
-      <c r="N24" s="33"/>
-      <c r="O24" s="33"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="49"/>
+      <c r="I24" s="48"/>
+      <c r="J24" s="48"/>
+      <c r="K24" s="48"/>
+      <c r="L24" s="48"/>
+      <c r="M24" s="48"/>
+      <c r="N24" s="48"/>
+      <c r="O24" s="48"/>
       <c r="Q24" s="41"/>
       <c r="R24" s="41"/>
       <c r="S24" s="41"/>
@@ -2642,21 +3996,21 @@
       <c r="B25" s="7" t="str">
         <v>Few_indicators_SPI_preferred</v>
       </c>
-      <c r="C25" s="37" t="s">
+      <c r="C25" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="D25" s="37"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="37"/>
-      <c r="G25" s="37"/>
-      <c r="H25" s="37"/>
-      <c r="I25" s="33"/>
-      <c r="J25" s="33"/>
-      <c r="K25" s="33"/>
-      <c r="L25" s="33"/>
-      <c r="M25" s="33"/>
-      <c r="N25" s="33"/>
-      <c r="O25" s="33"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="49"/>
+      <c r="I25" s="48"/>
+      <c r="J25" s="48"/>
+      <c r="K25" s="48"/>
+      <c r="L25" s="48"/>
+      <c r="M25" s="48"/>
+      <c r="N25" s="48"/>
+      <c r="O25" s="48"/>
       <c r="Q25" s="41"/>
       <c r="R25" s="41"/>
       <c r="S25" s="41"/>
@@ -2692,21 +4046,21 @@
       <c r="B26" s="7" t="str">
         <v>No_non_DLS</v>
       </c>
-      <c r="C26" s="32" t="s">
+      <c r="C26" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="32"/>
-      <c r="I26" s="33"/>
-      <c r="J26" s="33"/>
-      <c r="K26" s="33"/>
-      <c r="L26" s="33"/>
-      <c r="M26" s="33"/>
-      <c r="N26" s="33"/>
-      <c r="O26" s="33"/>
+      <c r="D26" s="50"/>
+      <c r="E26" s="50"/>
+      <c r="F26" s="50"/>
+      <c r="G26" s="50"/>
+      <c r="H26" s="50"/>
+      <c r="I26" s="48"/>
+      <c r="J26" s="48"/>
+      <c r="K26" s="48"/>
+      <c r="L26" s="48"/>
+      <c r="M26" s="48"/>
+      <c r="N26" s="48"/>
+      <c r="O26" s="48"/>
       <c r="Q26" s="41" t="e" vm="4">
         <v>#VALUE!</v>
       </c>
@@ -2744,21 +4098,21 @@
       <c r="B27" s="7" t="str">
         <v>Only_%_of_pop</v>
       </c>
-      <c r="C27" s="32" t="s">
+      <c r="C27" s="50" t="s">
         <v>50</v>
       </c>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="32"/>
-      <c r="H27" s="32"/>
-      <c r="I27" s="33"/>
-      <c r="J27" s="33"/>
-      <c r="K27" s="33"/>
-      <c r="L27" s="33"/>
-      <c r="M27" s="33"/>
-      <c r="N27" s="33"/>
-      <c r="O27" s="33"/>
+      <c r="D27" s="50"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="50"/>
+      <c r="G27" s="50"/>
+      <c r="H27" s="50"/>
+      <c r="I27" s="48"/>
+      <c r="J27" s="48"/>
+      <c r="K27" s="48"/>
+      <c r="L27" s="48"/>
+      <c r="M27" s="48"/>
+      <c r="N27" s="48"/>
+      <c r="O27" s="48"/>
       <c r="Q27" s="41"/>
       <c r="R27" s="41"/>
       <c r="S27" s="41"/>
@@ -2794,21 +4148,21 @@
       <c r="B28" s="17" t="str">
         <v>Few_indicators_closest_DLS_coverage_90</v>
       </c>
-      <c r="C28" s="39" t="s">
+      <c r="C28" s="44" t="s">
         <v>60</v>
       </c>
-      <c r="D28" s="39"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="39"/>
-      <c r="H28" s="39"/>
-      <c r="I28" s="40"/>
-      <c r="J28" s="40"/>
-      <c r="K28" s="40"/>
-      <c r="L28" s="40"/>
-      <c r="M28" s="40"/>
-      <c r="N28" s="40"/>
-      <c r="O28" s="40"/>
+      <c r="D28" s="44"/>
+      <c r="E28" s="44"/>
+      <c r="F28" s="44"/>
+      <c r="G28" s="44"/>
+      <c r="H28" s="44"/>
+      <c r="I28" s="46"/>
+      <c r="J28" s="46"/>
+      <c r="K28" s="46"/>
+      <c r="L28" s="46"/>
+      <c r="M28" s="46"/>
+      <c r="N28" s="46"/>
+      <c r="O28" s="46"/>
       <c r="Q28" s="41"/>
       <c r="R28" s="41"/>
       <c r="S28" s="41"/>
@@ -2846,21 +4200,21 @@
       <c r="B29" s="17" t="str">
         <v>Few_indicators_SPI_preferred_90</v>
       </c>
-      <c r="C29" s="39" t="s">
+      <c r="C29" s="44" t="s">
         <v>60</v>
       </c>
-      <c r="D29" s="39"/>
-      <c r="E29" s="39"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="39"/>
-      <c r="H29" s="39"/>
-      <c r="I29" s="40"/>
-      <c r="J29" s="40"/>
-      <c r="K29" s="40"/>
-      <c r="L29" s="40"/>
-      <c r="M29" s="40"/>
-      <c r="N29" s="40"/>
-      <c r="O29" s="40"/>
+      <c r="D29" s="44"/>
+      <c r="E29" s="44"/>
+      <c r="F29" s="44"/>
+      <c r="G29" s="44"/>
+      <c r="H29" s="44"/>
+      <c r="I29" s="46"/>
+      <c r="J29" s="46"/>
+      <c r="K29" s="46"/>
+      <c r="L29" s="46"/>
+      <c r="M29" s="46"/>
+      <c r="N29" s="46"/>
+      <c r="O29" s="46"/>
       <c r="Q29" s="41"/>
       <c r="R29" s="41"/>
       <c r="S29" s="41"/>
@@ -2896,21 +4250,21 @@
       <c r="B30" s="17" t="str">
         <v>Few_indicators_closeDLS_subPrimSchool</v>
       </c>
-      <c r="C30" s="44" t="s">
+      <c r="C30" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="D30" s="44"/>
-      <c r="E30" s="44"/>
-      <c r="F30" s="44"/>
-      <c r="G30" s="44"/>
-      <c r="H30" s="44"/>
-      <c r="I30" s="40"/>
-      <c r="J30" s="40"/>
-      <c r="K30" s="40"/>
-      <c r="L30" s="40"/>
-      <c r="M30" s="40"/>
-      <c r="N30" s="40"/>
-      <c r="O30" s="40"/>
+      <c r="D30" s="42"/>
+      <c r="E30" s="42"/>
+      <c r="F30" s="42"/>
+      <c r="G30" s="42"/>
+      <c r="H30" s="42"/>
+      <c r="I30" s="46"/>
+      <c r="J30" s="46"/>
+      <c r="K30" s="46"/>
+      <c r="L30" s="46"/>
+      <c r="M30" s="46"/>
+      <c r="N30" s="46"/>
+      <c r="O30" s="46"/>
       <c r="Q30" s="41" t="e" vm="6">
         <v>#VALUE!</v>
       </c>
@@ -2948,21 +4302,21 @@
       <c r="B31" s="17" t="str">
         <v>No_non_DLS_90</v>
       </c>
-      <c r="C31" s="39" t="s">
+      <c r="C31" s="44" t="s">
         <v>60</v>
       </c>
-      <c r="D31" s="39"/>
-      <c r="E31" s="39"/>
-      <c r="F31" s="39"/>
-      <c r="G31" s="39"/>
-      <c r="H31" s="39"/>
-      <c r="I31" s="40"/>
-      <c r="J31" s="40"/>
-      <c r="K31" s="40"/>
-      <c r="L31" s="40"/>
-      <c r="M31" s="40"/>
-      <c r="N31" s="40"/>
-      <c r="O31" s="40"/>
+      <c r="D31" s="44"/>
+      <c r="E31" s="44"/>
+      <c r="F31" s="44"/>
+      <c r="G31" s="44"/>
+      <c r="H31" s="44"/>
+      <c r="I31" s="46"/>
+      <c r="J31" s="46"/>
+      <c r="K31" s="46"/>
+      <c r="L31" s="46"/>
+      <c r="M31" s="46"/>
+      <c r="N31" s="46"/>
+      <c r="O31" s="46"/>
       <c r="Q31" s="41"/>
       <c r="R31" s="41"/>
       <c r="S31" s="41"/>
@@ -2998,21 +4352,21 @@
       <c r="B32" s="17" t="str">
         <v>Few_Indicators_subWatSani</v>
       </c>
-      <c r="C32" s="39" t="s">
+      <c r="C32" s="44" t="s">
         <v>65</v>
       </c>
-      <c r="D32" s="39"/>
-      <c r="E32" s="39"/>
-      <c r="F32" s="39"/>
-      <c r="G32" s="39"/>
-      <c r="H32" s="39"/>
-      <c r="I32" s="40"/>
-      <c r="J32" s="40"/>
-      <c r="K32" s="40"/>
-      <c r="L32" s="40"/>
-      <c r="M32" s="40"/>
-      <c r="N32" s="40"/>
-      <c r="O32" s="40"/>
+      <c r="D32" s="44"/>
+      <c r="E32" s="44"/>
+      <c r="F32" s="44"/>
+      <c r="G32" s="44"/>
+      <c r="H32" s="44"/>
+      <c r="I32" s="46"/>
+      <c r="J32" s="46"/>
+      <c r="K32" s="46"/>
+      <c r="L32" s="46"/>
+      <c r="M32" s="46"/>
+      <c r="N32" s="46"/>
+      <c r="O32" s="46"/>
       <c r="Q32" s="41"/>
       <c r="R32" s="41"/>
       <c r="S32" s="41"/>
@@ -3058,13 +4412,13 @@
       <c r="F33" s="45"/>
       <c r="G33" s="45"/>
       <c r="H33" s="45"/>
-      <c r="I33" s="42"/>
-      <c r="J33" s="42"/>
-      <c r="K33" s="42"/>
-      <c r="L33" s="42"/>
-      <c r="M33" s="42"/>
-      <c r="N33" s="42"/>
-      <c r="O33" s="42"/>
+      <c r="I33" s="43"/>
+      <c r="J33" s="43"/>
+      <c r="K33" s="43"/>
+      <c r="L33" s="43"/>
+      <c r="M33" s="43"/>
+      <c r="N33" s="43"/>
+      <c r="O33" s="43"/>
       <c r="Q33" s="41"/>
       <c r="R33" s="41"/>
       <c r="S33" s="41"/>
@@ -3097,19 +4451,19 @@
       <c r="B34" s="6" t="str">
         <v>Baseline</v>
       </c>
-      <c r="C34" s="42"/>
-      <c r="D34" s="42"/>
-      <c r="E34" s="42"/>
-      <c r="F34" s="42"/>
-      <c r="G34" s="42"/>
-      <c r="H34" s="42"/>
-      <c r="I34" s="42"/>
-      <c r="J34" s="42"/>
-      <c r="K34" s="42"/>
-      <c r="L34" s="42"/>
-      <c r="M34" s="42"/>
-      <c r="N34" s="42"/>
-      <c r="O34" s="42"/>
+      <c r="C34" s="43"/>
+      <c r="D34" s="43"/>
+      <c r="E34" s="43"/>
+      <c r="F34" s="43"/>
+      <c r="G34" s="43"/>
+      <c r="H34" s="43"/>
+      <c r="I34" s="43"/>
+      <c r="J34" s="43"/>
+      <c r="K34" s="43"/>
+      <c r="L34" s="43"/>
+      <c r="M34" s="43"/>
+      <c r="N34" s="43"/>
+      <c r="O34" s="43"/>
       <c r="Q34" s="41"/>
       <c r="R34" s="41"/>
       <c r="S34" s="41"/>
@@ -3142,21 +4496,21 @@
       <c r="B35" s="6" t="str">
         <v>No_nonDLS_limExt</v>
       </c>
-      <c r="C35" s="42"/>
-      <c r="D35" s="42"/>
-      <c r="E35" s="42"/>
-      <c r="F35" s="42"/>
-      <c r="G35" s="42"/>
-      <c r="H35" s="42"/>
-      <c r="I35" s="42" t="s">
+      <c r="C35" s="43"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="43"/>
+      <c r="H35" s="43"/>
+      <c r="I35" s="43" t="s">
         <v>71</v>
       </c>
-      <c r="J35" s="42"/>
-      <c r="K35" s="42"/>
-      <c r="L35" s="42"/>
-      <c r="M35" s="42"/>
-      <c r="N35" s="42"/>
-      <c r="O35" s="42"/>
+      <c r="J35" s="43"/>
+      <c r="K35" s="43"/>
+      <c r="L35" s="43"/>
+      <c r="M35" s="43"/>
+      <c r="N35" s="43"/>
+      <c r="O35" s="43"/>
       <c r="Q35" s="41"/>
       <c r="R35" s="41"/>
       <c r="S35" s="41"/>
@@ -3189,21 +4543,21 @@
       <c r="B36" s="6" t="str">
         <v>BHN</v>
       </c>
-      <c r="C36" s="46" t="s">
+      <c r="C36" s="47" t="s">
         <v>72</v>
       </c>
-      <c r="D36" s="46"/>
-      <c r="E36" s="46"/>
-      <c r="F36" s="46"/>
-      <c r="G36" s="46"/>
-      <c r="H36" s="46"/>
-      <c r="I36" s="42"/>
-      <c r="J36" s="42"/>
-      <c r="K36" s="42"/>
-      <c r="L36" s="42"/>
-      <c r="M36" s="42"/>
-      <c r="N36" s="42"/>
-      <c r="O36" s="42"/>
+      <c r="D36" s="47"/>
+      <c r="E36" s="47"/>
+      <c r="F36" s="47"/>
+      <c r="G36" s="47"/>
+      <c r="H36" s="47"/>
+      <c r="I36" s="43"/>
+      <c r="J36" s="43"/>
+      <c r="K36" s="43"/>
+      <c r="L36" s="43"/>
+      <c r="M36" s="43"/>
+      <c r="N36" s="43"/>
+      <c r="O36" s="43"/>
       <c r="Q36" s="41"/>
       <c r="R36" s="41"/>
       <c r="S36" s="41"/>
@@ -3542,6 +4896,33 @@
     </row>
   </sheetData>
   <mergeCells count="43">
+    <mergeCell ref="C27:H27"/>
+    <mergeCell ref="I24:O24"/>
+    <mergeCell ref="I25:O25"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="I21:O21"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
+    <mergeCell ref="I22:O22"/>
+    <mergeCell ref="I23:O23"/>
+    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C28:H28"/>
+    <mergeCell ref="I28:O28"/>
+    <mergeCell ref="I29:O29"/>
+    <mergeCell ref="AR22:AY24"/>
+    <mergeCell ref="Q30:AA36"/>
+    <mergeCell ref="AB32:AQ41"/>
+    <mergeCell ref="I26:O26"/>
+    <mergeCell ref="I27:O27"/>
+    <mergeCell ref="I32:O32"/>
+    <mergeCell ref="I33:O33"/>
+    <mergeCell ref="I34:O34"/>
+    <mergeCell ref="AB22:AQ27"/>
+    <mergeCell ref="Q22:AA25"/>
+    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C26:H26"/>
     <mergeCell ref="T4:X4"/>
     <mergeCell ref="AB42:AQ53"/>
     <mergeCell ref="C30:H30"/>
@@ -3558,33 +4939,6 @@
     <mergeCell ref="I31:O31"/>
     <mergeCell ref="C36:H36"/>
     <mergeCell ref="I36:O36"/>
-    <mergeCell ref="C28:H28"/>
-    <mergeCell ref="I28:O28"/>
-    <mergeCell ref="I29:O29"/>
-    <mergeCell ref="AR22:AY24"/>
-    <mergeCell ref="Q30:AA36"/>
-    <mergeCell ref="AB32:AQ41"/>
-    <mergeCell ref="I26:O26"/>
-    <mergeCell ref="I27:O27"/>
-    <mergeCell ref="I32:O32"/>
-    <mergeCell ref="I33:O33"/>
-    <mergeCell ref="I34:O34"/>
-    <mergeCell ref="AB22:AQ27"/>
-    <mergeCell ref="Q22:AA25"/>
-    <mergeCell ref="C24:H24"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C26:H26"/>
-    <mergeCell ref="C27:H27"/>
-    <mergeCell ref="I24:O24"/>
-    <mergeCell ref="I25:O25"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="I21:O21"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C23:H23"/>
-    <mergeCell ref="I22:O22"/>
-    <mergeCell ref="I23:O23"/>
-    <mergeCell ref="C3:H3"/>
-    <mergeCell ref="C21:H21"/>
   </mergeCells>
   <conditionalFormatting sqref="C5:Q15">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
@@ -3618,14 +4972,14 @@
       <c r="B3" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C3" s="34"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="35"/>
-      <c r="G3" s="35"/>
-      <c r="H3" s="38"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="35"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="52"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="52"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="52"/>
       <c r="K3" s="8"/>
       <c r="L3" s="8"/>
       <c r="M3" s="8"/>
@@ -3695,13 +5049,13 @@
       <c r="S4" s="29" t="str">
         <v>All_indicators</v>
       </c>
-      <c r="T4" s="43" t="s">
+      <c r="T4" s="40" t="s">
         <v>75</v>
       </c>
-      <c r="U4" s="43"/>
-      <c r="V4" s="43"/>
-      <c r="W4" s="43"/>
-      <c r="X4" s="43"/>
+      <c r="U4" s="40"/>
+      <c r="V4" s="40"/>
+      <c r="W4" s="40"/>
+      <c r="X4" s="40"/>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B5" s="11" t="str" cm="1">
@@ -4756,23 +6110,23 @@
       <c r="B21" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="36" t="s">
+      <c r="C21" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="36"/>
-      <c r="I21" s="36" t="s">
+      <c r="D21" s="53"/>
+      <c r="E21" s="53"/>
+      <c r="F21" s="53"/>
+      <c r="G21" s="53"/>
+      <c r="H21" s="53"/>
+      <c r="I21" s="53" t="s">
         <v>41</v>
       </c>
-      <c r="J21" s="36"/>
-      <c r="K21" s="36"/>
-      <c r="L21" s="36"/>
-      <c r="M21" s="36"/>
-      <c r="N21" s="36"/>
-      <c r="O21" s="36"/>
+      <c r="J21" s="53"/>
+      <c r="K21" s="53"/>
+      <c r="L21" s="53"/>
+      <c r="M21" s="53"/>
+      <c r="N21" s="53"/>
+      <c r="O21" s="53"/>
       <c r="Q21" s="1" t="s">
         <v>58</v>
       </c>
@@ -4788,21 +6142,21 @@
         <f t="array" ref="B22:B38">TRANSPOSE(_xlfn.ANCHORARRAY(C4))</f>
         <v>BHN_FWB</v>
       </c>
-      <c r="C22" s="37" t="s">
+      <c r="C22" s="49" t="s">
         <v>43</v>
       </c>
-      <c r="D22" s="37"/>
-      <c r="E22" s="37"/>
-      <c r="F22" s="37"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="37"/>
-      <c r="I22" s="33"/>
-      <c r="J22" s="33"/>
-      <c r="K22" s="33"/>
-      <c r="L22" s="33"/>
-      <c r="M22" s="33"/>
-      <c r="N22" s="33"/>
-      <c r="O22" s="33"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="49"/>
+      <c r="I22" s="48"/>
+      <c r="J22" s="48"/>
+      <c r="K22" s="48"/>
+      <c r="L22" s="48"/>
+      <c r="M22" s="48"/>
+      <c r="N22" s="48"/>
+      <c r="O22" s="48"/>
       <c r="Q22" s="41" t="e" vm="9">
         <v>#VALUE!</v>
       </c>
@@ -4852,21 +6206,21 @@
       <c r="B23" s="26" t="str">
         <v>BHN_FWB_AllExt</v>
       </c>
-      <c r="C23" s="50" t="s">
+      <c r="C23" s="57" t="s">
         <v>42</v>
       </c>
-      <c r="D23" s="50"/>
-      <c r="E23" s="50"/>
-      <c r="F23" s="50"/>
-      <c r="G23" s="50"/>
-      <c r="H23" s="50"/>
-      <c r="I23" s="33"/>
-      <c r="J23" s="33"/>
-      <c r="K23" s="33"/>
-      <c r="L23" s="33"/>
-      <c r="M23" s="33"/>
-      <c r="N23" s="33"/>
-      <c r="O23" s="33"/>
+      <c r="D23" s="57"/>
+      <c r="E23" s="57"/>
+      <c r="F23" s="57"/>
+      <c r="G23" s="57"/>
+      <c r="H23" s="57"/>
+      <c r="I23" s="48"/>
+      <c r="J23" s="48"/>
+      <c r="K23" s="48"/>
+      <c r="L23" s="48"/>
+      <c r="M23" s="48"/>
+      <c r="N23" s="48"/>
+      <c r="O23" s="48"/>
       <c r="Q23" s="41"/>
       <c r="R23" s="41"/>
       <c r="S23" s="41"/>
@@ -4910,21 +6264,21 @@
       <c r="B24" s="7" t="str">
         <v>Few_indicators_closest_DLS_coverage</v>
       </c>
-      <c r="C24" s="37" t="s">
+      <c r="C24" s="49" t="s">
         <v>46</v>
       </c>
-      <c r="D24" s="37"/>
-      <c r="E24" s="37"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="37"/>
-      <c r="I24" s="33"/>
-      <c r="J24" s="33"/>
-      <c r="K24" s="33"/>
-      <c r="L24" s="33"/>
-      <c r="M24" s="33"/>
-      <c r="N24" s="33"/>
-      <c r="O24" s="33"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="49"/>
+      <c r="I24" s="48"/>
+      <c r="J24" s="48"/>
+      <c r="K24" s="48"/>
+      <c r="L24" s="48"/>
+      <c r="M24" s="48"/>
+      <c r="N24" s="48"/>
+      <c r="O24" s="48"/>
       <c r="Q24" s="41"/>
       <c r="R24" s="41"/>
       <c r="S24" s="41"/>
@@ -4968,21 +6322,21 @@
       <c r="B25" s="7" t="str">
         <v>Few_indicators_SPI_preferred</v>
       </c>
-      <c r="C25" s="37" t="s">
+      <c r="C25" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="D25" s="37"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="37"/>
-      <c r="G25" s="37"/>
-      <c r="H25" s="37"/>
-      <c r="I25" s="33"/>
-      <c r="J25" s="33"/>
-      <c r="K25" s="33"/>
-      <c r="L25" s="33"/>
-      <c r="M25" s="33"/>
-      <c r="N25" s="33"/>
-      <c r="O25" s="33"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="49"/>
+      <c r="I25" s="48"/>
+      <c r="J25" s="48"/>
+      <c r="K25" s="48"/>
+      <c r="L25" s="48"/>
+      <c r="M25" s="48"/>
+      <c r="N25" s="48"/>
+      <c r="O25" s="48"/>
       <c r="AB25" s="41"/>
       <c r="AC25" s="41"/>
       <c r="AD25" s="41"/>
@@ -5007,21 +6361,21 @@
       <c r="B26" s="7" t="str">
         <v>No_non_DLS</v>
       </c>
-      <c r="C26" s="32" t="s">
+      <c r="C26" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="32"/>
-      <c r="I26" s="33"/>
-      <c r="J26" s="33"/>
-      <c r="K26" s="33"/>
-      <c r="L26" s="33"/>
-      <c r="M26" s="33"/>
-      <c r="N26" s="33"/>
-      <c r="O26" s="33"/>
+      <c r="D26" s="50"/>
+      <c r="E26" s="50"/>
+      <c r="F26" s="50"/>
+      <c r="G26" s="50"/>
+      <c r="H26" s="50"/>
+      <c r="I26" s="48"/>
+      <c r="J26" s="48"/>
+      <c r="K26" s="48"/>
+      <c r="L26" s="48"/>
+      <c r="M26" s="48"/>
+      <c r="N26" s="48"/>
+      <c r="O26" s="48"/>
       <c r="Q26" s="41"/>
       <c r="R26" s="41"/>
       <c r="S26" s="41"/>
@@ -5057,21 +6411,21 @@
       <c r="B27" s="26" t="str">
         <v>Only_%_of_pop</v>
       </c>
-      <c r="C27" s="51" t="s">
+      <c r="C27" s="55" t="s">
         <v>50</v>
       </c>
-      <c r="D27" s="51"/>
-      <c r="E27" s="51"/>
-      <c r="F27" s="51"/>
-      <c r="G27" s="51"/>
-      <c r="H27" s="51"/>
-      <c r="I27" s="33"/>
-      <c r="J27" s="33"/>
-      <c r="K27" s="33"/>
-      <c r="L27" s="33"/>
-      <c r="M27" s="33"/>
-      <c r="N27" s="33"/>
-      <c r="O27" s="33"/>
+      <c r="D27" s="55"/>
+      <c r="E27" s="55"/>
+      <c r="F27" s="55"/>
+      <c r="G27" s="55"/>
+      <c r="H27" s="55"/>
+      <c r="I27" s="48"/>
+      <c r="J27" s="48"/>
+      <c r="K27" s="48"/>
+      <c r="L27" s="48"/>
+      <c r="M27" s="48"/>
+      <c r="N27" s="48"/>
+      <c r="O27" s="48"/>
       <c r="Q27" s="41"/>
       <c r="R27" s="41"/>
       <c r="S27" s="41"/>
@@ -5107,21 +6461,21 @@
       <c r="B28" s="17" t="str">
         <v>Few_indicators_closest_DLS_coverage_90</v>
       </c>
-      <c r="C28" s="39" t="s">
+      <c r="C28" s="44" t="s">
         <v>60</v>
       </c>
-      <c r="D28" s="39"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="39"/>
-      <c r="H28" s="39"/>
-      <c r="I28" s="40"/>
-      <c r="J28" s="40"/>
-      <c r="K28" s="40"/>
-      <c r="L28" s="40"/>
-      <c r="M28" s="40"/>
-      <c r="N28" s="40"/>
-      <c r="O28" s="40"/>
+      <c r="D28" s="44"/>
+      <c r="E28" s="44"/>
+      <c r="F28" s="44"/>
+      <c r="G28" s="44"/>
+      <c r="H28" s="44"/>
+      <c r="I28" s="46"/>
+      <c r="J28" s="46"/>
+      <c r="K28" s="46"/>
+      <c r="L28" s="46"/>
+      <c r="M28" s="46"/>
+      <c r="N28" s="46"/>
+      <c r="O28" s="46"/>
       <c r="Q28" s="41"/>
       <c r="R28" s="41"/>
       <c r="S28" s="41"/>
@@ -5157,21 +6511,21 @@
       <c r="B29" s="17" t="str">
         <v>Few_indicators_SPI_preferred_90</v>
       </c>
-      <c r="C29" s="39" t="s">
+      <c r="C29" s="44" t="s">
         <v>60</v>
       </c>
-      <c r="D29" s="39"/>
-      <c r="E29" s="39"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="39"/>
-      <c r="H29" s="39"/>
-      <c r="I29" s="40"/>
-      <c r="J29" s="40"/>
-      <c r="K29" s="40"/>
-      <c r="L29" s="40"/>
-      <c r="M29" s="40"/>
-      <c r="N29" s="40"/>
-      <c r="O29" s="40"/>
+      <c r="D29" s="44"/>
+      <c r="E29" s="44"/>
+      <c r="F29" s="44"/>
+      <c r="G29" s="44"/>
+      <c r="H29" s="44"/>
+      <c r="I29" s="46"/>
+      <c r="J29" s="46"/>
+      <c r="K29" s="46"/>
+      <c r="L29" s="46"/>
+      <c r="M29" s="46"/>
+      <c r="N29" s="46"/>
+      <c r="O29" s="46"/>
       <c r="Q29" s="41"/>
       <c r="R29" s="41"/>
       <c r="S29" s="41"/>
@@ -5207,21 +6561,21 @@
       <c r="B30" s="17" t="str">
         <v>Few_indicators_closeDLS_subPrimSchool</v>
       </c>
-      <c r="C30" s="44" t="s">
+      <c r="C30" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="D30" s="44"/>
-      <c r="E30" s="44"/>
-      <c r="F30" s="44"/>
-      <c r="G30" s="44"/>
-      <c r="H30" s="44"/>
-      <c r="I30" s="40"/>
-      <c r="J30" s="40"/>
-      <c r="K30" s="40"/>
-      <c r="L30" s="40"/>
-      <c r="M30" s="40"/>
-      <c r="N30" s="40"/>
-      <c r="O30" s="40"/>
+      <c r="D30" s="42"/>
+      <c r="E30" s="42"/>
+      <c r="F30" s="42"/>
+      <c r="G30" s="42"/>
+      <c r="H30" s="42"/>
+      <c r="I30" s="46"/>
+      <c r="J30" s="46"/>
+      <c r="K30" s="46"/>
+      <c r="L30" s="46"/>
+      <c r="M30" s="46"/>
+      <c r="N30" s="46"/>
+      <c r="O30" s="46"/>
       <c r="Q30" s="41"/>
       <c r="R30" s="41"/>
       <c r="S30" s="41"/>
@@ -5257,23 +6611,23 @@
       <c r="B31" s="27" t="str">
         <v>No_non_DLS_90</v>
       </c>
-      <c r="C31" s="47" t="s">
+      <c r="C31" s="58" t="s">
         <v>60</v>
       </c>
-      <c r="D31" s="47"/>
-      <c r="E31" s="47"/>
-      <c r="F31" s="47"/>
-      <c r="G31" s="47"/>
-      <c r="H31" s="47"/>
-      <c r="I31" s="47" t="s">
+      <c r="D31" s="58"/>
+      <c r="E31" s="58"/>
+      <c r="F31" s="58"/>
+      <c r="G31" s="58"/>
+      <c r="H31" s="58"/>
+      <c r="I31" s="58" t="s">
         <v>74</v>
       </c>
-      <c r="J31" s="47"/>
-      <c r="K31" s="47"/>
-      <c r="L31" s="47"/>
-      <c r="M31" s="47"/>
-      <c r="N31" s="47"/>
-      <c r="O31" s="47"/>
+      <c r="J31" s="58"/>
+      <c r="K31" s="58"/>
+      <c r="L31" s="58"/>
+      <c r="M31" s="58"/>
+      <c r="N31" s="58"/>
+      <c r="O31" s="58"/>
       <c r="Q31" s="41"/>
       <c r="R31" s="41"/>
       <c r="S31" s="41"/>
@@ -5309,21 +6663,21 @@
       <c r="B32" s="27" t="str">
         <v>Few_Indicators_subWatSani</v>
       </c>
-      <c r="C32" s="47" t="s">
+      <c r="C32" s="58" t="s">
         <v>65</v>
       </c>
-      <c r="D32" s="47"/>
-      <c r="E32" s="47"/>
-      <c r="F32" s="47"/>
-      <c r="G32" s="47"/>
-      <c r="H32" s="47"/>
-      <c r="I32" s="40"/>
-      <c r="J32" s="40"/>
-      <c r="K32" s="40"/>
-      <c r="L32" s="40"/>
-      <c r="M32" s="40"/>
-      <c r="N32" s="40"/>
-      <c r="O32" s="40"/>
+      <c r="D32" s="58"/>
+      <c r="E32" s="58"/>
+      <c r="F32" s="58"/>
+      <c r="G32" s="58"/>
+      <c r="H32" s="58"/>
+      <c r="I32" s="46"/>
+      <c r="J32" s="46"/>
+      <c r="K32" s="46"/>
+      <c r="L32" s="46"/>
+      <c r="M32" s="46"/>
+      <c r="N32" s="46"/>
+      <c r="O32" s="46"/>
       <c r="Q32" s="41"/>
       <c r="R32" s="41"/>
       <c r="S32" s="41"/>
@@ -5359,21 +6713,21 @@
       <c r="B33" s="28" t="str">
         <v>Only_OPP</v>
       </c>
-      <c r="C33" s="48" t="s">
+      <c r="C33" s="59" t="s">
         <v>68</v>
       </c>
-      <c r="D33" s="48"/>
-      <c r="E33" s="48"/>
-      <c r="F33" s="48"/>
-      <c r="G33" s="48"/>
-      <c r="H33" s="48"/>
-      <c r="I33" s="42"/>
-      <c r="J33" s="42"/>
-      <c r="K33" s="42"/>
-      <c r="L33" s="42"/>
-      <c r="M33" s="42"/>
-      <c r="N33" s="42"/>
-      <c r="O33" s="42"/>
+      <c r="D33" s="59"/>
+      <c r="E33" s="59"/>
+      <c r="F33" s="59"/>
+      <c r="G33" s="59"/>
+      <c r="H33" s="59"/>
+      <c r="I33" s="43"/>
+      <c r="J33" s="43"/>
+      <c r="K33" s="43"/>
+      <c r="L33" s="43"/>
+      <c r="M33" s="43"/>
+      <c r="N33" s="43"/>
+      <c r="O33" s="43"/>
       <c r="Q33" s="41"/>
       <c r="R33" s="41"/>
       <c r="S33" s="41"/>
@@ -5406,19 +6760,19 @@
       <c r="B34" s="6" t="str">
         <v>Baseline</v>
       </c>
-      <c r="C34" s="42"/>
-      <c r="D34" s="42"/>
-      <c r="E34" s="42"/>
-      <c r="F34" s="42"/>
-      <c r="G34" s="42"/>
-      <c r="H34" s="42"/>
-      <c r="I34" s="42"/>
-      <c r="J34" s="42"/>
-      <c r="K34" s="42"/>
-      <c r="L34" s="42"/>
-      <c r="M34" s="42"/>
-      <c r="N34" s="42"/>
-      <c r="O34" s="42"/>
+      <c r="C34" s="43"/>
+      <c r="D34" s="43"/>
+      <c r="E34" s="43"/>
+      <c r="F34" s="43"/>
+      <c r="G34" s="43"/>
+      <c r="H34" s="43"/>
+      <c r="I34" s="43"/>
+      <c r="J34" s="43"/>
+      <c r="K34" s="43"/>
+      <c r="L34" s="43"/>
+      <c r="M34" s="43"/>
+      <c r="N34" s="43"/>
+      <c r="O34" s="43"/>
       <c r="Q34" s="41"/>
       <c r="R34" s="41"/>
       <c r="S34" s="41"/>
@@ -5451,21 +6805,21 @@
       <c r="B35" s="28" t="str">
         <v>No_nonDLS_limExt</v>
       </c>
-      <c r="C35" s="49"/>
-      <c r="D35" s="49"/>
-      <c r="E35" s="49"/>
-      <c r="F35" s="49"/>
-      <c r="G35" s="49"/>
-      <c r="H35" s="49"/>
-      <c r="I35" s="49" t="s">
+      <c r="C35" s="56"/>
+      <c r="D35" s="56"/>
+      <c r="E35" s="56"/>
+      <c r="F35" s="56"/>
+      <c r="G35" s="56"/>
+      <c r="H35" s="56"/>
+      <c r="I35" s="56" t="s">
         <v>71</v>
       </c>
-      <c r="J35" s="49"/>
-      <c r="K35" s="49"/>
-      <c r="L35" s="49"/>
-      <c r="M35" s="49"/>
-      <c r="N35" s="49"/>
-      <c r="O35" s="49"/>
+      <c r="J35" s="56"/>
+      <c r="K35" s="56"/>
+      <c r="L35" s="56"/>
+      <c r="M35" s="56"/>
+      <c r="N35" s="56"/>
+      <c r="O35" s="56"/>
       <c r="Q35" s="41"/>
       <c r="R35" s="41"/>
       <c r="S35" s="41"/>
@@ -5498,21 +6852,21 @@
       <c r="B36" s="6" t="str">
         <v>BHN</v>
       </c>
-      <c r="C36" s="46" t="s">
+      <c r="C36" s="47" t="s">
         <v>72</v>
       </c>
-      <c r="D36" s="46"/>
-      <c r="E36" s="46"/>
-      <c r="F36" s="46"/>
-      <c r="G36" s="46"/>
-      <c r="H36" s="46"/>
-      <c r="I36" s="42"/>
-      <c r="J36" s="42"/>
-      <c r="K36" s="42"/>
-      <c r="L36" s="42"/>
-      <c r="M36" s="42"/>
-      <c r="N36" s="42"/>
-      <c r="O36" s="42"/>
+      <c r="D36" s="47"/>
+      <c r="E36" s="47"/>
+      <c r="F36" s="47"/>
+      <c r="G36" s="47"/>
+      <c r="H36" s="47"/>
+      <c r="I36" s="43"/>
+      <c r="J36" s="43"/>
+      <c r="K36" s="43"/>
+      <c r="L36" s="43"/>
+      <c r="M36" s="43"/>
+      <c r="N36" s="43"/>
+      <c r="O36" s="43"/>
       <c r="Q36" s="41"/>
       <c r="R36" s="41"/>
       <c r="S36" s="41"/>
@@ -5857,16 +7211,22 @@
     </row>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="C27:H27"/>
-    <mergeCell ref="I27:O27"/>
-    <mergeCell ref="C28:H28"/>
-    <mergeCell ref="I28:O28"/>
-    <mergeCell ref="C3:H3"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="I21:O21"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="I22:O22"/>
+    <mergeCell ref="AB42:AQ53"/>
+    <mergeCell ref="T4:X4"/>
+    <mergeCell ref="AB32:AQ41"/>
+    <mergeCell ref="Q30:AA36"/>
+    <mergeCell ref="C36:H36"/>
+    <mergeCell ref="I36:O36"/>
+    <mergeCell ref="C29:H29"/>
+    <mergeCell ref="I29:O29"/>
+    <mergeCell ref="C30:H30"/>
+    <mergeCell ref="I30:O30"/>
+    <mergeCell ref="C31:H31"/>
+    <mergeCell ref="I31:O31"/>
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="I32:O32"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="I33:O33"/>
     <mergeCell ref="C34:H34"/>
     <mergeCell ref="I34:O34"/>
     <mergeCell ref="C35:H35"/>
@@ -5883,22 +7243,16 @@
     <mergeCell ref="C26:H26"/>
     <mergeCell ref="I26:O26"/>
     <mergeCell ref="Q26:AA29"/>
-    <mergeCell ref="AB42:AQ53"/>
-    <mergeCell ref="T4:X4"/>
-    <mergeCell ref="AB32:AQ41"/>
-    <mergeCell ref="Q30:AA36"/>
-    <mergeCell ref="C36:H36"/>
-    <mergeCell ref="I36:O36"/>
-    <mergeCell ref="C29:H29"/>
-    <mergeCell ref="I29:O29"/>
-    <mergeCell ref="C30:H30"/>
-    <mergeCell ref="I30:O30"/>
-    <mergeCell ref="C31:H31"/>
-    <mergeCell ref="I31:O31"/>
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="I32:O32"/>
-    <mergeCell ref="C33:H33"/>
-    <mergeCell ref="I33:O33"/>
+    <mergeCell ref="C27:H27"/>
+    <mergeCell ref="I27:O27"/>
+    <mergeCell ref="C28:H28"/>
+    <mergeCell ref="I28:O28"/>
+    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="I21:O21"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="I22:O22"/>
   </mergeCells>
   <conditionalFormatting sqref="C5:S15">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
@@ -9722,14 +11076,16 @@
   <sheetPr>
     <tabColor theme="2" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A3:D67"/>
+  <dimension ref="A3:F67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="61.7109375" customWidth="1"/>
     <col min="3" max="3" width="22.140625" customWidth="1"/>
+    <col min="6" max="6" width="24.5703125" customWidth="1"/>
+    <col min="7" max="7" width="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -9740,7 +11096,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -9751,72 +11107,81 @@
       <c r="C4" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F4" s="60"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="str">
         <v>Deaths from infectious diseases (deaths/100,000)</v>
       </c>
       <c r="C5" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F5" s="60"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="str">
         <v xml:space="preserve">Maternal mortality  (deaths/100,000 live births) </v>
       </c>
       <c r="C6" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F6" s="60"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="str">
         <v xml:space="preserve">Nutritional deficiencies (% of pop.) </v>
       </c>
       <c r="C7" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F7" s="60"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="str">
         <v xml:space="preserve">Diet low in fruits and vegetables (0=low risk; 100=high risk) </v>
       </c>
       <c r="C8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F8" s="60"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="str">
         <v xml:space="preserve">Child mortality (deaths/1,000 live births) </v>
       </c>
       <c r="C9" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F9" s="60"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="str">
         <v xml:space="preserve">No access to a handwashing facility (0=low risk; 100=high risk) </v>
       </c>
       <c r="C10" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F10" s="60"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="str">
         <v>Deaths from unsafe water, sanitation and hygiene (deaths/100,000)</v>
       </c>
       <c r="C11" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F11" s="60"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="str">
         <v xml:space="preserve">Improved sanitation (proportion of pop.) </v>
       </c>
       <c r="C12" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F12" s="60"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="str">
         <v xml:space="preserve">Improved water source (proportion of pop.) </v>
       </c>
@@ -9824,7 +11189,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -9835,7 +11200,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="str">
         <v xml:space="preserve">Prevalence of cooking with coal/biomass (proportion of pop.) </v>
       </c>
@@ -9843,7 +11208,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="str">
         <v xml:space="preserve">Access to electricity (% of pop.) </v>
       </c>
@@ -10280,45 +11645,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="127.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="54" t="s">
+      <c r="B1" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="C1" s="54" t="s">
+      <c r="C1" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="D1" s="54" t="s">
+      <c r="D1" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="E1" s="54" t="s">
+      <c r="E1" s="34" t="s">
         <v>81</v>
       </c>
-      <c r="F1" s="54" t="s">
+      <c r="F1" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="G1" s="54" t="s">
+      <c r="G1" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="H1" s="54" t="s">
+      <c r="H1" s="34" t="s">
         <v>84</v>
       </c>
-      <c r="I1" s="54" t="s">
+      <c r="I1" s="34" t="s">
         <v>85</v>
       </c>
-      <c r="J1" s="54" t="s">
+      <c r="J1" s="34" t="s">
         <v>86</v>
       </c>
-      <c r="K1" s="54" t="s">
+      <c r="K1" s="34" t="s">
         <v>87</v>
       </c>
-      <c r="M1" s="52"/>
-      <c r="N1" s="52"/>
-      <c r="P1" s="52"/>
+      <c r="M1" s="32"/>
+      <c r="N1" s="32"/>
+      <c r="P1" s="32"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="56" t="s">
+      <c r="A2" s="36" t="s">
         <v>18</v>
       </c>
       <c r="B2" s="31">
@@ -10353,7 +11718,7 @@
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="36" t="s">
         <v>25</v>
       </c>
       <c r="B3" s="31">
@@ -10388,7 +11753,7 @@
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="56" t="s">
+      <c r="A4" s="36" t="s">
         <v>22</v>
       </c>
       <c r="B4" s="31">
@@ -10423,7 +11788,7 @@
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="56" t="s">
+      <c r="A5" s="36" t="s">
         <v>24</v>
       </c>
       <c r="B5" s="31">
@@ -10462,7 +11827,7 @@
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="56" t="s">
+      <c r="A6" s="36" t="s">
         <v>21</v>
       </c>
       <c r="B6" s="31">
@@ -10500,7 +11865,7 @@
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="56" t="s">
+      <c r="A7" s="36" t="s">
         <v>20</v>
       </c>
       <c r="B7" s="31">
@@ -10538,7 +11903,7 @@
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="56" t="s">
+      <c r="A8" s="36" t="s">
         <v>23</v>
       </c>
       <c r="B8" s="31">
@@ -10576,7 +11941,7 @@
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="56" t="s">
+      <c r="A9" s="36" t="s">
         <v>26</v>
       </c>
       <c r="B9" s="31">
@@ -10614,7 +11979,7 @@
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="56" t="s">
+      <c r="A10" s="36" t="s">
         <v>19</v>
       </c>
       <c r="B10" s="31">
@@ -10652,37 +12017,37 @@
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="56" t="s">
+      <c r="A11" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="59">
-        <v>0</v>
-      </c>
-      <c r="C11" s="59">
-        <v>0</v>
-      </c>
-      <c r="D11" s="59">
-        <v>0</v>
-      </c>
-      <c r="E11" s="59">
-        <v>0</v>
-      </c>
-      <c r="F11" s="59">
-        <v>0</v>
-      </c>
-      <c r="G11" s="59">
-        <v>0</v>
-      </c>
-      <c r="H11" s="59">
-        <v>0</v>
-      </c>
-      <c r="I11" s="59">
-        <v>0</v>
-      </c>
-      <c r="J11" s="59">
-        <v>0</v>
-      </c>
-      <c r="K11" s="59">
+      <c r="B11" s="31">
+        <v>0</v>
+      </c>
+      <c r="C11" s="31">
+        <v>0</v>
+      </c>
+      <c r="D11" s="31">
+        <v>0</v>
+      </c>
+      <c r="E11" s="31">
+        <v>0</v>
+      </c>
+      <c r="F11" s="31">
+        <v>0</v>
+      </c>
+      <c r="G11" s="31">
+        <v>0</v>
+      </c>
+      <c r="H11" s="31">
+        <v>0</v>
+      </c>
+      <c r="I11" s="31">
+        <v>0</v>
+      </c>
+      <c r="J11" s="31">
+        <v>0</v>
+      </c>
+      <c r="K11" s="31">
         <v>0</v>
       </c>
       <c r="P11" t="str">
@@ -10690,37 +12055,37 @@
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A12" s="57" t="s">
+      <c r="A12" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="53">
+      <c r="B12" s="33">
         <v>24</v>
       </c>
-      <c r="C12" s="53">
+      <c r="C12" s="33">
         <v>9</v>
       </c>
-      <c r="D12" s="53">
+      <c r="D12" s="33">
         <v>25</v>
       </c>
-      <c r="E12" s="53">
-        <v>0</v>
-      </c>
-      <c r="F12" s="53">
-        <v>0</v>
-      </c>
-      <c r="G12" s="53">
-        <v>0</v>
-      </c>
-      <c r="H12" s="53">
-        <v>0</v>
-      </c>
-      <c r="I12" s="53">
-        <v>0</v>
-      </c>
-      <c r="J12" s="53">
-        <v>0</v>
-      </c>
-      <c r="K12" s="53">
+      <c r="E12" s="33">
+        <v>0</v>
+      </c>
+      <c r="F12" s="33">
+        <v>0</v>
+      </c>
+      <c r="G12" s="33">
+        <v>0</v>
+      </c>
+      <c r="H12" s="33">
+        <v>0</v>
+      </c>
+      <c r="I12" s="33">
+        <v>0</v>
+      </c>
+      <c r="J12" s="33">
+        <v>0</v>
+      </c>
+      <c r="K12" s="33">
         <v>0</v>
       </c>
       <c r="P12" t="str">
@@ -10728,37 +12093,37 @@
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" s="58" t="s">
+      <c r="A13" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="60">
+      <c r="B13" s="39">
         <v>52</v>
       </c>
-      <c r="C13" s="60">
+      <c r="C13" s="39">
         <v>33</v>
       </c>
-      <c r="D13" s="60">
+      <c r="D13" s="39">
         <v>62</v>
       </c>
-      <c r="E13" s="60">
+      <c r="E13" s="39">
         <v>37</v>
       </c>
-      <c r="F13" s="60">
+      <c r="F13" s="39">
         <v>29</v>
       </c>
-      <c r="G13" s="60">
+      <c r="G13" s="39">
         <v>33</v>
       </c>
-      <c r="H13" s="60">
+      <c r="H13" s="39">
         <v>11</v>
       </c>
-      <c r="I13" s="60">
+      <c r="I13" s="39">
         <v>11</v>
       </c>
-      <c r="J13" s="60">
+      <c r="J13" s="39">
         <v>11</v>
       </c>
-      <c r="K13" s="60">
+      <c r="K13" s="39">
         <v>11</v>
       </c>
       <c r="P13" t="str">
@@ -10766,7 +12131,7 @@
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" s="56" t="s">
+      <c r="A14" s="36" t="s">
         <v>34</v>
       </c>
       <c r="B14" s="31">
@@ -10804,7 +12169,7 @@
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" s="56" t="s">
+      <c r="A15" s="36" t="s">
         <v>35</v>
       </c>
       <c r="B15" s="31">
@@ -10859,4 +12224,1262 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C45A346D-1A16-4F68-93D6-C1A89543708A}">
+  <dimension ref="A1:H72"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.28515625" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" style="31" customWidth="1"/>
+    <col min="3" max="3" width="71" customWidth="1"/>
+    <col min="4" max="4" width="34" customWidth="1"/>
+    <col min="6" max="6" width="24.28515625" style="31" customWidth="1"/>
+    <col min="7" max="7" width="32" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="68" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" s="68" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" s="68" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" s="68" t="s">
+        <v>98</v>
+      </c>
+      <c r="E1" s="68" t="s">
+        <v>139</v>
+      </c>
+      <c r="F1" s="66" t="s">
+        <v>161</v>
+      </c>
+      <c r="G1" s="61" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="69">
+        <v>1</v>
+      </c>
+      <c r="B2" s="68" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="70" t="s">
+        <v>143</v>
+      </c>
+      <c r="D2" s="71" t="s">
+        <v>165</v>
+      </c>
+      <c r="E2" s="71" t="s">
+        <v>140</v>
+      </c>
+      <c r="F2" s="78" t="s">
+        <v>162</v>
+      </c>
+      <c r="G2" t="s">
+        <v>152</v>
+      </c>
+      <c r="H2" s="67" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A3" s="69">
+        <v>2</v>
+      </c>
+      <c r="B3" s="68" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="70" t="s">
+        <v>142</v>
+      </c>
+      <c r="D3" s="71" t="s">
+        <v>99</v>
+      </c>
+      <c r="E3" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F3" s="78" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="72">
+        <v>3</v>
+      </c>
+      <c r="B4" s="73" t="s">
+        <v>91</v>
+      </c>
+      <c r="C4" s="74" t="s">
+        <v>141</v>
+      </c>
+      <c r="D4" s="71" t="s">
+        <v>135</v>
+      </c>
+      <c r="E4" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F4" s="79" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="72"/>
+      <c r="B5" s="73"/>
+      <c r="C5" s="74"/>
+      <c r="D5" s="71" t="s">
+        <v>101</v>
+      </c>
+      <c r="E5" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F5" s="79"/>
+    </row>
+    <row r="6" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="72"/>
+      <c r="B6" s="73"/>
+      <c r="C6" s="74"/>
+      <c r="D6" s="71" t="s">
+        <v>102</v>
+      </c>
+      <c r="E6" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F6" s="79"/>
+    </row>
+    <row r="7" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="72"/>
+      <c r="B7" s="73"/>
+      <c r="C7" s="74"/>
+      <c r="D7" s="71" t="s">
+        <v>103</v>
+      </c>
+      <c r="E7" s="71" t="s">
+        <v>146</v>
+      </c>
+      <c r="F7" s="79"/>
+    </row>
+    <row r="8" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="72"/>
+      <c r="B8" s="73"/>
+      <c r="C8" s="74"/>
+      <c r="D8" s="71" t="s">
+        <v>104</v>
+      </c>
+      <c r="E8" s="71" t="s">
+        <v>146</v>
+      </c>
+      <c r="F8" s="79"/>
+    </row>
+    <row r="9" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="72">
+        <v>4</v>
+      </c>
+      <c r="B9" s="73" t="s">
+        <v>92</v>
+      </c>
+      <c r="C9" s="74" t="s">
+        <v>144</v>
+      </c>
+      <c r="D9" s="71" t="s">
+        <v>105</v>
+      </c>
+      <c r="E9" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F9" s="79" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="72"/>
+      <c r="B10" s="73"/>
+      <c r="C10" s="74"/>
+      <c r="D10" s="71" t="s">
+        <v>106</v>
+      </c>
+      <c r="E10" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F10" s="79"/>
+    </row>
+    <row r="11" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="72"/>
+      <c r="B11" s="73"/>
+      <c r="C11" s="74"/>
+      <c r="D11" s="71" t="s">
+        <v>107</v>
+      </c>
+      <c r="E11" s="71" t="s">
+        <v>158</v>
+      </c>
+      <c r="F11" s="79"/>
+      <c r="G11" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="72">
+        <v>5</v>
+      </c>
+      <c r="B12" s="73" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="74" t="s">
+        <v>93</v>
+      </c>
+      <c r="D12" s="71" t="s">
+        <v>108</v>
+      </c>
+      <c r="E12" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F12" s="79" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="72"/>
+      <c r="B13" s="73"/>
+      <c r="C13" s="74"/>
+      <c r="D13" s="71" t="s">
+        <v>109</v>
+      </c>
+      <c r="E13" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F13" s="79"/>
+    </row>
+    <row r="14" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="72"/>
+      <c r="B14" s="73"/>
+      <c r="C14" s="74"/>
+      <c r="D14" s="71" t="s">
+        <v>110</v>
+      </c>
+      <c r="E14" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F14" s="79"/>
+    </row>
+    <row r="15" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A15" s="72"/>
+      <c r="B15" s="73"/>
+      <c r="C15" s="74"/>
+      <c r="D15" s="71" t="s">
+        <v>111</v>
+      </c>
+      <c r="E15" s="71" t="s">
+        <v>155</v>
+      </c>
+      <c r="F15" s="79"/>
+      <c r="G15" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="72">
+        <v>6</v>
+      </c>
+      <c r="B16" s="73" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="74" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" s="71" t="s">
+        <v>112</v>
+      </c>
+      <c r="E16" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F16" s="79" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A17" s="72"/>
+      <c r="B17" s="73"/>
+      <c r="C17" s="74"/>
+      <c r="D17" s="71" t="s">
+        <v>113</v>
+      </c>
+      <c r="E17" s="71" t="s">
+        <v>155</v>
+      </c>
+      <c r="F17" s="79"/>
+      <c r="G17" s="77" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="72">
+        <v>7</v>
+      </c>
+      <c r="B18" s="73" t="s">
+        <v>95</v>
+      </c>
+      <c r="C18" s="74" t="s">
+        <v>96</v>
+      </c>
+      <c r="D18" s="71" t="s">
+        <v>114</v>
+      </c>
+      <c r="E18" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F18" s="79" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="72"/>
+      <c r="B19" s="73"/>
+      <c r="C19" s="74"/>
+      <c r="D19" s="71" t="s">
+        <v>115</v>
+      </c>
+      <c r="E19" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F19" s="79"/>
+    </row>
+    <row r="20" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="72"/>
+      <c r="B20" s="73"/>
+      <c r="C20" s="74"/>
+      <c r="D20" s="71" t="s">
+        <v>116</v>
+      </c>
+      <c r="E20" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F20" s="79"/>
+    </row>
+    <row r="21" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="72"/>
+      <c r="B21" s="73"/>
+      <c r="C21" s="74"/>
+      <c r="D21" s="71" t="s">
+        <v>117</v>
+      </c>
+      <c r="E21" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F21" s="79"/>
+    </row>
+    <row r="22" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="72"/>
+      <c r="B22" s="73"/>
+      <c r="C22" s="74"/>
+      <c r="D22" s="71" t="s">
+        <v>118</v>
+      </c>
+      <c r="E22" s="71" t="s">
+        <v>160</v>
+      </c>
+      <c r="F22" s="79"/>
+      <c r="G22" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A23" s="72"/>
+      <c r="B23" s="73"/>
+      <c r="C23" s="74"/>
+      <c r="D23" s="71" t="s">
+        <v>119</v>
+      </c>
+      <c r="E23" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F23" s="79"/>
+    </row>
+    <row r="24" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="72"/>
+      <c r="B24" s="73"/>
+      <c r="C24" s="74"/>
+      <c r="D24" s="71" t="s">
+        <v>120</v>
+      </c>
+      <c r="E24" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F24" s="79"/>
+    </row>
+    <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="72"/>
+      <c r="B25" s="73"/>
+      <c r="C25" s="74"/>
+      <c r="D25" s="71" t="s">
+        <v>121</v>
+      </c>
+      <c r="E25" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F25" s="79"/>
+    </row>
+    <row r="26" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A26" s="72"/>
+      <c r="B26" s="73"/>
+      <c r="C26" s="74"/>
+      <c r="D26" s="71" t="s">
+        <v>122</v>
+      </c>
+      <c r="E26" s="71" t="s">
+        <v>147</v>
+      </c>
+      <c r="F26" s="79"/>
+      <c r="G26" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A27" s="72"/>
+      <c r="B27" s="73"/>
+      <c r="C27" s="74"/>
+      <c r="D27" s="71" t="s">
+        <v>123</v>
+      </c>
+      <c r="E27" s="71" t="s">
+        <v>147</v>
+      </c>
+      <c r="F27" s="79"/>
+      <c r="G27" s="76" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="72">
+        <v>8</v>
+      </c>
+      <c r="B28" s="73" t="s">
+        <v>23</v>
+      </c>
+      <c r="C28" s="74" t="s">
+        <v>138</v>
+      </c>
+      <c r="D28" s="71" t="s">
+        <v>124</v>
+      </c>
+      <c r="E28" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="F28" s="79" t="s">
+        <v>163</v>
+      </c>
+      <c r="G28" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="72"/>
+      <c r="B29" s="73"/>
+      <c r="C29" s="74"/>
+      <c r="D29" s="71" t="s">
+        <v>125</v>
+      </c>
+      <c r="E29" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F29" s="79"/>
+    </row>
+    <row r="30" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A30" s="72"/>
+      <c r="B30" s="73"/>
+      <c r="C30" s="74"/>
+      <c r="D30" s="71" t="s">
+        <v>126</v>
+      </c>
+      <c r="E30" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F30" s="79"/>
+    </row>
+    <row r="31" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="72"/>
+      <c r="B31" s="73"/>
+      <c r="C31" s="74"/>
+      <c r="D31" s="71" t="s">
+        <v>127</v>
+      </c>
+      <c r="E31" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F31" s="79"/>
+    </row>
+    <row r="32" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A32" s="72"/>
+      <c r="B32" s="73"/>
+      <c r="C32" s="74"/>
+      <c r="D32" s="71" t="s">
+        <v>128</v>
+      </c>
+      <c r="E32" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F32" s="79"/>
+    </row>
+    <row r="33" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A33" s="72"/>
+      <c r="B33" s="73"/>
+      <c r="C33" s="74"/>
+      <c r="D33" s="71" t="s">
+        <v>129</v>
+      </c>
+      <c r="E33" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F33" s="79"/>
+    </row>
+    <row r="34" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A34" s="72"/>
+      <c r="B34" s="73"/>
+      <c r="C34" s="74"/>
+      <c r="D34" s="71" t="s">
+        <v>130</v>
+      </c>
+      <c r="E34" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F34" s="79"/>
+    </row>
+    <row r="35" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="72"/>
+      <c r="B35" s="73"/>
+      <c r="C35" s="74"/>
+      <c r="D35" s="71" t="s">
+        <v>131</v>
+      </c>
+      <c r="E35" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F35" s="79"/>
+    </row>
+    <row r="36" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A36" s="72">
+        <v>9</v>
+      </c>
+      <c r="B36" s="73" t="s">
+        <v>97</v>
+      </c>
+      <c r="C36" s="74" t="s">
+        <v>137</v>
+      </c>
+      <c r="D36" s="71" t="s">
+        <v>132</v>
+      </c>
+      <c r="E36" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F36" s="79" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A37" s="72"/>
+      <c r="B37" s="73"/>
+      <c r="C37" s="74"/>
+      <c r="D37" s="71" t="s">
+        <v>133</v>
+      </c>
+      <c r="E37" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F37" s="79"/>
+    </row>
+    <row r="38" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A38" s="72"/>
+      <c r="B38" s="73"/>
+      <c r="C38" s="74"/>
+      <c r="D38" s="71" t="s">
+        <v>134</v>
+      </c>
+      <c r="E38" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="F38" s="79"/>
+    </row>
+    <row r="39" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A39" s="69">
+        <v>10</v>
+      </c>
+      <c r="B39" s="68" t="s">
+        <v>27</v>
+      </c>
+      <c r="C39" s="70" t="s">
+        <v>136</v>
+      </c>
+      <c r="D39" s="75"/>
+      <c r="E39" s="71"/>
+      <c r="F39" s="80" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E40" s="62"/>
+      <c r="F40" s="78"/>
+    </row>
+    <row r="41" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D41" s="63"/>
+      <c r="E41" s="62"/>
+      <c r="F41" s="78"/>
+    </row>
+    <row r="42" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D42" s="63"/>
+      <c r="E42" s="62"/>
+      <c r="F42" s="78"/>
+    </row>
+    <row r="43" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D43" s="63"/>
+      <c r="E43" s="62"/>
+      <c r="F43" s="78"/>
+    </row>
+    <row r="44" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D44" s="63"/>
+      <c r="E44" s="62"/>
+      <c r="F44" s="78"/>
+    </row>
+    <row r="45" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E45" s="62"/>
+      <c r="F45" s="78"/>
+    </row>
+    <row r="46" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E46" s="62"/>
+      <c r="F46" s="78"/>
+    </row>
+    <row r="47" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E47" s="62"/>
+      <c r="F47" s="78"/>
+    </row>
+    <row r="48" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E48" s="62"/>
+      <c r="F48" s="78"/>
+    </row>
+    <row r="49" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E49" s="62"/>
+      <c r="F49" s="78"/>
+    </row>
+    <row r="50" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E50" s="62"/>
+      <c r="F50" s="78"/>
+    </row>
+    <row r="51" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E51" s="62"/>
+      <c r="F51" s="78"/>
+    </row>
+    <row r="52" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E52" s="62"/>
+      <c r="F52" s="78"/>
+    </row>
+    <row r="53" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E53" s="62"/>
+      <c r="F53" s="78"/>
+    </row>
+    <row r="54" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E54" s="62"/>
+      <c r="F54" s="78"/>
+    </row>
+    <row r="55" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E55" s="62"/>
+      <c r="F55" s="78"/>
+    </row>
+    <row r="56" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E56" s="62"/>
+      <c r="F56" s="78"/>
+    </row>
+    <row r="57" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E57" s="62"/>
+      <c r="F57" s="78"/>
+    </row>
+    <row r="58" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E58" s="62"/>
+      <c r="F58" s="78"/>
+    </row>
+    <row r="59" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E59" s="62"/>
+      <c r="F59" s="78"/>
+    </row>
+    <row r="60" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E60" s="62"/>
+      <c r="F60" s="78"/>
+    </row>
+    <row r="61" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E61" s="62"/>
+      <c r="F61" s="78"/>
+    </row>
+    <row r="62" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E62" s="62"/>
+      <c r="F62" s="78"/>
+    </row>
+    <row r="63" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E63" s="62"/>
+      <c r="F63" s="78"/>
+    </row>
+    <row r="64" spans="5:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E64" s="62"/>
+      <c r="F64" s="78"/>
+    </row>
+    <row r="65" spans="4:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E65" s="62"/>
+      <c r="F65" s="78"/>
+    </row>
+    <row r="66" spans="4:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E66" s="62"/>
+      <c r="F66" s="78"/>
+    </row>
+    <row r="67" spans="4:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E67" s="62"/>
+      <c r="F67" s="78"/>
+    </row>
+    <row r="68" spans="4:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E68" s="62"/>
+      <c r="F68" s="78"/>
+    </row>
+    <row r="69" spans="4:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E69" s="62"/>
+      <c r="F69" s="78"/>
+    </row>
+    <row r="70" spans="4:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E70" s="62"/>
+      <c r="F70" s="78"/>
+    </row>
+    <row r="71" spans="4:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E71" s="62"/>
+      <c r="F71" s="78"/>
+    </row>
+    <row r="72" spans="4:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D72" s="64"/>
+      <c r="E72" s="65"/>
+      <c r="F72" s="78"/>
+    </row>
+  </sheetData>
+  <mergeCells count="28">
+    <mergeCell ref="F4:F8"/>
+    <mergeCell ref="F9:F11"/>
+    <mergeCell ref="F12:F15"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="F36:F38"/>
+    <mergeCell ref="F28:F35"/>
+    <mergeCell ref="F18:F27"/>
+    <mergeCell ref="C28:C35"/>
+    <mergeCell ref="B28:B35"/>
+    <mergeCell ref="A28:A35"/>
+    <mergeCell ref="C36:C38"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="C12:C15"/>
+    <mergeCell ref="A12:A15"/>
+    <mergeCell ref="C18:C27"/>
+    <mergeCell ref="B18:B27"/>
+    <mergeCell ref="A18:A27"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="A4:A8"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B12:B15"/>
+    <mergeCell ref="B4:B8"/>
+    <mergeCell ref="C4:C8"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="C9:C11"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="G27" r:id="rId1" xr:uid="{8F82EA5A-B040-442D-8D33-D437ACD7D892}"/>
+    <hyperlink ref="G17" r:id="rId2" xr:uid="{EDA6AEEC-14A3-4778-9A3E-A0590D612609}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{004663A5-903D-4F33-9CF8-4B48BA1B1476}">
+  <dimension ref="A1:E45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" ht="54.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="85" t="s">
+        <v>166</v>
+      </c>
+      <c r="B1" s="86" t="s">
+        <v>167</v>
+      </c>
+      <c r="C1" s="86" t="s">
+        <v>168</v>
+      </c>
+      <c r="D1" s="86" t="s">
+        <v>169</v>
+      </c>
+      <c r="E1" s="87" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="22.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="96" t="s">
+        <v>171</v>
+      </c>
+      <c r="B2" s="81" t="s">
+        <v>172</v>
+      </c>
+      <c r="C2" s="99" t="s">
+        <v>173</v>
+      </c>
+      <c r="D2" s="81"/>
+      <c r="E2" s="88"/>
+    </row>
+    <row r="3" spans="1:5" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="97"/>
+      <c r="B3" s="81" t="s">
+        <v>174</v>
+      </c>
+      <c r="C3" s="100"/>
+      <c r="D3" s="81"/>
+      <c r="E3" s="88"/>
+    </row>
+    <row r="4" spans="1:5" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="98"/>
+      <c r="B4" s="81" t="s">
+        <v>175</v>
+      </c>
+      <c r="C4" s="101"/>
+      <c r="D4" s="81"/>
+      <c r="E4" s="88"/>
+    </row>
+    <row r="5" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="95" t="s">
+        <v>176</v>
+      </c>
+      <c r="B5" s="81" t="s">
+        <v>177</v>
+      </c>
+      <c r="C5" s="102" t="s">
+        <v>99</v>
+      </c>
+      <c r="D5" s="82"/>
+      <c r="E5" s="89"/>
+    </row>
+    <row r="6" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="97"/>
+      <c r="B6" s="81" t="s">
+        <v>178</v>
+      </c>
+      <c r="C6" s="103"/>
+      <c r="D6" s="81"/>
+      <c r="E6" s="88"/>
+    </row>
+    <row r="7" spans="1:5" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="98"/>
+      <c r="B7" s="81" t="s">
+        <v>179</v>
+      </c>
+      <c r="C7" s="104"/>
+      <c r="D7" s="81"/>
+      <c r="E7" s="88"/>
+    </row>
+    <row r="8" spans="1:5" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="95" t="s">
+        <v>180</v>
+      </c>
+      <c r="B8" s="81" t="s">
+        <v>181</v>
+      </c>
+      <c r="C8" s="102" t="s">
+        <v>100</v>
+      </c>
+      <c r="D8" s="82"/>
+      <c r="E8" s="89"/>
+    </row>
+    <row r="9" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="97"/>
+      <c r="B9" s="105" t="s">
+        <v>182</v>
+      </c>
+      <c r="C9" s="104"/>
+      <c r="D9" s="82"/>
+      <c r="E9" s="89"/>
+    </row>
+    <row r="10" spans="1:5" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="97"/>
+      <c r="B10" s="106"/>
+      <c r="C10" s="82" t="s">
+        <v>101</v>
+      </c>
+      <c r="D10" s="82"/>
+      <c r="E10" s="89"/>
+    </row>
+    <row r="11" spans="1:5" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="97"/>
+      <c r="B11" s="106"/>
+      <c r="C11" s="82" t="s">
+        <v>102</v>
+      </c>
+      <c r="D11" s="82"/>
+      <c r="E11" s="89"/>
+    </row>
+    <row r="12" spans="1:5" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="97"/>
+      <c r="B12" s="106"/>
+      <c r="C12" s="82" t="s">
+        <v>103</v>
+      </c>
+      <c r="D12" s="82"/>
+      <c r="E12" s="89"/>
+    </row>
+    <row r="13" spans="1:5" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="98"/>
+      <c r="B13" s="107"/>
+      <c r="C13" s="82" t="s">
+        <v>104</v>
+      </c>
+      <c r="D13" s="82"/>
+      <c r="E13" s="89"/>
+    </row>
+    <row r="14" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="95" t="s">
+        <v>183</v>
+      </c>
+      <c r="B14" s="105" t="s">
+        <v>184</v>
+      </c>
+      <c r="C14" s="82" t="s">
+        <v>105</v>
+      </c>
+      <c r="D14" s="82"/>
+      <c r="E14" s="89"/>
+    </row>
+    <row r="15" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="97"/>
+      <c r="B15" s="106"/>
+      <c r="C15" s="82" t="s">
+        <v>106</v>
+      </c>
+      <c r="D15" s="82"/>
+      <c r="E15" s="89"/>
+    </row>
+    <row r="16" spans="1:5" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="97"/>
+      <c r="B16" s="107"/>
+      <c r="C16" s="82" t="s">
+        <v>107</v>
+      </c>
+      <c r="D16" s="82"/>
+      <c r="E16" s="89"/>
+    </row>
+    <row r="17" spans="1:5" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="98"/>
+      <c r="B17" s="81" t="s">
+        <v>185</v>
+      </c>
+      <c r="C17" s="82"/>
+      <c r="D17" s="82"/>
+      <c r="E17" s="89"/>
+    </row>
+    <row r="18" spans="1:5" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="95" t="s">
+        <v>186</v>
+      </c>
+      <c r="B18" s="105" t="s">
+        <v>187</v>
+      </c>
+      <c r="C18" s="82" t="s">
+        <v>108</v>
+      </c>
+      <c r="D18" s="82"/>
+      <c r="E18" s="89"/>
+    </row>
+    <row r="19" spans="1:5" ht="72.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="97"/>
+      <c r="B19" s="106"/>
+      <c r="C19" s="82" t="s">
+        <v>109</v>
+      </c>
+      <c r="D19" s="82"/>
+      <c r="E19" s="89"/>
+    </row>
+    <row r="20" spans="1:5" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="97"/>
+      <c r="B20" s="106"/>
+      <c r="C20" s="82" t="s">
+        <v>110</v>
+      </c>
+      <c r="D20" s="82"/>
+      <c r="E20" s="89"/>
+    </row>
+    <row r="21" spans="1:5" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="98"/>
+      <c r="B21" s="107"/>
+      <c r="C21" s="82" t="s">
+        <v>111</v>
+      </c>
+      <c r="D21" s="82"/>
+      <c r="E21" s="89"/>
+    </row>
+    <row r="22" spans="1:5" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="108" t="s">
+        <v>188</v>
+      </c>
+      <c r="B22" s="110" t="s">
+        <v>189</v>
+      </c>
+      <c r="C22" s="83" t="s">
+        <v>112</v>
+      </c>
+      <c r="D22" s="83"/>
+      <c r="E22" s="90"/>
+    </row>
+    <row r="23" spans="1:5" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="109"/>
+      <c r="B23" s="111"/>
+      <c r="C23" s="83" t="s">
+        <v>113</v>
+      </c>
+      <c r="D23" s="83"/>
+      <c r="E23" s="90"/>
+    </row>
+    <row r="24" spans="1:5" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="108" t="s">
+        <v>190</v>
+      </c>
+      <c r="B24" s="110"/>
+      <c r="C24" s="83" t="s">
+        <v>114</v>
+      </c>
+      <c r="D24" s="83"/>
+      <c r="E24" s="90"/>
+    </row>
+    <row r="25" spans="1:5" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="112"/>
+      <c r="B25" s="113"/>
+      <c r="C25" s="83" t="s">
+        <v>115</v>
+      </c>
+      <c r="D25" s="83"/>
+      <c r="E25" s="90"/>
+    </row>
+    <row r="26" spans="1:5" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="112"/>
+      <c r="B26" s="113"/>
+      <c r="C26" s="83" t="s">
+        <v>116</v>
+      </c>
+      <c r="D26" s="83"/>
+      <c r="E26" s="90"/>
+    </row>
+    <row r="27" spans="1:5" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="112"/>
+      <c r="B27" s="113"/>
+      <c r="C27" s="83" t="s">
+        <v>117</v>
+      </c>
+      <c r="D27" s="83"/>
+      <c r="E27" s="90"/>
+    </row>
+    <row r="28" spans="1:5" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="112"/>
+      <c r="B28" s="113"/>
+      <c r="C28" s="83" t="s">
+        <v>118</v>
+      </c>
+      <c r="D28" s="83"/>
+      <c r="E28" s="90"/>
+    </row>
+    <row r="29" spans="1:5" ht="72.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="112"/>
+      <c r="B29" s="111"/>
+      <c r="C29" s="83" t="s">
+        <v>119</v>
+      </c>
+      <c r="D29" s="83"/>
+      <c r="E29" s="90"/>
+    </row>
+    <row r="30" spans="1:5" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="112"/>
+      <c r="B30" s="110" t="s">
+        <v>191</v>
+      </c>
+      <c r="C30" s="83" t="s">
+        <v>120</v>
+      </c>
+      <c r="D30" s="83"/>
+      <c r="E30" s="90"/>
+    </row>
+    <row r="31" spans="1:5" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="112"/>
+      <c r="B31" s="113"/>
+      <c r="C31" s="83" t="s">
+        <v>121</v>
+      </c>
+      <c r="D31" s="83"/>
+      <c r="E31" s="90"/>
+    </row>
+    <row r="32" spans="1:5" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="112"/>
+      <c r="B32" s="113"/>
+      <c r="C32" s="83" t="s">
+        <v>122</v>
+      </c>
+      <c r="D32" s="83"/>
+      <c r="E32" s="90"/>
+    </row>
+    <row r="33" spans="1:5" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="109"/>
+      <c r="B33" s="111"/>
+      <c r="C33" s="83" t="s">
+        <v>123</v>
+      </c>
+      <c r="D33" s="83"/>
+      <c r="E33" s="90"/>
+    </row>
+    <row r="34" spans="1:5" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="108" t="s">
+        <v>192</v>
+      </c>
+      <c r="B34" s="110" t="s">
+        <v>181</v>
+      </c>
+      <c r="C34" s="83" t="s">
+        <v>124</v>
+      </c>
+      <c r="D34" s="83"/>
+      <c r="E34" s="90"/>
+    </row>
+    <row r="35" spans="1:5" ht="96.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="112"/>
+      <c r="B35" s="113"/>
+      <c r="C35" s="83" t="s">
+        <v>125</v>
+      </c>
+      <c r="D35" s="83"/>
+      <c r="E35" s="90"/>
+    </row>
+    <row r="36" spans="1:5" ht="72.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="112"/>
+      <c r="B36" s="111"/>
+      <c r="C36" s="83" t="s">
+        <v>126</v>
+      </c>
+      <c r="D36" s="83"/>
+      <c r="E36" s="90"/>
+    </row>
+    <row r="37" spans="1:5" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="112"/>
+      <c r="B37" s="110" t="s">
+        <v>193</v>
+      </c>
+      <c r="C37" s="83" t="s">
+        <v>127</v>
+      </c>
+      <c r="D37" s="83"/>
+      <c r="E37" s="90"/>
+    </row>
+    <row r="38" spans="1:5" ht="72.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="112"/>
+      <c r="B38" s="113"/>
+      <c r="C38" s="83" t="s">
+        <v>128</v>
+      </c>
+      <c r="D38" s="83"/>
+      <c r="E38" s="90"/>
+    </row>
+    <row r="39" spans="1:5" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="112"/>
+      <c r="B39" s="111"/>
+      <c r="C39" s="83" t="s">
+        <v>129</v>
+      </c>
+      <c r="D39" s="83"/>
+      <c r="E39" s="90"/>
+    </row>
+    <row r="40" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="109"/>
+      <c r="B40" s="84"/>
+      <c r="C40" s="83" t="s">
+        <v>130</v>
+      </c>
+      <c r="D40" s="83"/>
+      <c r="E40" s="90"/>
+    </row>
+    <row r="41" spans="1:5" ht="72.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="91"/>
+      <c r="B41" s="84"/>
+      <c r="C41" s="83" t="s">
+        <v>131</v>
+      </c>
+      <c r="D41" s="83"/>
+      <c r="E41" s="90"/>
+    </row>
+    <row r="42" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="108" t="s">
+        <v>194</v>
+      </c>
+      <c r="B42" s="110" t="s">
+        <v>195</v>
+      </c>
+      <c r="C42" s="83" t="s">
+        <v>132</v>
+      </c>
+      <c r="D42" s="83"/>
+      <c r="E42" s="90"/>
+    </row>
+    <row r="43" spans="1:5" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="112"/>
+      <c r="B43" s="111"/>
+      <c r="C43" s="83" t="s">
+        <v>133</v>
+      </c>
+      <c r="D43" s="83"/>
+      <c r="E43" s="90"/>
+    </row>
+    <row r="44" spans="1:5" ht="96.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="109"/>
+      <c r="B44" s="84" t="s">
+        <v>196</v>
+      </c>
+      <c r="C44" s="83" t="s">
+        <v>134</v>
+      </c>
+      <c r="D44" s="83"/>
+      <c r="E44" s="90"/>
+    </row>
+    <row r="45" spans="1:5" ht="36" x14ac:dyDescent="0.25">
+      <c r="A45" s="92" t="s">
+        <v>197</v>
+      </c>
+      <c r="B45" s="93"/>
+      <c r="C45" s="93"/>
+      <c r="D45" s="93"/>
+      <c r="E45" s="94"/>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="A42:A44"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="A24:A33"/>
+    <mergeCell ref="B24:B29"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="A34:A40"/>
+    <mergeCell ref="B34:B36"/>
+    <mergeCell ref="B37:B39"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="A8:A13"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="B9:B13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>